<commit_message>
remove post case action
</commit_message>
<xml_diff>
--- a/projects/automation_exercise/api/case/testcase-automation_exercise.xlsx
+++ b/projects/automation_exercise/api/case/testcase-automation_exercise.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/606929f86db40629/Documents/Python/automation_framework/projects/automation_exercise/api/case/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{B959E1B4-B71D-476A-B78C-D11EC8419DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A123DDBF-1FFA-4F27-9281-FA02210AA21A}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="8_{B959E1B4-B71D-476A-B78C-D11EC8419DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AABE53F2-9EE6-4B15-B3DD-CF0BBFA87018}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AB49B25E-9B57-422D-B60E-7F12796728DD}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Products" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Products!$A$1:$V$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Products!$A$1:$U$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -364,7 +364,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="35">
   <si>
     <t>JIRA ID</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -434,15 +434,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Expected Json Data</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Set Global Variable</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Post_Case_Action</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -477,10 +469,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Get All Products List</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>/api/productsList</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -490,6 +478,29 @@
   </si>
   <si>
     <t>["=","$.responseCode",200];</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Json Result Validation</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>POST To All Products List</t>
+  </si>
+  <si>
+    <t>Get All Products List</t>
+  </si>
+  <si>
+    <t>post_to_all_product_list</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>POST</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>["=","$.responseCode",405];
+["=","$.message","This request method is not supported."]</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -614,7 +625,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -670,6 +681,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -694,13 +708,13 @@
     <xdr:from>
       <xdr:col>22</xdr:col>
       <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>1802</xdr:row>
+      <xdr:row>1800</xdr:row>
       <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>23</xdr:col>
       <xdr:colOff>647700</xdr:colOff>
-      <xdr:row>1957</xdr:row>
+      <xdr:row>1955</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1033,7 +1047,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{571522A3-8A90-45FA-BDC2-DE8E1EFD9C0E}">
-  <dimension ref="A1:V154"/>
+  <dimension ref="A1:U154"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="8.5" style="12" bestFit="1" customWidth="1"/>
@@ -1054,12 +1068,11 @@
     <col min="18" max="18" width="16.125" style="12" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="53.75" style="12" customWidth="1"/>
     <col min="20" max="20" width="15" style="12" customWidth="1"/>
-    <col min="21" max="21" width="9" style="12"/>
-    <col min="22" max="22" width="27.875" style="12" customWidth="1"/>
-    <col min="23" max="16384" width="9" style="12"/>
+    <col min="21" max="21" width="27.875" style="12" customWidth="1"/>
+    <col min="22" max="16384" width="9" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="8" customFormat="1" ht="27">
+    <row r="1" spans="1:21" s="8" customFormat="1" ht="27">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1100,7 +1113,7 @@
         <v>12</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="O1" s="1" t="s">
         <v>13</v>
@@ -1115,49 +1128,46 @@
         <v>16</v>
       </c>
       <c r="S1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="U1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:21" ht="27">
+      <c r="A2" s="5"/>
+      <c r="B2" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="V1" s="7" t="s">
+      <c r="F2" s="5" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:22" ht="27">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>22</v>
-      </c>
       <c r="G2" s="5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H2" s="5"/>
       <c r="I2" s="5"/>
       <c r="J2" s="5"/>
       <c r="K2" s="5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="L2" s="9" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="N2" s="5"/>
       <c r="O2" s="5"/>
@@ -1167,39 +1177,61 @@
       <c r="Q2" s="10"/>
       <c r="R2" s="5"/>
       <c r="S2" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="T2" s="5"/>
-      <c r="U2" s="5"/>
-      <c r="V2" s="11" t="s">
+      <c r="U2" s="11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" ht="40.5">
+      <c r="A3" s="5"/>
+      <c r="B3" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="3" spans="1:22">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
+      <c r="D3" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H3" s="5"/>
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="9"/>
-      <c r="M3" s="5"/>
+      <c r="K3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="L3" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>33</v>
+      </c>
       <c r="N3" s="5"/>
       <c r="O3" s="5"/>
-      <c r="P3" s="5"/>
+      <c r="P3" s="5">
+        <v>200</v>
+      </c>
       <c r="Q3" s="10"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="5"/>
+      <c r="S3" s="5" t="s">
+        <v>34</v>
+      </c>
       <c r="T3" s="5"/>
-      <c r="U3" s="5"/>
-      <c r="V3" s="11"/>
-    </row>
-    <row r="4" spans="1:22">
+      <c r="U3" s="11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21">
       <c r="A4" s="5"/>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -1220,10 +1252,9 @@
       <c r="R4" s="5"/>
       <c r="S4" s="5"/>
       <c r="T4" s="5"/>
-      <c r="U4" s="5"/>
-      <c r="V4" s="11"/>
-    </row>
-    <row r="5" spans="1:22">
+      <c r="U4" s="11"/>
+    </row>
+    <row r="5" spans="1:21">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -1244,10 +1275,9 @@
       <c r="R5" s="5"/>
       <c r="S5" s="5"/>
       <c r="T5" s="5"/>
-      <c r="U5" s="5"/>
-      <c r="V5" s="11"/>
-    </row>
-    <row r="6" spans="1:22">
+      <c r="U5" s="11"/>
+    </row>
+    <row r="6" spans="1:21">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
@@ -1268,10 +1298,9 @@
       <c r="R6" s="5"/>
       <c r="S6" s="5"/>
       <c r="T6" s="5"/>
-      <c r="U6" s="5"/>
-      <c r="V6" s="11"/>
-    </row>
-    <row r="7" spans="1:22">
+      <c r="U6" s="11"/>
+    </row>
+    <row r="7" spans="1:21">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
@@ -1292,10 +1321,9 @@
       <c r="R7" s="5"/>
       <c r="S7" s="5"/>
       <c r="T7" s="5"/>
-      <c r="U7" s="5"/>
-      <c r="V7" s="11"/>
-    </row>
-    <row r="8" spans="1:22">
+      <c r="U7" s="11"/>
+    </row>
+    <row r="8" spans="1:21">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -1316,10 +1344,9 @@
       <c r="R8" s="5"/>
       <c r="S8" s="5"/>
       <c r="T8" s="5"/>
-      <c r="U8" s="5"/>
-      <c r="V8" s="11"/>
-    </row>
-    <row r="9" spans="1:22">
+      <c r="U8" s="11"/>
+    </row>
+    <row r="9" spans="1:21">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
@@ -1340,10 +1367,9 @@
       <c r="R9" s="5"/>
       <c r="S9" s="5"/>
       <c r="T9" s="5"/>
-      <c r="U9" s="5"/>
-      <c r="V9" s="11"/>
-    </row>
-    <row r="10" spans="1:22">
+      <c r="U9" s="11"/>
+    </row>
+    <row r="10" spans="1:21">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -1364,10 +1390,9 @@
       <c r="R10" s="5"/>
       <c r="S10" s="5"/>
       <c r="T10" s="5"/>
-      <c r="U10" s="5"/>
-      <c r="V10" s="11"/>
-    </row>
-    <row r="11" spans="1:22">
+      <c r="U10" s="11"/>
+    </row>
+    <row r="11" spans="1:21">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -1388,10 +1413,9 @@
       <c r="R11" s="5"/>
       <c r="S11" s="5"/>
       <c r="T11" s="5"/>
-      <c r="U11" s="5"/>
-      <c r="V11" s="11"/>
-    </row>
-    <row r="12" spans="1:22">
+      <c r="U11" s="11"/>
+    </row>
+    <row r="12" spans="1:21">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -1412,10 +1436,9 @@
       <c r="R12" s="5"/>
       <c r="S12" s="5"/>
       <c r="T12" s="5"/>
-      <c r="U12" s="5"/>
-      <c r="V12" s="11"/>
-    </row>
-    <row r="13" spans="1:22">
+      <c r="U12" s="11"/>
+    </row>
+    <row r="13" spans="1:21">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -1436,10 +1459,9 @@
       <c r="R13" s="5"/>
       <c r="S13" s="5"/>
       <c r="T13" s="5"/>
-      <c r="U13" s="5"/>
-      <c r="V13" s="11"/>
-    </row>
-    <row r="14" spans="1:22">
+      <c r="U13" s="11"/>
+    </row>
+    <row r="14" spans="1:21">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -1460,10 +1482,9 @@
       <c r="R14" s="5"/>
       <c r="S14" s="5"/>
       <c r="T14" s="5"/>
-      <c r="U14" s="5"/>
-      <c r="V14" s="11"/>
-    </row>
-    <row r="15" spans="1:22">
+      <c r="U14" s="11"/>
+    </row>
+    <row r="15" spans="1:21">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -1484,10 +1505,9 @@
       <c r="R15" s="5"/>
       <c r="S15" s="5"/>
       <c r="T15" s="5"/>
-      <c r="U15" s="5"/>
-      <c r="V15" s="11"/>
-    </row>
-    <row r="16" spans="1:22">
+      <c r="U15" s="11"/>
+    </row>
+    <row r="16" spans="1:21">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -1508,10 +1528,9 @@
       <c r="R16" s="5"/>
       <c r="S16" s="5"/>
       <c r="T16" s="5"/>
-      <c r="U16" s="5"/>
-      <c r="V16" s="11"/>
-    </row>
-    <row r="17" spans="1:22">
+      <c r="U16" s="11"/>
+    </row>
+    <row r="17" spans="1:21">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -1532,10 +1551,9 @@
       <c r="R17" s="5"/>
       <c r="S17" s="5"/>
       <c r="T17" s="5"/>
-      <c r="U17" s="5"/>
-      <c r="V17" s="11"/>
-    </row>
-    <row r="18" spans="1:22">
+      <c r="U17" s="11"/>
+    </row>
+    <row r="18" spans="1:21">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -1556,10 +1574,9 @@
       <c r="R18" s="5"/>
       <c r="S18" s="5"/>
       <c r="T18" s="5"/>
-      <c r="U18" s="5"/>
-      <c r="V18" s="11"/>
-    </row>
-    <row r="19" spans="1:22">
+      <c r="U18" s="11"/>
+    </row>
+    <row r="19" spans="1:21">
       <c r="A19" s="5"/>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -1580,10 +1597,9 @@
       <c r="R19" s="5"/>
       <c r="S19" s="5"/>
       <c r="T19" s="5"/>
-      <c r="U19" s="5"/>
-      <c r="V19" s="11"/>
-    </row>
-    <row r="20" spans="1:22">
+      <c r="U19" s="11"/>
+    </row>
+    <row r="20" spans="1:21">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -1604,10 +1620,9 @@
       <c r="R20" s="5"/>
       <c r="S20" s="5"/>
       <c r="T20" s="5"/>
-      <c r="U20" s="5"/>
-      <c r="V20" s="11"/>
-    </row>
-    <row r="21" spans="1:22">
+      <c r="U20" s="11"/>
+    </row>
+    <row r="21" spans="1:21">
       <c r="A21" s="5"/>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -1628,10 +1643,9 @@
       <c r="R21" s="5"/>
       <c r="S21" s="5"/>
       <c r="T21" s="5"/>
-      <c r="U21" s="5"/>
-      <c r="V21" s="11"/>
-    </row>
-    <row r="22" spans="1:22">
+      <c r="U21" s="11"/>
+    </row>
+    <row r="22" spans="1:21">
       <c r="A22" s="5"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -1652,10 +1666,9 @@
       <c r="R22" s="5"/>
       <c r="S22" s="5"/>
       <c r="T22" s="5"/>
-      <c r="U22" s="5"/>
-      <c r="V22" s="11"/>
-    </row>
-    <row r="23" spans="1:22">
+      <c r="U22" s="11"/>
+    </row>
+    <row r="23" spans="1:21">
       <c r="A23" s="5"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -1676,10 +1689,9 @@
       <c r="R23" s="5"/>
       <c r="S23" s="5"/>
       <c r="T23" s="5"/>
-      <c r="U23" s="5"/>
-      <c r="V23" s="11"/>
-    </row>
-    <row r="24" spans="1:22">
+      <c r="U23" s="11"/>
+    </row>
+    <row r="24" spans="1:21">
       <c r="A24" s="5"/>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
@@ -1700,10 +1712,9 @@
       <c r="R24" s="5"/>
       <c r="S24" s="5"/>
       <c r="T24" s="5"/>
-      <c r="U24" s="5"/>
-      <c r="V24" s="11"/>
-    </row>
-    <row r="25" spans="1:22">
+      <c r="U24" s="11"/>
+    </row>
+    <row r="25" spans="1:21">
       <c r="A25" s="5"/>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -1724,10 +1735,9 @@
       <c r="R25" s="5"/>
       <c r="S25" s="5"/>
       <c r="T25" s="5"/>
-      <c r="U25" s="5"/>
-      <c r="V25" s="11"/>
-    </row>
-    <row r="26" spans="1:22">
+      <c r="U25" s="11"/>
+    </row>
+    <row r="26" spans="1:21">
       <c r="A26" s="5"/>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
@@ -1748,10 +1758,9 @@
       <c r="R26" s="5"/>
       <c r="S26" s="5"/>
       <c r="T26" s="5"/>
-      <c r="U26" s="5"/>
-      <c r="V26" s="11"/>
-    </row>
-    <row r="27" spans="1:22">
+      <c r="U26" s="11"/>
+    </row>
+    <row r="27" spans="1:21">
       <c r="A27" s="5"/>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -1772,10 +1781,9 @@
       <c r="R27" s="5"/>
       <c r="S27" s="5"/>
       <c r="T27" s="5"/>
-      <c r="U27" s="5"/>
-      <c r="V27" s="11"/>
-    </row>
-    <row r="28" spans="1:22">
+      <c r="U27" s="11"/>
+    </row>
+    <row r="28" spans="1:21">
       <c r="A28" s="5"/>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -1796,10 +1804,9 @@
       <c r="R28" s="5"/>
       <c r="S28" s="5"/>
       <c r="T28" s="5"/>
-      <c r="U28" s="5"/>
-      <c r="V28" s="11"/>
-    </row>
-    <row r="29" spans="1:22">
+      <c r="U28" s="11"/>
+    </row>
+    <row r="29" spans="1:21">
       <c r="A29" s="5"/>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -1820,10 +1827,9 @@
       <c r="R29" s="5"/>
       <c r="S29" s="5"/>
       <c r="T29" s="5"/>
-      <c r="U29" s="5"/>
-      <c r="V29" s="11"/>
-    </row>
-    <row r="30" spans="1:22">
+      <c r="U29" s="11"/>
+    </row>
+    <row r="30" spans="1:21">
       <c r="A30" s="5"/>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
@@ -1844,10 +1850,9 @@
       <c r="R30" s="5"/>
       <c r="S30" s="5"/>
       <c r="T30" s="5"/>
-      <c r="U30" s="5"/>
-      <c r="V30" s="11"/>
-    </row>
-    <row r="31" spans="1:22">
+      <c r="U30" s="11"/>
+    </row>
+    <row r="31" spans="1:21">
       <c r="A31" s="5"/>
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>
@@ -1868,10 +1873,9 @@
       <c r="R31" s="5"/>
       <c r="S31" s="5"/>
       <c r="T31" s="5"/>
-      <c r="U31" s="5"/>
-      <c r="V31" s="11"/>
-    </row>
-    <row r="32" spans="1:22">
+      <c r="U31" s="11"/>
+    </row>
+    <row r="32" spans="1:21">
       <c r="A32" s="5"/>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -1892,10 +1896,9 @@
       <c r="R32" s="5"/>
       <c r="S32" s="5"/>
       <c r="T32" s="5"/>
-      <c r="U32" s="5"/>
-      <c r="V32" s="11"/>
-    </row>
-    <row r="33" spans="1:22">
+      <c r="U32" s="11"/>
+    </row>
+    <row r="33" spans="1:21">
       <c r="A33" s="5"/>
       <c r="B33" s="5"/>
       <c r="C33" s="5"/>
@@ -1916,10 +1919,9 @@
       <c r="R33" s="5"/>
       <c r="S33" s="5"/>
       <c r="T33" s="5"/>
-      <c r="U33" s="5"/>
-      <c r="V33" s="11"/>
-    </row>
-    <row r="34" spans="1:22">
+      <c r="U33" s="11"/>
+    </row>
+    <row r="34" spans="1:21">
       <c r="A34" s="5"/>
       <c r="B34" s="5"/>
       <c r="C34" s="5"/>
@@ -1940,10 +1942,9 @@
       <c r="R34" s="5"/>
       <c r="S34" s="5"/>
       <c r="T34" s="5"/>
-      <c r="U34" s="5"/>
-      <c r="V34" s="11"/>
-    </row>
-    <row r="35" spans="1:22">
+      <c r="U34" s="11"/>
+    </row>
+    <row r="35" spans="1:21">
       <c r="A35" s="5"/>
       <c r="B35" s="5"/>
       <c r="C35" s="5"/>
@@ -1964,10 +1965,9 @@
       <c r="R35" s="5"/>
       <c r="S35" s="5"/>
       <c r="T35" s="5"/>
-      <c r="U35" s="5"/>
-      <c r="V35" s="11"/>
-    </row>
-    <row r="36" spans="1:22">
+      <c r="U35" s="11"/>
+    </row>
+    <row r="36" spans="1:21">
       <c r="A36" s="5"/>
       <c r="B36" s="5"/>
       <c r="C36" s="5"/>
@@ -1988,10 +1988,9 @@
       <c r="R36" s="5"/>
       <c r="S36" s="5"/>
       <c r="T36" s="5"/>
-      <c r="U36" s="5"/>
-      <c r="V36" s="11"/>
-    </row>
-    <row r="37" spans="1:22">
+      <c r="U36" s="11"/>
+    </row>
+    <row r="37" spans="1:21">
       <c r="A37" s="5"/>
       <c r="B37" s="5"/>
       <c r="C37" s="5"/>
@@ -2012,10 +2011,9 @@
       <c r="R37" s="5"/>
       <c r="S37" s="5"/>
       <c r="T37" s="5"/>
-      <c r="U37" s="5"/>
-      <c r="V37" s="11"/>
-    </row>
-    <row r="38" spans="1:22">
+      <c r="U37" s="11"/>
+    </row>
+    <row r="38" spans="1:21">
       <c r="A38" s="5"/>
       <c r="B38" s="5"/>
       <c r="C38" s="5"/>
@@ -2036,10 +2034,9 @@
       <c r="R38" s="5"/>
       <c r="S38" s="5"/>
       <c r="T38" s="5"/>
-      <c r="U38" s="5"/>
-      <c r="V38" s="11"/>
-    </row>
-    <row r="39" spans="1:22">
+      <c r="U38" s="11"/>
+    </row>
+    <row r="39" spans="1:21">
       <c r="A39" s="5"/>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
@@ -2060,10 +2057,9 @@
       <c r="R39" s="5"/>
       <c r="S39" s="5"/>
       <c r="T39" s="5"/>
-      <c r="U39" s="5"/>
-      <c r="V39" s="11"/>
-    </row>
-    <row r="40" spans="1:22">
+      <c r="U39" s="11"/>
+    </row>
+    <row r="40" spans="1:21">
       <c r="A40" s="5"/>
       <c r="B40" s="5"/>
       <c r="C40" s="5"/>
@@ -2084,10 +2080,9 @@
       <c r="R40" s="5"/>
       <c r="S40" s="5"/>
       <c r="T40" s="5"/>
-      <c r="U40" s="5"/>
-      <c r="V40" s="11"/>
-    </row>
-    <row r="41" spans="1:22">
+      <c r="U40" s="11"/>
+    </row>
+    <row r="41" spans="1:21">
       <c r="A41" s="5"/>
       <c r="B41" s="5"/>
       <c r="C41" s="5"/>
@@ -2108,10 +2103,9 @@
       <c r="R41" s="5"/>
       <c r="S41" s="5"/>
       <c r="T41" s="5"/>
-      <c r="U41" s="5"/>
-      <c r="V41" s="11"/>
-    </row>
-    <row r="42" spans="1:22">
+      <c r="U41" s="11"/>
+    </row>
+    <row r="42" spans="1:21">
       <c r="A42" s="5"/>
       <c r="B42" s="5"/>
       <c r="C42" s="5"/>
@@ -2132,10 +2126,9 @@
       <c r="R42" s="5"/>
       <c r="S42" s="5"/>
       <c r="T42" s="5"/>
-      <c r="U42" s="5"/>
-      <c r="V42" s="11"/>
-    </row>
-    <row r="43" spans="1:22">
+      <c r="U42" s="11"/>
+    </row>
+    <row r="43" spans="1:21">
       <c r="A43" s="5"/>
       <c r="B43" s="5"/>
       <c r="C43" s="5"/>
@@ -2156,10 +2149,9 @@
       <c r="R43" s="5"/>
       <c r="S43" s="5"/>
       <c r="T43" s="5"/>
-      <c r="U43" s="5"/>
-      <c r="V43" s="11"/>
-    </row>
-    <row r="44" spans="1:22">
+      <c r="U43" s="11"/>
+    </row>
+    <row r="44" spans="1:21">
       <c r="A44" s="5"/>
       <c r="B44" s="5"/>
       <c r="C44" s="5"/>
@@ -2180,10 +2172,9 @@
       <c r="R44" s="5"/>
       <c r="S44" s="5"/>
       <c r="T44" s="5"/>
-      <c r="U44" s="5"/>
-      <c r="V44" s="11"/>
-    </row>
-    <row r="45" spans="1:22">
+      <c r="U44" s="11"/>
+    </row>
+    <row r="45" spans="1:21">
       <c r="A45" s="5"/>
       <c r="B45" s="5"/>
       <c r="C45" s="5"/>
@@ -2204,10 +2195,9 @@
       <c r="R45" s="5"/>
       <c r="S45" s="5"/>
       <c r="T45" s="5"/>
-      <c r="U45" s="5"/>
-      <c r="V45" s="11"/>
-    </row>
-    <row r="46" spans="1:22">
+      <c r="U45" s="11"/>
+    </row>
+    <row r="46" spans="1:21">
       <c r="A46" s="5"/>
       <c r="B46" s="5"/>
       <c r="C46" s="5"/>
@@ -2228,10 +2218,9 @@
       <c r="R46" s="5"/>
       <c r="S46" s="10"/>
       <c r="T46" s="5"/>
-      <c r="U46" s="5"/>
-      <c r="V46" s="11"/>
-    </row>
-    <row r="47" spans="1:22">
+      <c r="U46" s="11"/>
+    </row>
+    <row r="47" spans="1:21">
       <c r="A47" s="5"/>
       <c r="B47" s="5"/>
       <c r="C47" s="5"/>
@@ -2252,10 +2241,9 @@
       <c r="R47" s="5"/>
       <c r="S47" s="5"/>
       <c r="T47" s="5"/>
-      <c r="U47" s="5"/>
-      <c r="V47" s="11"/>
-    </row>
-    <row r="48" spans="1:22">
+      <c r="U47" s="11"/>
+    </row>
+    <row r="48" spans="1:21">
       <c r="A48" s="5"/>
       <c r="B48" s="5"/>
       <c r="C48" s="5"/>
@@ -2276,10 +2264,9 @@
       <c r="R48" s="5"/>
       <c r="S48" s="5"/>
       <c r="T48" s="5"/>
-      <c r="U48" s="5"/>
-      <c r="V48" s="11"/>
-    </row>
-    <row r="49" spans="1:22">
+      <c r="U48" s="11"/>
+    </row>
+    <row r="49" spans="1:21">
       <c r="A49" s="5"/>
       <c r="B49" s="5"/>
       <c r="C49" s="5"/>
@@ -2300,10 +2287,9 @@
       <c r="R49" s="5"/>
       <c r="S49" s="5"/>
       <c r="T49" s="5"/>
-      <c r="U49" s="5"/>
-      <c r="V49" s="11"/>
-    </row>
-    <row r="50" spans="1:22">
+      <c r="U49" s="11"/>
+    </row>
+    <row r="50" spans="1:21">
       <c r="A50" s="5"/>
       <c r="B50" s="5"/>
       <c r="C50" s="5"/>
@@ -2324,10 +2310,9 @@
       <c r="R50" s="5"/>
       <c r="S50" s="5"/>
       <c r="T50" s="5"/>
-      <c r="U50" s="5"/>
-      <c r="V50" s="11"/>
-    </row>
-    <row r="51" spans="1:22">
+      <c r="U50" s="11"/>
+    </row>
+    <row r="51" spans="1:21">
       <c r="A51" s="5"/>
       <c r="B51" s="5"/>
       <c r="C51" s="5"/>
@@ -2348,10 +2333,9 @@
       <c r="R51" s="5"/>
       <c r="S51" s="5"/>
       <c r="T51" s="5"/>
-      <c r="U51" s="5"/>
-      <c r="V51" s="11"/>
-    </row>
-    <row r="52" spans="1:22">
+      <c r="U51" s="11"/>
+    </row>
+    <row r="52" spans="1:21">
       <c r="A52" s="5"/>
       <c r="B52" s="5"/>
       <c r="C52" s="5"/>
@@ -2372,10 +2356,9 @@
       <c r="R52" s="5"/>
       <c r="S52" s="10"/>
       <c r="T52" s="5"/>
-      <c r="U52" s="5"/>
-      <c r="V52" s="11"/>
-    </row>
-    <row r="53" spans="1:22">
+      <c r="U52" s="11"/>
+    </row>
+    <row r="53" spans="1:21">
       <c r="A53" s="5"/>
       <c r="B53" s="5"/>
       <c r="C53" s="5"/>
@@ -2396,10 +2379,9 @@
       <c r="R53" s="5"/>
       <c r="S53" s="5"/>
       <c r="T53" s="5"/>
-      <c r="U53" s="5"/>
-      <c r="V53" s="11"/>
-    </row>
-    <row r="54" spans="1:22">
+      <c r="U53" s="11"/>
+    </row>
+    <row r="54" spans="1:21">
       <c r="A54" s="5"/>
       <c r="B54" s="5"/>
       <c r="C54" s="5"/>
@@ -2420,10 +2402,9 @@
       <c r="R54" s="5"/>
       <c r="S54" s="5"/>
       <c r="T54" s="5"/>
-      <c r="U54" s="5"/>
-      <c r="V54" s="11"/>
-    </row>
-    <row r="55" spans="1:22">
+      <c r="U54" s="11"/>
+    </row>
+    <row r="55" spans="1:21">
       <c r="A55" s="5"/>
       <c r="B55" s="5"/>
       <c r="C55" s="5"/>
@@ -2444,10 +2425,9 @@
       <c r="R55" s="5"/>
       <c r="S55" s="10"/>
       <c r="T55" s="5"/>
-      <c r="U55" s="5"/>
-      <c r="V55" s="11"/>
-    </row>
-    <row r="56" spans="1:22">
+      <c r="U55" s="11"/>
+    </row>
+    <row r="56" spans="1:21">
       <c r="A56" s="5"/>
       <c r="B56" s="5"/>
       <c r="C56" s="5"/>
@@ -2468,10 +2448,9 @@
       <c r="R56" s="5"/>
       <c r="S56" s="5"/>
       <c r="T56" s="5"/>
-      <c r="U56" s="5"/>
-      <c r="V56" s="11"/>
-    </row>
-    <row r="57" spans="1:22">
+      <c r="U56" s="11"/>
+    </row>
+    <row r="57" spans="1:21">
       <c r="A57" s="5"/>
       <c r="B57" s="5"/>
       <c r="C57" s="5"/>
@@ -2492,10 +2471,9 @@
       <c r="R57" s="5"/>
       <c r="S57" s="5"/>
       <c r="T57" s="5"/>
-      <c r="U57" s="5"/>
-      <c r="V57" s="11"/>
-    </row>
-    <row r="58" spans="1:22">
+      <c r="U57" s="11"/>
+    </row>
+    <row r="58" spans="1:21">
       <c r="A58" s="5"/>
       <c r="B58" s="5"/>
       <c r="C58" s="5"/>
@@ -2516,10 +2494,9 @@
       <c r="R58" s="5"/>
       <c r="S58" s="5"/>
       <c r="T58" s="5"/>
-      <c r="U58" s="5"/>
-      <c r="V58" s="11"/>
-    </row>
-    <row r="59" spans="1:22">
+      <c r="U58" s="11"/>
+    </row>
+    <row r="59" spans="1:21">
       <c r="A59" s="5"/>
       <c r="B59" s="5"/>
       <c r="C59" s="5"/>
@@ -2540,10 +2517,9 @@
       <c r="R59" s="5"/>
       <c r="S59" s="5"/>
       <c r="T59" s="5"/>
-      <c r="U59" s="5"/>
-      <c r="V59" s="11"/>
-    </row>
-    <row r="60" spans="1:22">
+      <c r="U59" s="11"/>
+    </row>
+    <row r="60" spans="1:21">
       <c r="A60" s="5"/>
       <c r="B60" s="5"/>
       <c r="C60" s="5"/>
@@ -2564,10 +2540,9 @@
       <c r="R60" s="5"/>
       <c r="S60" s="5"/>
       <c r="T60" s="5"/>
-      <c r="U60" s="5"/>
-      <c r="V60" s="11"/>
-    </row>
-    <row r="61" spans="1:22">
+      <c r="U60" s="11"/>
+    </row>
+    <row r="61" spans="1:21">
       <c r="A61" s="5"/>
       <c r="B61" s="5"/>
       <c r="C61" s="5"/>
@@ -2588,10 +2563,9 @@
       <c r="R61" s="5"/>
       <c r="S61" s="5"/>
       <c r="T61" s="5"/>
-      <c r="U61" s="5"/>
-      <c r="V61" s="11"/>
-    </row>
-    <row r="62" spans="1:22">
+      <c r="U61" s="11"/>
+    </row>
+    <row r="62" spans="1:21">
       <c r="A62" s="5"/>
       <c r="B62" s="5"/>
       <c r="C62" s="5"/>
@@ -2612,10 +2586,9 @@
       <c r="R62" s="5"/>
       <c r="S62" s="5"/>
       <c r="T62" s="5"/>
-      <c r="U62" s="5"/>
-      <c r="V62" s="11"/>
-    </row>
-    <row r="63" spans="1:22">
+      <c r="U62" s="11"/>
+    </row>
+    <row r="63" spans="1:21">
       <c r="A63" s="5"/>
       <c r="B63" s="5"/>
       <c r="C63" s="5"/>
@@ -2636,10 +2609,9 @@
       <c r="R63" s="5"/>
       <c r="S63" s="5"/>
       <c r="T63" s="5"/>
-      <c r="U63" s="5"/>
-      <c r="V63" s="11"/>
-    </row>
-    <row r="64" spans="1:22">
+      <c r="U63" s="11"/>
+    </row>
+    <row r="64" spans="1:21">
       <c r="A64" s="5"/>
       <c r="B64" s="5"/>
       <c r="C64" s="5"/>
@@ -2660,10 +2632,9 @@
       <c r="R64" s="5"/>
       <c r="S64" s="5"/>
       <c r="T64" s="5"/>
-      <c r="U64" s="5"/>
-      <c r="V64" s="11"/>
-    </row>
-    <row r="65" spans="1:22">
+      <c r="U64" s="11"/>
+    </row>
+    <row r="65" spans="1:21">
       <c r="A65" s="5"/>
       <c r="B65" s="5"/>
       <c r="C65" s="5"/>
@@ -2684,10 +2655,9 @@
       <c r="R65" s="5"/>
       <c r="S65" s="5"/>
       <c r="T65" s="5"/>
-      <c r="U65" s="5"/>
-      <c r="V65" s="11"/>
-    </row>
-    <row r="66" spans="1:22">
+      <c r="U65" s="11"/>
+    </row>
+    <row r="66" spans="1:21">
       <c r="A66" s="5"/>
       <c r="B66" s="5"/>
       <c r="C66" s="5"/>
@@ -2708,10 +2678,9 @@
       <c r="R66" s="5"/>
       <c r="S66" s="5"/>
       <c r="T66" s="5"/>
-      <c r="U66" s="5"/>
-      <c r="V66" s="11"/>
-    </row>
-    <row r="67" spans="1:22">
+      <c r="U66" s="11"/>
+    </row>
+    <row r="67" spans="1:21">
       <c r="A67" s="5"/>
       <c r="B67" s="5"/>
       <c r="C67" s="5"/>
@@ -2732,10 +2701,9 @@
       <c r="R67" s="5"/>
       <c r="S67" s="5"/>
       <c r="T67" s="5"/>
-      <c r="U67" s="5"/>
-      <c r="V67" s="11"/>
-    </row>
-    <row r="68" spans="1:22">
+      <c r="U67" s="11"/>
+    </row>
+    <row r="68" spans="1:21">
       <c r="A68" s="5"/>
       <c r="B68" s="5"/>
       <c r="C68" s="5"/>
@@ -2756,10 +2724,9 @@
       <c r="R68" s="5"/>
       <c r="S68" s="5"/>
       <c r="T68" s="5"/>
-      <c r="U68" s="5"/>
-      <c r="V68" s="11"/>
-    </row>
-    <row r="69" spans="1:22">
+      <c r="U68" s="11"/>
+    </row>
+    <row r="69" spans="1:21">
       <c r="A69" s="5"/>
       <c r="B69" s="5"/>
       <c r="C69" s="5"/>
@@ -2780,10 +2747,9 @@
       <c r="R69" s="5"/>
       <c r="S69" s="5"/>
       <c r="T69" s="5"/>
-      <c r="U69" s="5"/>
-      <c r="V69" s="11"/>
-    </row>
-    <row r="70" spans="1:22">
+      <c r="U69" s="11"/>
+    </row>
+    <row r="70" spans="1:21">
       <c r="A70" s="5"/>
       <c r="B70" s="5"/>
       <c r="C70" s="5"/>
@@ -2804,10 +2770,9 @@
       <c r="R70" s="5"/>
       <c r="S70" s="5"/>
       <c r="T70" s="5"/>
-      <c r="U70" s="5"/>
-      <c r="V70" s="11"/>
-    </row>
-    <row r="71" spans="1:22">
+      <c r="U70" s="11"/>
+    </row>
+    <row r="71" spans="1:21">
       <c r="A71" s="5"/>
       <c r="B71" s="5"/>
       <c r="C71" s="5"/>
@@ -2828,10 +2793,9 @@
       <c r="R71" s="5"/>
       <c r="S71" s="5"/>
       <c r="T71" s="5"/>
-      <c r="U71" s="5"/>
-      <c r="V71" s="11"/>
-    </row>
-    <row r="72" spans="1:22">
+      <c r="U71" s="11"/>
+    </row>
+    <row r="72" spans="1:21">
       <c r="A72" s="5"/>
       <c r="B72" s="5"/>
       <c r="C72" s="5"/>
@@ -2852,10 +2816,9 @@
       <c r="R72" s="5"/>
       <c r="S72" s="5"/>
       <c r="T72" s="5"/>
-      <c r="U72" s="5"/>
-      <c r="V72" s="11"/>
-    </row>
-    <row r="73" spans="1:22">
+      <c r="U72" s="11"/>
+    </row>
+    <row r="73" spans="1:21">
       <c r="A73" s="5"/>
       <c r="B73" s="5"/>
       <c r="C73" s="5"/>
@@ -2876,10 +2839,9 @@
       <c r="R73" s="5"/>
       <c r="S73" s="5"/>
       <c r="T73" s="5"/>
-      <c r="U73" s="5"/>
-      <c r="V73" s="11"/>
-    </row>
-    <row r="74" spans="1:22">
+      <c r="U73" s="11"/>
+    </row>
+    <row r="74" spans="1:21">
       <c r="A74" s="5"/>
       <c r="B74" s="5"/>
       <c r="C74" s="5"/>
@@ -2900,10 +2862,9 @@
       <c r="R74" s="5"/>
       <c r="S74" s="5"/>
       <c r="T74" s="5"/>
-      <c r="U74" s="5"/>
-      <c r="V74" s="11"/>
-    </row>
-    <row r="75" spans="1:22">
+      <c r="U74" s="11"/>
+    </row>
+    <row r="75" spans="1:21">
       <c r="A75" s="5"/>
       <c r="B75" s="5"/>
       <c r="C75" s="5"/>
@@ -2924,10 +2885,9 @@
       <c r="R75" s="5"/>
       <c r="S75" s="5"/>
       <c r="T75" s="5"/>
-      <c r="U75" s="5"/>
-      <c r="V75" s="11"/>
-    </row>
-    <row r="76" spans="1:22">
+      <c r="U75" s="11"/>
+    </row>
+    <row r="76" spans="1:21">
       <c r="A76" s="5"/>
       <c r="B76" s="5"/>
       <c r="C76" s="5"/>
@@ -2948,10 +2908,9 @@
       <c r="R76" s="5"/>
       <c r="S76" s="5"/>
       <c r="T76" s="5"/>
-      <c r="U76" s="5"/>
-      <c r="V76" s="11"/>
-    </row>
-    <row r="77" spans="1:22">
+      <c r="U76" s="11"/>
+    </row>
+    <row r="77" spans="1:21">
       <c r="A77" s="5"/>
       <c r="B77" s="5"/>
       <c r="C77" s="5"/>
@@ -2972,10 +2931,9 @@
       <c r="R77" s="5"/>
       <c r="S77" s="5"/>
       <c r="T77" s="5"/>
-      <c r="U77" s="5"/>
-      <c r="V77" s="11"/>
-    </row>
-    <row r="78" spans="1:22">
+      <c r="U77" s="11"/>
+    </row>
+    <row r="78" spans="1:21">
       <c r="A78" s="5"/>
       <c r="B78" s="5"/>
       <c r="C78" s="5"/>
@@ -2996,10 +2954,9 @@
       <c r="R78" s="5"/>
       <c r="S78" s="5"/>
       <c r="T78" s="5"/>
-      <c r="U78" s="5"/>
-      <c r="V78" s="11"/>
-    </row>
-    <row r="79" spans="1:22">
+      <c r="U78" s="11"/>
+    </row>
+    <row r="79" spans="1:21">
       <c r="A79" s="5"/>
       <c r="B79" s="5"/>
       <c r="C79" s="5"/>
@@ -3020,10 +2977,9 @@
       <c r="R79" s="5"/>
       <c r="S79" s="5"/>
       <c r="T79" s="5"/>
-      <c r="U79" s="5"/>
-      <c r="V79" s="11"/>
-    </row>
-    <row r="80" spans="1:22">
+      <c r="U79" s="11"/>
+    </row>
+    <row r="80" spans="1:21">
       <c r="A80" s="5"/>
       <c r="B80" s="5"/>
       <c r="C80" s="5"/>
@@ -3044,10 +3000,9 @@
       <c r="R80" s="5"/>
       <c r="S80" s="5"/>
       <c r="T80" s="5"/>
-      <c r="U80" s="5"/>
-      <c r="V80" s="11"/>
-    </row>
-    <row r="81" spans="1:22">
+      <c r="U80" s="11"/>
+    </row>
+    <row r="81" spans="1:21">
       <c r="A81" s="5"/>
       <c r="B81" s="5"/>
       <c r="C81" s="5"/>
@@ -3068,10 +3023,9 @@
       <c r="R81" s="5"/>
       <c r="S81" s="5"/>
       <c r="T81" s="5"/>
-      <c r="U81" s="5"/>
-      <c r="V81" s="11"/>
-    </row>
-    <row r="82" spans="1:22">
+      <c r="U81" s="11"/>
+    </row>
+    <row r="82" spans="1:21">
       <c r="A82" s="5"/>
       <c r="B82" s="5"/>
       <c r="C82" s="5"/>
@@ -3092,10 +3046,9 @@
       <c r="R82" s="5"/>
       <c r="S82" s="5"/>
       <c r="T82" s="5"/>
-      <c r="U82" s="5"/>
-      <c r="V82" s="11"/>
-    </row>
-    <row r="83" spans="1:22">
+      <c r="U82" s="11"/>
+    </row>
+    <row r="83" spans="1:21">
       <c r="A83" s="5"/>
       <c r="B83" s="5"/>
       <c r="C83" s="5"/>
@@ -3116,10 +3069,9 @@
       <c r="R83" s="5"/>
       <c r="S83" s="5"/>
       <c r="T83" s="5"/>
-      <c r="U83" s="5"/>
-      <c r="V83" s="11"/>
-    </row>
-    <row r="84" spans="1:22">
+      <c r="U83" s="11"/>
+    </row>
+    <row r="84" spans="1:21">
       <c r="A84" s="5"/>
       <c r="B84" s="5"/>
       <c r="C84" s="5"/>
@@ -3140,10 +3092,9 @@
       <c r="R84" s="5"/>
       <c r="S84" s="5"/>
       <c r="T84" s="5"/>
-      <c r="U84" s="5"/>
-      <c r="V84" s="11"/>
-    </row>
-    <row r="85" spans="1:22">
+      <c r="U84" s="11"/>
+    </row>
+    <row r="85" spans="1:21">
       <c r="A85" s="5"/>
       <c r="B85" s="5"/>
       <c r="C85" s="5"/>
@@ -3164,10 +3115,9 @@
       <c r="R85" s="5"/>
       <c r="S85" s="5"/>
       <c r="T85" s="5"/>
-      <c r="U85" s="5"/>
-      <c r="V85" s="11"/>
-    </row>
-    <row r="86" spans="1:22">
+      <c r="U85" s="11"/>
+    </row>
+    <row r="86" spans="1:21">
       <c r="A86" s="5"/>
       <c r="B86" s="5"/>
       <c r="C86" s="5"/>
@@ -3188,10 +3138,9 @@
       <c r="R86" s="5"/>
       <c r="S86" s="5"/>
       <c r="T86" s="5"/>
-      <c r="U86" s="5"/>
-      <c r="V86" s="11"/>
-    </row>
-    <row r="87" spans="1:22">
+      <c r="U86" s="11"/>
+    </row>
+    <row r="87" spans="1:21">
       <c r="A87" s="5"/>
       <c r="B87" s="5"/>
       <c r="C87" s="5"/>
@@ -3212,10 +3161,9 @@
       <c r="R87" s="5"/>
       <c r="S87" s="5"/>
       <c r="T87" s="5"/>
-      <c r="U87" s="5"/>
-      <c r="V87" s="11"/>
-    </row>
-    <row r="88" spans="1:22">
+      <c r="U87" s="11"/>
+    </row>
+    <row r="88" spans="1:21">
       <c r="A88" s="5"/>
       <c r="B88" s="5"/>
       <c r="C88" s="5"/>
@@ -3236,10 +3184,9 @@
       <c r="R88" s="5"/>
       <c r="S88" s="5"/>
       <c r="T88" s="5"/>
-      <c r="U88" s="5"/>
-      <c r="V88" s="11"/>
-    </row>
-    <row r="89" spans="1:22">
+      <c r="U88" s="11"/>
+    </row>
+    <row r="89" spans="1:21">
       <c r="A89" s="5"/>
       <c r="B89" s="5"/>
       <c r="C89" s="5"/>
@@ -3260,10 +3207,9 @@
       <c r="R89" s="5"/>
       <c r="S89" s="5"/>
       <c r="T89" s="5"/>
-      <c r="U89" s="5"/>
-      <c r="V89" s="11"/>
-    </row>
-    <row r="90" spans="1:22">
+      <c r="U89" s="11"/>
+    </row>
+    <row r="90" spans="1:21">
       <c r="A90" s="5"/>
       <c r="B90" s="5"/>
       <c r="C90" s="5"/>
@@ -3284,10 +3230,9 @@
       <c r="R90" s="5"/>
       <c r="S90" s="5"/>
       <c r="T90" s="5"/>
-      <c r="U90" s="5"/>
-      <c r="V90" s="11"/>
-    </row>
-    <row r="91" spans="1:22" ht="14.25">
+      <c r="U90" s="11"/>
+    </row>
+    <row r="91" spans="1:21" ht="14.25">
       <c r="A91" s="5"/>
       <c r="B91" s="5"/>
       <c r="C91" s="5"/>
@@ -3308,10 +3253,9 @@
       <c r="R91" s="5"/>
       <c r="S91" s="5"/>
       <c r="T91" s="5"/>
-      <c r="U91" s="5"/>
-      <c r="V91" s="11"/>
-    </row>
-    <row r="92" spans="1:22">
+      <c r="U91" s="11"/>
+    </row>
+    <row r="92" spans="1:21">
       <c r="A92" s="5"/>
       <c r="B92" s="5"/>
       <c r="C92" s="5"/>
@@ -3332,10 +3276,9 @@
       <c r="R92" s="5"/>
       <c r="S92" s="5"/>
       <c r="T92" s="5"/>
-      <c r="U92" s="5"/>
-      <c r="V92" s="11"/>
-    </row>
-    <row r="93" spans="1:22">
+      <c r="U92" s="11"/>
+    </row>
+    <row r="93" spans="1:21">
       <c r="A93" s="5"/>
       <c r="B93" s="5"/>
       <c r="C93" s="5"/>
@@ -3356,10 +3299,9 @@
       <c r="R93" s="5"/>
       <c r="S93" s="5"/>
       <c r="T93" s="5"/>
-      <c r="U93" s="5"/>
-      <c r="V93" s="11"/>
-    </row>
-    <row r="94" spans="1:22">
+      <c r="U93" s="11"/>
+    </row>
+    <row r="94" spans="1:21">
       <c r="A94" s="5"/>
       <c r="B94" s="5"/>
       <c r="C94" s="5"/>
@@ -3380,10 +3322,9 @@
       <c r="R94" s="5"/>
       <c r="S94" s="5"/>
       <c r="T94" s="5"/>
-      <c r="U94" s="5"/>
-      <c r="V94" s="11"/>
-    </row>
-    <row r="95" spans="1:22">
+      <c r="U94" s="11"/>
+    </row>
+    <row r="95" spans="1:21">
       <c r="A95" s="5"/>
       <c r="B95" s="5"/>
       <c r="C95" s="5"/>
@@ -3404,10 +3345,9 @@
       <c r="R95" s="5"/>
       <c r="S95" s="5"/>
       <c r="T95" s="5"/>
-      <c r="U95" s="5"/>
-      <c r="V95" s="11"/>
-    </row>
-    <row r="96" spans="1:22">
+      <c r="U95" s="11"/>
+    </row>
+    <row r="96" spans="1:21">
       <c r="A96" s="5"/>
       <c r="B96" s="5"/>
       <c r="C96" s="5"/>
@@ -3428,10 +3368,9 @@
       <c r="R96" s="5"/>
       <c r="S96" s="5"/>
       <c r="T96" s="5"/>
-      <c r="U96" s="5"/>
-      <c r="V96" s="11"/>
-    </row>
-    <row r="97" spans="1:22">
+      <c r="U96" s="11"/>
+    </row>
+    <row r="97" spans="1:21">
       <c r="A97" s="5"/>
       <c r="B97" s="5"/>
       <c r="C97" s="5"/>
@@ -3452,10 +3391,9 @@
       <c r="R97" s="5"/>
       <c r="S97" s="5"/>
       <c r="T97" s="5"/>
-      <c r="U97" s="5"/>
-      <c r="V97" s="11"/>
-    </row>
-    <row r="98" spans="1:22" ht="14.25">
+      <c r="U97" s="11"/>
+    </row>
+    <row r="98" spans="1:21" ht="14.25">
       <c r="A98" s="5"/>
       <c r="B98" s="5"/>
       <c r="C98" s="5"/>
@@ -3476,10 +3414,9 @@
       <c r="R98" s="5"/>
       <c r="S98" s="5"/>
       <c r="T98" s="5"/>
-      <c r="U98" s="5"/>
-      <c r="V98" s="11"/>
-    </row>
-    <row r="99" spans="1:22">
+      <c r="U98" s="11"/>
+    </row>
+    <row r="99" spans="1:21">
       <c r="A99" s="5"/>
       <c r="B99" s="5"/>
       <c r="C99" s="5"/>
@@ -3500,10 +3437,9 @@
       <c r="R99" s="5"/>
       <c r="S99" s="5"/>
       <c r="T99" s="5"/>
-      <c r="U99" s="5"/>
-      <c r="V99" s="11"/>
-    </row>
-    <row r="100" spans="1:22">
+      <c r="U99" s="11"/>
+    </row>
+    <row r="100" spans="1:21">
       <c r="A100" s="5"/>
       <c r="B100" s="5"/>
       <c r="C100" s="5"/>
@@ -3524,10 +3460,9 @@
       <c r="R100" s="5"/>
       <c r="S100" s="5"/>
       <c r="T100" s="5"/>
-      <c r="U100" s="5"/>
-      <c r="V100" s="11"/>
-    </row>
-    <row r="101" spans="1:22">
+      <c r="U100" s="11"/>
+    </row>
+    <row r="101" spans="1:21">
       <c r="A101" s="5"/>
       <c r="B101" s="5"/>
       <c r="C101" s="5"/>
@@ -3548,10 +3483,9 @@
       <c r="R101" s="5"/>
       <c r="S101" s="5"/>
       <c r="T101" s="5"/>
-      <c r="U101" s="5"/>
-      <c r="V101" s="11"/>
-    </row>
-    <row r="102" spans="1:22">
+      <c r="U101" s="11"/>
+    </row>
+    <row r="102" spans="1:21">
       <c r="A102" s="5"/>
       <c r="B102" s="5"/>
       <c r="C102" s="5"/>
@@ -3572,10 +3506,9 @@
       <c r="R102" s="5"/>
       <c r="S102" s="5"/>
       <c r="T102" s="5"/>
-      <c r="U102" s="5"/>
-      <c r="V102" s="11"/>
-    </row>
-    <row r="103" spans="1:22">
+      <c r="U102" s="11"/>
+    </row>
+    <row r="103" spans="1:21">
       <c r="A103" s="5"/>
       <c r="B103" s="5"/>
       <c r="C103" s="5"/>
@@ -3596,10 +3529,9 @@
       <c r="R103" s="5"/>
       <c r="S103" s="5"/>
       <c r="T103" s="5"/>
-      <c r="U103" s="5"/>
-      <c r="V103" s="11"/>
-    </row>
-    <row r="104" spans="1:22">
+      <c r="U103" s="11"/>
+    </row>
+    <row r="104" spans="1:21">
       <c r="A104" s="5"/>
       <c r="B104" s="5"/>
       <c r="C104" s="5"/>
@@ -3620,10 +3552,9 @@
       <c r="R104" s="5"/>
       <c r="S104" s="5"/>
       <c r="T104" s="5"/>
-      <c r="U104" s="5"/>
-      <c r="V104" s="11"/>
-    </row>
-    <row r="105" spans="1:22" ht="14.25">
+      <c r="U104" s="11"/>
+    </row>
+    <row r="105" spans="1:21" ht="14.25">
       <c r="A105" s="5"/>
       <c r="B105" s="5"/>
       <c r="C105" s="5"/>
@@ -3644,10 +3575,9 @@
       <c r="R105" s="5"/>
       <c r="S105" s="5"/>
       <c r="T105" s="5"/>
-      <c r="U105" s="5"/>
-      <c r="V105" s="11"/>
-    </row>
-    <row r="106" spans="1:22">
+      <c r="U105" s="11"/>
+    </row>
+    <row r="106" spans="1:21">
       <c r="A106" s="5"/>
       <c r="B106" s="5"/>
       <c r="C106" s="5"/>
@@ -3668,10 +3598,9 @@
       <c r="R106" s="5"/>
       <c r="S106" s="5"/>
       <c r="T106" s="5"/>
-      <c r="U106" s="5"/>
-      <c r="V106" s="11"/>
-    </row>
-    <row r="107" spans="1:22">
+      <c r="U106" s="11"/>
+    </row>
+    <row r="107" spans="1:21">
       <c r="A107" s="5"/>
       <c r="B107" s="5"/>
       <c r="C107" s="5"/>
@@ -3692,10 +3621,9 @@
       <c r="R107" s="5"/>
       <c r="S107" s="5"/>
       <c r="T107" s="5"/>
-      <c r="U107" s="5"/>
-      <c r="V107" s="11"/>
-    </row>
-    <row r="108" spans="1:22">
+      <c r="U107" s="11"/>
+    </row>
+    <row r="108" spans="1:21">
       <c r="A108" s="5"/>
       <c r="B108" s="5"/>
       <c r="C108" s="5"/>
@@ -3716,10 +3644,9 @@
       <c r="R108" s="5"/>
       <c r="S108" s="5"/>
       <c r="T108" s="5"/>
-      <c r="U108" s="5"/>
-      <c r="V108" s="11"/>
-    </row>
-    <row r="109" spans="1:22">
+      <c r="U108" s="11"/>
+    </row>
+    <row r="109" spans="1:21">
       <c r="A109" s="5"/>
       <c r="B109" s="5"/>
       <c r="C109" s="5"/>
@@ -3740,10 +3667,9 @@
       <c r="R109" s="5"/>
       <c r="S109" s="5"/>
       <c r="T109" s="5"/>
-      <c r="U109" s="5"/>
-      <c r="V109" s="11"/>
-    </row>
-    <row r="110" spans="1:22">
+      <c r="U109" s="11"/>
+    </row>
+    <row r="110" spans="1:21">
       <c r="A110" s="5"/>
       <c r="B110" s="5"/>
       <c r="C110" s="5"/>
@@ -3764,10 +3690,9 @@
       <c r="R110" s="5"/>
       <c r="S110" s="5"/>
       <c r="T110" s="5"/>
-      <c r="U110" s="5"/>
-      <c r="V110" s="11"/>
-    </row>
-    <row r="111" spans="1:22">
+      <c r="U110" s="11"/>
+    </row>
+    <row r="111" spans="1:21">
       <c r="A111" s="5"/>
       <c r="B111" s="5"/>
       <c r="C111" s="5"/>
@@ -3788,10 +3713,9 @@
       <c r="R111" s="5"/>
       <c r="S111" s="5"/>
       <c r="T111" s="5"/>
-      <c r="U111" s="5"/>
-      <c r="V111" s="11"/>
-    </row>
-    <row r="112" spans="1:22">
+      <c r="U111" s="11"/>
+    </row>
+    <row r="112" spans="1:21">
       <c r="A112" s="5"/>
       <c r="B112" s="5"/>
       <c r="C112" s="5"/>
@@ -3812,10 +3736,9 @@
       <c r="R112" s="5"/>
       <c r="S112" s="5"/>
       <c r="T112" s="5"/>
-      <c r="U112" s="5"/>
-      <c r="V112" s="11"/>
-    </row>
-    <row r="113" spans="1:22">
+      <c r="U112" s="11"/>
+    </row>
+    <row r="113" spans="1:21">
       <c r="A113" s="5"/>
       <c r="B113" s="5"/>
       <c r="C113" s="5"/>
@@ -3836,10 +3759,9 @@
       <c r="R113" s="5"/>
       <c r="S113" s="5"/>
       <c r="T113" s="5"/>
-      <c r="U113" s="5"/>
-      <c r="V113" s="11"/>
-    </row>
-    <row r="114" spans="1:22">
+      <c r="U113" s="11"/>
+    </row>
+    <row r="114" spans="1:21">
       <c r="A114" s="5"/>
       <c r="B114" s="5"/>
       <c r="C114" s="5"/>
@@ -3860,10 +3782,9 @@
       <c r="R114" s="5"/>
       <c r="S114" s="5"/>
       <c r="T114" s="5"/>
-      <c r="U114" s="5"/>
-      <c r="V114" s="11"/>
-    </row>
-    <row r="115" spans="1:22">
+      <c r="U114" s="11"/>
+    </row>
+    <row r="115" spans="1:21">
       <c r="A115" s="5"/>
       <c r="B115" s="5"/>
       <c r="C115" s="5"/>
@@ -3884,10 +3805,9 @@
       <c r="R115" s="5"/>
       <c r="S115" s="5"/>
       <c r="T115" s="5"/>
-      <c r="U115" s="5"/>
-      <c r="V115" s="11"/>
-    </row>
-    <row r="116" spans="1:22">
+      <c r="U115" s="11"/>
+    </row>
+    <row r="116" spans="1:21">
       <c r="A116" s="5"/>
       <c r="B116" s="5"/>
       <c r="C116" s="5"/>
@@ -3908,10 +3828,9 @@
       <c r="R116" s="5"/>
       <c r="S116" s="5"/>
       <c r="T116" s="5"/>
-      <c r="U116" s="5"/>
-      <c r="V116" s="11"/>
-    </row>
-    <row r="117" spans="1:22">
+      <c r="U116" s="11"/>
+    </row>
+    <row r="117" spans="1:21">
       <c r="A117" s="5"/>
       <c r="B117" s="5"/>
       <c r="C117" s="5"/>
@@ -3932,10 +3851,9 @@
       <c r="R117" s="5"/>
       <c r="S117" s="5"/>
       <c r="T117" s="5"/>
-      <c r="U117" s="5"/>
-      <c r="V117" s="11"/>
-    </row>
-    <row r="118" spans="1:22">
+      <c r="U117" s="11"/>
+    </row>
+    <row r="118" spans="1:21">
       <c r="A118" s="5"/>
       <c r="B118" s="5"/>
       <c r="C118" s="5"/>
@@ -3956,10 +3874,9 @@
       <c r="R118" s="5"/>
       <c r="S118" s="5"/>
       <c r="T118" s="5"/>
-      <c r="U118" s="5"/>
-      <c r="V118" s="11"/>
-    </row>
-    <row r="119" spans="1:22">
+      <c r="U118" s="11"/>
+    </row>
+    <row r="119" spans="1:21">
       <c r="A119" s="5"/>
       <c r="B119" s="5"/>
       <c r="C119" s="5"/>
@@ -3980,10 +3897,9 @@
       <c r="R119" s="5"/>
       <c r="S119" s="5"/>
       <c r="T119" s="5"/>
-      <c r="U119" s="5"/>
-      <c r="V119" s="11"/>
-    </row>
-    <row r="120" spans="1:22">
+      <c r="U119" s="11"/>
+    </row>
+    <row r="120" spans="1:21">
       <c r="A120" s="5"/>
       <c r="B120" s="5"/>
       <c r="C120" s="5"/>
@@ -4004,10 +3920,9 @@
       <c r="R120" s="5"/>
       <c r="S120" s="5"/>
       <c r="T120" s="5"/>
-      <c r="U120" s="5"/>
-      <c r="V120" s="11"/>
-    </row>
-    <row r="121" spans="1:22">
+      <c r="U120" s="11"/>
+    </row>
+    <row r="121" spans="1:21">
       <c r="A121" s="5"/>
       <c r="B121" s="5"/>
       <c r="C121" s="5"/>
@@ -4028,10 +3943,9 @@
       <c r="R121" s="5"/>
       <c r="S121" s="5"/>
       <c r="T121" s="5"/>
-      <c r="U121" s="5"/>
-      <c r="V121" s="11"/>
-    </row>
-    <row r="122" spans="1:22">
+      <c r="U121" s="11"/>
+    </row>
+    <row r="122" spans="1:21">
       <c r="A122" s="5"/>
       <c r="B122" s="5"/>
       <c r="C122" s="5"/>
@@ -4052,10 +3966,9 @@
       <c r="R122" s="5"/>
       <c r="S122" s="5"/>
       <c r="T122" s="5"/>
-      <c r="U122" s="5"/>
-      <c r="V122" s="11"/>
-    </row>
-    <row r="123" spans="1:22">
+      <c r="U122" s="11"/>
+    </row>
+    <row r="123" spans="1:21">
       <c r="A123" s="5"/>
       <c r="B123" s="5"/>
       <c r="C123" s="5"/>
@@ -4076,10 +3989,9 @@
       <c r="R123" s="5"/>
       <c r="S123" s="5"/>
       <c r="T123" s="5"/>
-      <c r="U123" s="5"/>
-      <c r="V123" s="11"/>
-    </row>
-    <row r="124" spans="1:22">
+      <c r="U123" s="11"/>
+    </row>
+    <row r="124" spans="1:21">
       <c r="A124" s="5"/>
       <c r="B124" s="5"/>
       <c r="C124" s="5"/>
@@ -4100,10 +4012,9 @@
       <c r="R124" s="5"/>
       <c r="S124" s="5"/>
       <c r="T124" s="5"/>
-      <c r="U124" s="5"/>
-      <c r="V124" s="11"/>
-    </row>
-    <row r="125" spans="1:22">
+      <c r="U124" s="11"/>
+    </row>
+    <row r="125" spans="1:21">
       <c r="A125" s="5"/>
       <c r="B125" s="5"/>
       <c r="C125" s="5"/>
@@ -4124,10 +4035,9 @@
       <c r="R125" s="5"/>
       <c r="S125" s="5"/>
       <c r="T125" s="5"/>
-      <c r="U125" s="5"/>
-      <c r="V125" s="11"/>
-    </row>
-    <row r="126" spans="1:22">
+      <c r="U125" s="11"/>
+    </row>
+    <row r="126" spans="1:21">
       <c r="A126" s="5"/>
       <c r="B126" s="5"/>
       <c r="C126" s="5"/>
@@ -4148,10 +4058,9 @@
       <c r="R126" s="5"/>
       <c r="S126" s="5"/>
       <c r="T126" s="5"/>
-      <c r="U126" s="5"/>
-      <c r="V126" s="11"/>
-    </row>
-    <row r="127" spans="1:22">
+      <c r="U126" s="11"/>
+    </row>
+    <row r="127" spans="1:21">
       <c r="A127" s="5"/>
       <c r="B127" s="5"/>
       <c r="C127" s="5"/>
@@ -4172,10 +4081,9 @@
       <c r="R127" s="5"/>
       <c r="S127" s="5"/>
       <c r="T127" s="5"/>
-      <c r="U127" s="5"/>
-      <c r="V127" s="11"/>
-    </row>
-    <row r="128" spans="1:22">
+      <c r="U127" s="11"/>
+    </row>
+    <row r="128" spans="1:21">
       <c r="A128" s="5"/>
       <c r="B128" s="5"/>
       <c r="C128" s="5"/>
@@ -4196,10 +4104,9 @@
       <c r="R128" s="5"/>
       <c r="S128" s="5"/>
       <c r="T128" s="5"/>
-      <c r="U128" s="5"/>
-      <c r="V128" s="11"/>
-    </row>
-    <row r="129" spans="1:22">
+      <c r="U128" s="11"/>
+    </row>
+    <row r="129" spans="1:21">
       <c r="A129" s="5"/>
       <c r="B129" s="5"/>
       <c r="C129" s="5"/>
@@ -4220,10 +4127,9 @@
       <c r="R129" s="5"/>
       <c r="S129" s="5"/>
       <c r="T129" s="5"/>
-      <c r="U129" s="5"/>
-      <c r="V129" s="11"/>
-    </row>
-    <row r="130" spans="1:22">
+      <c r="U129" s="11"/>
+    </row>
+    <row r="130" spans="1:21">
       <c r="A130" s="5"/>
       <c r="B130" s="5"/>
       <c r="C130" s="5"/>
@@ -4244,10 +4150,9 @@
       <c r="R130" s="5"/>
       <c r="S130" s="5"/>
       <c r="T130" s="5"/>
-      <c r="U130" s="5"/>
-      <c r="V130" s="11"/>
-    </row>
-    <row r="131" spans="1:22">
+      <c r="U130" s="11"/>
+    </row>
+    <row r="131" spans="1:21">
       <c r="A131" s="5"/>
       <c r="B131" s="5"/>
       <c r="C131" s="5"/>
@@ -4268,10 +4173,9 @@
       <c r="R131" s="5"/>
       <c r="S131" s="5"/>
       <c r="T131" s="5"/>
-      <c r="U131" s="5"/>
-      <c r="V131" s="11"/>
-    </row>
-    <row r="132" spans="1:22">
+      <c r="U131" s="11"/>
+    </row>
+    <row r="132" spans="1:21">
       <c r="A132" s="5"/>
       <c r="B132" s="5"/>
       <c r="C132" s="5"/>
@@ -4292,10 +4196,9 @@
       <c r="R132" s="5"/>
       <c r="S132" s="11"/>
       <c r="T132" s="5"/>
-      <c r="U132" s="5"/>
-      <c r="V132" s="11"/>
-    </row>
-    <row r="133" spans="1:22">
+      <c r="U132" s="11"/>
+    </row>
+    <row r="133" spans="1:21">
       <c r="A133" s="5"/>
       <c r="B133" s="5"/>
       <c r="C133" s="5"/>
@@ -4316,10 +4219,9 @@
       <c r="R133" s="5"/>
       <c r="S133" s="11"/>
       <c r="T133" s="5"/>
-      <c r="U133" s="5"/>
-      <c r="V133" s="11"/>
-    </row>
-    <row r="134" spans="1:22">
+      <c r="U133" s="11"/>
+    </row>
+    <row r="134" spans="1:21">
       <c r="A134" s="5"/>
       <c r="B134" s="5"/>
       <c r="C134" s="5"/>
@@ -4340,10 +4242,9 @@
       <c r="R134" s="5"/>
       <c r="S134" s="11"/>
       <c r="T134" s="5"/>
-      <c r="U134" s="5"/>
-      <c r="V134" s="11"/>
-    </row>
-    <row r="135" spans="1:22">
+      <c r="U134" s="11"/>
+    </row>
+    <row r="135" spans="1:21">
       <c r="A135" s="5"/>
       <c r="B135" s="5"/>
       <c r="C135" s="5"/>
@@ -4364,10 +4265,9 @@
       <c r="R135" s="5"/>
       <c r="S135" s="11"/>
       <c r="T135" s="5"/>
-      <c r="U135" s="5"/>
-      <c r="V135" s="11"/>
-    </row>
-    <row r="136" spans="1:22">
+      <c r="U135" s="11"/>
+    </row>
+    <row r="136" spans="1:21">
       <c r="A136" s="5"/>
       <c r="B136" s="5"/>
       <c r="C136" s="5"/>
@@ -4388,10 +4288,9 @@
       <c r="R136" s="5"/>
       <c r="S136" s="11"/>
       <c r="T136" s="5"/>
-      <c r="U136" s="5"/>
-      <c r="V136" s="11"/>
-    </row>
-    <row r="137" spans="1:22">
+      <c r="U136" s="11"/>
+    </row>
+    <row r="137" spans="1:21">
       <c r="A137" s="5"/>
       <c r="B137" s="5"/>
       <c r="C137" s="5"/>
@@ -4412,10 +4311,9 @@
       <c r="R137" s="5"/>
       <c r="S137" s="11"/>
       <c r="T137" s="5"/>
-      <c r="U137" s="5"/>
-      <c r="V137" s="11"/>
-    </row>
-    <row r="138" spans="1:22">
+      <c r="U137" s="11"/>
+    </row>
+    <row r="138" spans="1:21">
       <c r="A138" s="5"/>
       <c r="B138" s="5"/>
       <c r="C138" s="5"/>
@@ -4436,10 +4334,9 @@
       <c r="R138" s="5"/>
       <c r="S138" s="11"/>
       <c r="T138" s="5"/>
-      <c r="U138" s="5"/>
-      <c r="V138" s="11"/>
-    </row>
-    <row r="139" spans="1:22">
+      <c r="U138" s="11"/>
+    </row>
+    <row r="139" spans="1:21">
       <c r="A139" s="5"/>
       <c r="B139" s="5"/>
       <c r="C139" s="5"/>
@@ -4460,10 +4357,9 @@
       <c r="R139" s="5"/>
       <c r="S139" s="11"/>
       <c r="T139" s="5"/>
-      <c r="U139" s="5"/>
-      <c r="V139" s="11"/>
-    </row>
-    <row r="140" spans="1:22">
+      <c r="U139" s="11"/>
+    </row>
+    <row r="140" spans="1:21">
       <c r="A140" s="5"/>
       <c r="B140" s="5"/>
       <c r="C140" s="5"/>
@@ -4484,10 +4380,9 @@
       <c r="R140" s="5"/>
       <c r="S140" s="11"/>
       <c r="T140" s="5"/>
-      <c r="U140" s="5"/>
-      <c r="V140" s="11"/>
-    </row>
-    <row r="141" spans="1:22" s="16" customFormat="1">
+      <c r="U140" s="11"/>
+    </row>
+    <row r="141" spans="1:21" s="16" customFormat="1">
       <c r="A141" s="5"/>
       <c r="B141" s="5"/>
       <c r="C141" s="5"/>
@@ -4508,10 +4403,9 @@
       <c r="R141" s="5"/>
       <c r="S141" s="5"/>
       <c r="T141" s="5"/>
-      <c r="U141" s="5"/>
-      <c r="V141" s="11"/>
-    </row>
-    <row r="142" spans="1:22" s="17" customFormat="1">
+      <c r="U141" s="11"/>
+    </row>
+    <row r="142" spans="1:21" s="17" customFormat="1">
       <c r="A142" s="5"/>
       <c r="B142" s="5"/>
       <c r="C142" s="5"/>
@@ -4532,10 +4426,9 @@
       <c r="R142" s="5"/>
       <c r="S142" s="5"/>
       <c r="T142" s="5"/>
-      <c r="U142" s="5"/>
-      <c r="V142" s="11"/>
-    </row>
-    <row r="143" spans="1:22" s="17" customFormat="1">
+      <c r="U142" s="11"/>
+    </row>
+    <row r="143" spans="1:21" s="17" customFormat="1">
       <c r="A143" s="5"/>
       <c r="B143" s="5"/>
       <c r="C143" s="5"/>
@@ -4556,10 +4449,9 @@
       <c r="R143" s="5"/>
       <c r="S143" s="5"/>
       <c r="T143" s="5"/>
-      <c r="U143" s="5"/>
-      <c r="V143" s="11"/>
-    </row>
-    <row r="144" spans="1:22" s="17" customFormat="1">
+      <c r="U143" s="11"/>
+    </row>
+    <row r="144" spans="1:21" s="17" customFormat="1">
       <c r="A144" s="5"/>
       <c r="B144" s="5"/>
       <c r="C144" s="5"/>
@@ -4580,10 +4472,9 @@
       <c r="R144" s="5"/>
       <c r="S144" s="18"/>
       <c r="T144" s="5"/>
-      <c r="U144" s="5"/>
-      <c r="V144" s="11"/>
-    </row>
-    <row r="145" spans="1:22" s="17" customFormat="1">
+      <c r="U144" s="11"/>
+    </row>
+    <row r="145" spans="1:21" s="17" customFormat="1">
       <c r="A145" s="5"/>
       <c r="B145" s="5"/>
       <c r="C145" s="5"/>
@@ -4604,10 +4495,9 @@
       <c r="R145" s="5"/>
       <c r="S145" s="5"/>
       <c r="T145" s="5"/>
-      <c r="U145" s="5"/>
-      <c r="V145" s="11"/>
-    </row>
-    <row r="146" spans="1:22" s="17" customFormat="1">
+      <c r="U145" s="11"/>
+    </row>
+    <row r="146" spans="1:21" s="17" customFormat="1">
       <c r="A146" s="5"/>
       <c r="B146" s="5"/>
       <c r="C146" s="5"/>
@@ -4628,10 +4518,9 @@
       <c r="R146" s="5"/>
       <c r="S146" s="18"/>
       <c r="T146" s="5"/>
-      <c r="U146" s="5"/>
-      <c r="V146" s="11"/>
-    </row>
-    <row r="147" spans="1:22" s="17" customFormat="1">
+      <c r="U146" s="11"/>
+    </row>
+    <row r="147" spans="1:21" s="17" customFormat="1">
       <c r="A147" s="5"/>
       <c r="B147" s="5"/>
       <c r="C147" s="5"/>
@@ -4652,10 +4541,9 @@
       <c r="R147" s="5"/>
       <c r="S147" s="5"/>
       <c r="T147" s="5"/>
-      <c r="U147" s="5"/>
-      <c r="V147" s="11"/>
-    </row>
-    <row r="148" spans="1:22" s="17" customFormat="1">
+      <c r="U147" s="11"/>
+    </row>
+    <row r="148" spans="1:21" s="17" customFormat="1">
       <c r="A148" s="5"/>
       <c r="B148" s="5"/>
       <c r="C148" s="5"/>
@@ -4676,10 +4564,9 @@
       <c r="R148" s="5"/>
       <c r="S148" s="5"/>
       <c r="T148" s="5"/>
-      <c r="U148" s="5"/>
-      <c r="V148" s="11"/>
-    </row>
-    <row r="149" spans="1:22" s="17" customFormat="1">
+      <c r="U148" s="11"/>
+    </row>
+    <row r="149" spans="1:21" s="17" customFormat="1">
       <c r="A149" s="5"/>
       <c r="B149" s="5"/>
       <c r="C149" s="5"/>
@@ -4700,10 +4587,9 @@
       <c r="R149" s="5"/>
       <c r="S149" s="5"/>
       <c r="T149" s="5"/>
-      <c r="U149" s="5"/>
-      <c r="V149" s="11"/>
-    </row>
-    <row r="150" spans="1:22" s="17" customFormat="1">
+      <c r="U149" s="11"/>
+    </row>
+    <row r="150" spans="1:21" s="17" customFormat="1">
       <c r="A150" s="5"/>
       <c r="B150" s="5"/>
       <c r="C150" s="5"/>
@@ -4724,10 +4610,9 @@
       <c r="R150" s="5"/>
       <c r="S150" s="18"/>
       <c r="T150" s="5"/>
-      <c r="U150" s="5"/>
-      <c r="V150" s="11"/>
-    </row>
-    <row r="151" spans="1:22">
+      <c r="U150" s="11"/>
+    </row>
+    <row r="151" spans="1:21">
       <c r="A151" s="5"/>
       <c r="B151" s="5"/>
       <c r="C151" s="5"/>
@@ -4748,10 +4633,9 @@
       <c r="R151" s="5"/>
       <c r="S151" s="5"/>
       <c r="T151" s="5"/>
-      <c r="U151" s="5"/>
-      <c r="V151" s="11"/>
-    </row>
-    <row r="152" spans="1:22" s="17" customFormat="1">
+      <c r="U151" s="11"/>
+    </row>
+    <row r="152" spans="1:21" s="17" customFormat="1">
       <c r="A152" s="5"/>
       <c r="B152" s="5"/>
       <c r="C152" s="5"/>
@@ -4772,10 +4656,9 @@
       <c r="R152" s="5"/>
       <c r="S152" s="5"/>
       <c r="T152" s="5"/>
-      <c r="U152" s="5"/>
-      <c r="V152" s="11"/>
-    </row>
-    <row r="153" spans="1:22">
+      <c r="U152" s="11"/>
+    </row>
+    <row r="153" spans="1:21">
       <c r="A153" s="5"/>
       <c r="B153" s="5"/>
       <c r="C153" s="5"/>
@@ -4796,10 +4679,9 @@
       <c r="R153" s="5"/>
       <c r="S153" s="5"/>
       <c r="T153" s="5"/>
-      <c r="U153" s="5"/>
-      <c r="V153" s="11"/>
-    </row>
-    <row r="154" spans="1:22" s="17" customFormat="1">
+      <c r="U153" s="11"/>
+    </row>
+    <row r="154" spans="1:21" s="17" customFormat="1">
       <c r="A154" s="5"/>
       <c r="B154" s="5"/>
       <c r="C154" s="5"/>
@@ -4820,11 +4702,10 @@
       <c r="R154" s="5"/>
       <c r="S154" s="5"/>
       <c r="T154" s="5"/>
-      <c r="U154" s="5"/>
-      <c r="V154" s="11"/>
+      <c r="U154" s="11"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V1" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
+  <autoFilter ref="A1:U1" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
   <dataConsolidate/>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="1">
@@ -4832,9 +4713,13 @@
       <formula1>"Smoke,Sanity,Regression"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="D3" r:id="rId1" location="collapse2" display="https://automationexercise.com/api_list - collapse2" xr:uid="{4CB74369-E6C3-4251-A75E-F43B9505B933}"/>
+    <hyperlink ref="D2" r:id="rId2" location="collapse1" display="https://automationexercise.com/api_list - collapse1" xr:uid="{E10F699E-A2FA-4AA4-AD4F-F02AFFC6D94A}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
-  <legacyDrawing r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <drawing r:id="rId4"/>
+  <legacyDrawing r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
modify function calling in excel test case
</commit_message>
<xml_diff>
--- a/projects/automation_exercise/api/case/testcase-automation_exercise.xlsx
+++ b/projects/automation_exercise/api/case/testcase-automation_exercise.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/606929f86db40629/Documents/Python/automation_framework/projects/automation_exercise/api/case/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="8_{B959E1B4-B71D-476A-B78C-D11EC8419DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AABE53F2-9EE6-4B15-B3DD-CF0BBFA87018}"/>
+  <xr:revisionPtr revIDLastSave="72" documentId="8_{B959E1B4-B71D-476A-B78C-D11EC8419DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3429BE0B-1A9D-4980-BE0F-62970DB06951}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AB49B25E-9B57-422D-B60E-7F12796728DD}"/>
   </bookViews>
   <sheets>
-    <sheet name="Products" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Products!$A$1:$U$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$V$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -364,11 +364,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="35">
-  <si>
-    <t>JIRA ID</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="38">
   <si>
     <t>Case_Name</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -390,51 +386,11 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>New Session</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>SetUp</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Specify Header</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Header Content</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Root_URL</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>relative_URL</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Request Type</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Request Data</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Expected Code</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Expected Text</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Compare Method</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Set Global Variable</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -473,15 +429,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Data Type</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>["=","$.responseCode",200];</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Json Result Validation</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -501,6 +449,70 @@
   <si>
     <t>["=","$.responseCode",405];
 ["=","$.message","This request method is not supported."]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>New_Session</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Requirement_ID</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Specify_Header</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Header_Content</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Request_Type</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Data_Type</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Request_Data</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Expected_Code</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Expected_Text</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Compare_Method</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Json_Result_Validation</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Set_Global_Variable</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Tear_Down</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Set_Up</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>${projects.automation_exercise.libs.demo.py::function_used_by_setup()}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>${projects.automation_exercise.libs.demo.py::function_used_by_teardown()}</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -706,15 +718,15 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>1800</xdr:row>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>1047750</xdr:colOff>
+      <xdr:row>1795</xdr:row>
       <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>647700</xdr:colOff>
-      <xdr:row>1955</xdr:row>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>142875</xdr:colOff>
+      <xdr:row>1950</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -754,10 +766,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1047,10 +1055,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{571522A3-8A90-45FA-BDC2-DE8E1EFD9C0E}">
-  <dimension ref="A1:U154"/>
+  <dimension ref="A1:V154"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="8.5" style="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.125" style="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.5" style="12" customWidth="1"/>
     <col min="3" max="3" width="8.125" style="12" customWidth="1"/>
     <col min="4" max="4" width="15.25" style="12" customWidth="1"/>
@@ -1067,107 +1075,110 @@
     <col min="17" max="17" width="13.875" style="12" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="16.125" style="12" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="53.75" style="12" customWidth="1"/>
-    <col min="20" max="20" width="15" style="12" customWidth="1"/>
-    <col min="21" max="21" width="27.875" style="12" customWidth="1"/>
-    <col min="22" max="16384" width="9" style="12"/>
+    <col min="20" max="21" width="15" style="12" customWidth="1"/>
+    <col min="22" max="22" width="27.875" style="12" customWidth="1"/>
+    <col min="23" max="16384" width="9" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="8" customFormat="1" ht="27">
+    <row r="1" spans="1:22" s="8" customFormat="1" ht="27">
       <c r="A1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
       <c r="M1" s="1" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>27</v>
       </c>
       <c r="O1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="P1" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q1" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="U1" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="V1" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" ht="67.5">
+      <c r="A2" s="5"/>
+      <c r="B2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="C2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="U1" s="7" t="s">
+      <c r="D2" s="19" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" ht="27">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D2" s="19" t="s">
-        <v>31</v>
-      </c>
       <c r="E2" s="5" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
-      <c r="G2" s="5" t="s">
-        <v>19</v>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5" t="s">
+        <v>36</v>
       </c>
-      <c r="H2" s="5"/>
       <c r="I2" s="5"/>
       <c r="J2" s="5"/>
       <c r="K2" s="5" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="L2" s="9" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="N2" s="5"/>
       <c r="O2" s="5"/>
@@ -1177,44 +1188,45 @@
       <c r="Q2" s="10"/>
       <c r="R2" s="5"/>
       <c r="S2" s="5" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="T2" s="5"/>
-      <c r="U2" s="11" t="s">
-        <v>23</v>
+      <c r="U2" s="5"/>
+      <c r="V2" s="11" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:21" ht="40.5">
+    <row r="3" spans="1:22" ht="67.5">
       <c r="A3" s="5"/>
       <c r="B3" s="5" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="D3" s="19" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
-      <c r="G3" s="5" t="s">
-        <v>19</v>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5" t="s">
+        <v>37</v>
       </c>
-      <c r="H3" s="5"/>
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
       <c r="K3" s="5" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="M3" s="5" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="N3" s="5"/>
       <c r="O3" s="5"/>
@@ -1224,14 +1236,15 @@
       <c r="Q3" s="10"/>
       <c r="R3" s="5"/>
       <c r="S3" s="5" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="T3" s="5"/>
-      <c r="U3" s="11" t="s">
-        <v>23</v>
+      <c r="U3" s="5"/>
+      <c r="V3" s="11" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:21">
+    <row r="4" spans="1:22">
       <c r="A4" s="5"/>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -1252,9 +1265,10 @@
       <c r="R4" s="5"/>
       <c r="S4" s="5"/>
       <c r="T4" s="5"/>
-      <c r="U4" s="11"/>
-    </row>
-    <row r="5" spans="1:21">
+      <c r="U4" s="5"/>
+      <c r="V4" s="11"/>
+    </row>
+    <row r="5" spans="1:22">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -1275,9 +1289,10 @@
       <c r="R5" s="5"/>
       <c r="S5" s="5"/>
       <c r="T5" s="5"/>
-      <c r="U5" s="11"/>
-    </row>
-    <row r="6" spans="1:21">
+      <c r="U5" s="5"/>
+      <c r="V5" s="11"/>
+    </row>
+    <row r="6" spans="1:22">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
@@ -1298,9 +1313,10 @@
       <c r="R6" s="5"/>
       <c r="S6" s="5"/>
       <c r="T6" s="5"/>
-      <c r="U6" s="11"/>
-    </row>
-    <row r="7" spans="1:21">
+      <c r="U6" s="5"/>
+      <c r="V6" s="11"/>
+    </row>
+    <row r="7" spans="1:22">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
@@ -1321,9 +1337,10 @@
       <c r="R7" s="5"/>
       <c r="S7" s="5"/>
       <c r="T7" s="5"/>
-      <c r="U7" s="11"/>
-    </row>
-    <row r="8" spans="1:21">
+      <c r="U7" s="5"/>
+      <c r="V7" s="11"/>
+    </row>
+    <row r="8" spans="1:22">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -1344,9 +1361,10 @@
       <c r="R8" s="5"/>
       <c r="S8" s="5"/>
       <c r="T8" s="5"/>
-      <c r="U8" s="11"/>
-    </row>
-    <row r="9" spans="1:21">
+      <c r="U8" s="5"/>
+      <c r="V8" s="11"/>
+    </row>
+    <row r="9" spans="1:22">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
@@ -1367,9 +1385,10 @@
       <c r="R9" s="5"/>
       <c r="S9" s="5"/>
       <c r="T9" s="5"/>
-      <c r="U9" s="11"/>
-    </row>
-    <row r="10" spans="1:21">
+      <c r="U9" s="5"/>
+      <c r="V9" s="11"/>
+    </row>
+    <row r="10" spans="1:22">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -1390,9 +1409,10 @@
       <c r="R10" s="5"/>
       <c r="S10" s="5"/>
       <c r="T10" s="5"/>
-      <c r="U10" s="11"/>
-    </row>
-    <row r="11" spans="1:21">
+      <c r="U10" s="5"/>
+      <c r="V10" s="11"/>
+    </row>
+    <row r="11" spans="1:22">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -1413,9 +1433,10 @@
       <c r="R11" s="5"/>
       <c r="S11" s="5"/>
       <c r="T11" s="5"/>
-      <c r="U11" s="11"/>
-    </row>
-    <row r="12" spans="1:21">
+      <c r="U11" s="5"/>
+      <c r="V11" s="11"/>
+    </row>
+    <row r="12" spans="1:22">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -1436,9 +1457,10 @@
       <c r="R12" s="5"/>
       <c r="S12" s="5"/>
       <c r="T12" s="5"/>
-      <c r="U12" s="11"/>
-    </row>
-    <row r="13" spans="1:21">
+      <c r="U12" s="5"/>
+      <c r="V12" s="11"/>
+    </row>
+    <row r="13" spans="1:22">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -1459,9 +1481,10 @@
       <c r="R13" s="5"/>
       <c r="S13" s="5"/>
       <c r="T13" s="5"/>
-      <c r="U13" s="11"/>
-    </row>
-    <row r="14" spans="1:21">
+      <c r="U13" s="5"/>
+      <c r="V13" s="11"/>
+    </row>
+    <row r="14" spans="1:22">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -1482,9 +1505,10 @@
       <c r="R14" s="5"/>
       <c r="S14" s="5"/>
       <c r="T14" s="5"/>
-      <c r="U14" s="11"/>
-    </row>
-    <row r="15" spans="1:21">
+      <c r="U14" s="5"/>
+      <c r="V14" s="11"/>
+    </row>
+    <row r="15" spans="1:22">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -1505,9 +1529,10 @@
       <c r="R15" s="5"/>
       <c r="S15" s="5"/>
       <c r="T15" s="5"/>
-      <c r="U15" s="11"/>
-    </row>
-    <row r="16" spans="1:21">
+      <c r="U15" s="5"/>
+      <c r="V15" s="11"/>
+    </row>
+    <row r="16" spans="1:22">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -1528,9 +1553,10 @@
       <c r="R16" s="5"/>
       <c r="S16" s="5"/>
       <c r="T16" s="5"/>
-      <c r="U16" s="11"/>
-    </row>
-    <row r="17" spans="1:21">
+      <c r="U16" s="5"/>
+      <c r="V16" s="11"/>
+    </row>
+    <row r="17" spans="1:22">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -1551,9 +1577,10 @@
       <c r="R17" s="5"/>
       <c r="S17" s="5"/>
       <c r="T17" s="5"/>
-      <c r="U17" s="11"/>
-    </row>
-    <row r="18" spans="1:21">
+      <c r="U17" s="5"/>
+      <c r="V17" s="11"/>
+    </row>
+    <row r="18" spans="1:22">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -1574,9 +1601,10 @@
       <c r="R18" s="5"/>
       <c r="S18" s="5"/>
       <c r="T18" s="5"/>
-      <c r="U18" s="11"/>
-    </row>
-    <row r="19" spans="1:21">
+      <c r="U18" s="5"/>
+      <c r="V18" s="11"/>
+    </row>
+    <row r="19" spans="1:22">
       <c r="A19" s="5"/>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -1597,9 +1625,10 @@
       <c r="R19" s="5"/>
       <c r="S19" s="5"/>
       <c r="T19" s="5"/>
-      <c r="U19" s="11"/>
-    </row>
-    <row r="20" spans="1:21">
+      <c r="U19" s="5"/>
+      <c r="V19" s="11"/>
+    </row>
+    <row r="20" spans="1:22">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -1620,9 +1649,10 @@
       <c r="R20" s="5"/>
       <c r="S20" s="5"/>
       <c r="T20" s="5"/>
-      <c r="U20" s="11"/>
-    </row>
-    <row r="21" spans="1:21">
+      <c r="U20" s="5"/>
+      <c r="V20" s="11"/>
+    </row>
+    <row r="21" spans="1:22">
       <c r="A21" s="5"/>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -1643,9 +1673,10 @@
       <c r="R21" s="5"/>
       <c r="S21" s="5"/>
       <c r="T21" s="5"/>
-      <c r="U21" s="11"/>
-    </row>
-    <row r="22" spans="1:21">
+      <c r="U21" s="5"/>
+      <c r="V21" s="11"/>
+    </row>
+    <row r="22" spans="1:22">
       <c r="A22" s="5"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -1666,9 +1697,10 @@
       <c r="R22" s="5"/>
       <c r="S22" s="5"/>
       <c r="T22" s="5"/>
-      <c r="U22" s="11"/>
-    </row>
-    <row r="23" spans="1:21">
+      <c r="U22" s="5"/>
+      <c r="V22" s="11"/>
+    </row>
+    <row r="23" spans="1:22">
       <c r="A23" s="5"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -1689,9 +1721,10 @@
       <c r="R23" s="5"/>
       <c r="S23" s="5"/>
       <c r="T23" s="5"/>
-      <c r="U23" s="11"/>
-    </row>
-    <row r="24" spans="1:21">
+      <c r="U23" s="5"/>
+      <c r="V23" s="11"/>
+    </row>
+    <row r="24" spans="1:22">
       <c r="A24" s="5"/>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
@@ -1712,9 +1745,10 @@
       <c r="R24" s="5"/>
       <c r="S24" s="5"/>
       <c r="T24" s="5"/>
-      <c r="U24" s="11"/>
-    </row>
-    <row r="25" spans="1:21">
+      <c r="U24" s="5"/>
+      <c r="V24" s="11"/>
+    </row>
+    <row r="25" spans="1:22">
       <c r="A25" s="5"/>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -1735,9 +1769,10 @@
       <c r="R25" s="5"/>
       <c r="S25" s="5"/>
       <c r="T25" s="5"/>
-      <c r="U25" s="11"/>
-    </row>
-    <row r="26" spans="1:21">
+      <c r="U25" s="5"/>
+      <c r="V25" s="11"/>
+    </row>
+    <row r="26" spans="1:22">
       <c r="A26" s="5"/>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
@@ -1758,9 +1793,10 @@
       <c r="R26" s="5"/>
       <c r="S26" s="5"/>
       <c r="T26" s="5"/>
-      <c r="U26" s="11"/>
-    </row>
-    <row r="27" spans="1:21">
+      <c r="U26" s="5"/>
+      <c r="V26" s="11"/>
+    </row>
+    <row r="27" spans="1:22">
       <c r="A27" s="5"/>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -1781,9 +1817,10 @@
       <c r="R27" s="5"/>
       <c r="S27" s="5"/>
       <c r="T27" s="5"/>
-      <c r="U27" s="11"/>
-    </row>
-    <row r="28" spans="1:21">
+      <c r="U27" s="5"/>
+      <c r="V27" s="11"/>
+    </row>
+    <row r="28" spans="1:22">
       <c r="A28" s="5"/>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -1804,9 +1841,10 @@
       <c r="R28" s="5"/>
       <c r="S28" s="5"/>
       <c r="T28" s="5"/>
-      <c r="U28" s="11"/>
-    </row>
-    <row r="29" spans="1:21">
+      <c r="U28" s="5"/>
+      <c r="V28" s="11"/>
+    </row>
+    <row r="29" spans="1:22">
       <c r="A29" s="5"/>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -1827,9 +1865,10 @@
       <c r="R29" s="5"/>
       <c r="S29" s="5"/>
       <c r="T29" s="5"/>
-      <c r="U29" s="11"/>
-    </row>
-    <row r="30" spans="1:21">
+      <c r="U29" s="5"/>
+      <c r="V29" s="11"/>
+    </row>
+    <row r="30" spans="1:22">
       <c r="A30" s="5"/>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
@@ -1850,9 +1889,10 @@
       <c r="R30" s="5"/>
       <c r="S30" s="5"/>
       <c r="T30" s="5"/>
-      <c r="U30" s="11"/>
-    </row>
-    <row r="31" spans="1:21">
+      <c r="U30" s="5"/>
+      <c r="V30" s="11"/>
+    </row>
+    <row r="31" spans="1:22">
       <c r="A31" s="5"/>
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>
@@ -1873,9 +1913,10 @@
       <c r="R31" s="5"/>
       <c r="S31" s="5"/>
       <c r="T31" s="5"/>
-      <c r="U31" s="11"/>
-    </row>
-    <row r="32" spans="1:21">
+      <c r="U31" s="5"/>
+      <c r="V31" s="11"/>
+    </row>
+    <row r="32" spans="1:22">
       <c r="A32" s="5"/>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -1896,9 +1937,10 @@
       <c r="R32" s="5"/>
       <c r="S32" s="5"/>
       <c r="T32" s="5"/>
-      <c r="U32" s="11"/>
-    </row>
-    <row r="33" spans="1:21">
+      <c r="U32" s="5"/>
+      <c r="V32" s="11"/>
+    </row>
+    <row r="33" spans="1:22">
       <c r="A33" s="5"/>
       <c r="B33" s="5"/>
       <c r="C33" s="5"/>
@@ -1919,9 +1961,10 @@
       <c r="R33" s="5"/>
       <c r="S33" s="5"/>
       <c r="T33" s="5"/>
-      <c r="U33" s="11"/>
-    </row>
-    <row r="34" spans="1:21">
+      <c r="U33" s="5"/>
+      <c r="V33" s="11"/>
+    </row>
+    <row r="34" spans="1:22">
       <c r="A34" s="5"/>
       <c r="B34" s="5"/>
       <c r="C34" s="5"/>
@@ -1942,9 +1985,10 @@
       <c r="R34" s="5"/>
       <c r="S34" s="5"/>
       <c r="T34" s="5"/>
-      <c r="U34" s="11"/>
-    </row>
-    <row r="35" spans="1:21">
+      <c r="U34" s="5"/>
+      <c r="V34" s="11"/>
+    </row>
+    <row r="35" spans="1:22">
       <c r="A35" s="5"/>
       <c r="B35" s="5"/>
       <c r="C35" s="5"/>
@@ -1965,9 +2009,10 @@
       <c r="R35" s="5"/>
       <c r="S35" s="5"/>
       <c r="T35" s="5"/>
-      <c r="U35" s="11"/>
-    </row>
-    <row r="36" spans="1:21">
+      <c r="U35" s="5"/>
+      <c r="V35" s="11"/>
+    </row>
+    <row r="36" spans="1:22">
       <c r="A36" s="5"/>
       <c r="B36" s="5"/>
       <c r="C36" s="5"/>
@@ -1988,9 +2033,10 @@
       <c r="R36" s="5"/>
       <c r="S36" s="5"/>
       <c r="T36" s="5"/>
-      <c r="U36" s="11"/>
-    </row>
-    <row r="37" spans="1:21">
+      <c r="U36" s="5"/>
+      <c r="V36" s="11"/>
+    </row>
+    <row r="37" spans="1:22">
       <c r="A37" s="5"/>
       <c r="B37" s="5"/>
       <c r="C37" s="5"/>
@@ -2011,9 +2057,10 @@
       <c r="R37" s="5"/>
       <c r="S37" s="5"/>
       <c r="T37" s="5"/>
-      <c r="U37" s="11"/>
-    </row>
-    <row r="38" spans="1:21">
+      <c r="U37" s="5"/>
+      <c r="V37" s="11"/>
+    </row>
+    <row r="38" spans="1:22">
       <c r="A38" s="5"/>
       <c r="B38" s="5"/>
       <c r="C38" s="5"/>
@@ -2034,9 +2081,10 @@
       <c r="R38" s="5"/>
       <c r="S38" s="5"/>
       <c r="T38" s="5"/>
-      <c r="U38" s="11"/>
-    </row>
-    <row r="39" spans="1:21">
+      <c r="U38" s="5"/>
+      <c r="V38" s="11"/>
+    </row>
+    <row r="39" spans="1:22">
       <c r="A39" s="5"/>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
@@ -2057,9 +2105,10 @@
       <c r="R39" s="5"/>
       <c r="S39" s="5"/>
       <c r="T39" s="5"/>
-      <c r="U39" s="11"/>
-    </row>
-    <row r="40" spans="1:21">
+      <c r="U39" s="5"/>
+      <c r="V39" s="11"/>
+    </row>
+    <row r="40" spans="1:22">
       <c r="A40" s="5"/>
       <c r="B40" s="5"/>
       <c r="C40" s="5"/>
@@ -2080,9 +2129,10 @@
       <c r="R40" s="5"/>
       <c r="S40" s="5"/>
       <c r="T40" s="5"/>
-      <c r="U40" s="11"/>
-    </row>
-    <row r="41" spans="1:21">
+      <c r="U40" s="5"/>
+      <c r="V40" s="11"/>
+    </row>
+    <row r="41" spans="1:22">
       <c r="A41" s="5"/>
       <c r="B41" s="5"/>
       <c r="C41" s="5"/>
@@ -2103,9 +2153,10 @@
       <c r="R41" s="5"/>
       <c r="S41" s="5"/>
       <c r="T41" s="5"/>
-      <c r="U41" s="11"/>
-    </row>
-    <row r="42" spans="1:21">
+      <c r="U41" s="5"/>
+      <c r="V41" s="11"/>
+    </row>
+    <row r="42" spans="1:22">
       <c r="A42" s="5"/>
       <c r="B42" s="5"/>
       <c r="C42" s="5"/>
@@ -2126,9 +2177,10 @@
       <c r="R42" s="5"/>
       <c r="S42" s="5"/>
       <c r="T42" s="5"/>
-      <c r="U42" s="11"/>
-    </row>
-    <row r="43" spans="1:21">
+      <c r="U42" s="5"/>
+      <c r="V42" s="11"/>
+    </row>
+    <row r="43" spans="1:22">
       <c r="A43" s="5"/>
       <c r="B43" s="5"/>
       <c r="C43" s="5"/>
@@ -2149,9 +2201,10 @@
       <c r="R43" s="5"/>
       <c r="S43" s="5"/>
       <c r="T43" s="5"/>
-      <c r="U43" s="11"/>
-    </row>
-    <row r="44" spans="1:21">
+      <c r="U43" s="5"/>
+      <c r="V43" s="11"/>
+    </row>
+    <row r="44" spans="1:22">
       <c r="A44" s="5"/>
       <c r="B44" s="5"/>
       <c r="C44" s="5"/>
@@ -2172,9 +2225,10 @@
       <c r="R44" s="5"/>
       <c r="S44" s="5"/>
       <c r="T44" s="5"/>
-      <c r="U44" s="11"/>
-    </row>
-    <row r="45" spans="1:21">
+      <c r="U44" s="5"/>
+      <c r="V44" s="11"/>
+    </row>
+    <row r="45" spans="1:22">
       <c r="A45" s="5"/>
       <c r="B45" s="5"/>
       <c r="C45" s="5"/>
@@ -2195,9 +2249,10 @@
       <c r="R45" s="5"/>
       <c r="S45" s="5"/>
       <c r="T45" s="5"/>
-      <c r="U45" s="11"/>
-    </row>
-    <row r="46" spans="1:21">
+      <c r="U45" s="5"/>
+      <c r="V45" s="11"/>
+    </row>
+    <row r="46" spans="1:22">
       <c r="A46" s="5"/>
       <c r="B46" s="5"/>
       <c r="C46" s="5"/>
@@ -2218,9 +2273,10 @@
       <c r="R46" s="5"/>
       <c r="S46" s="10"/>
       <c r="T46" s="5"/>
-      <c r="U46" s="11"/>
-    </row>
-    <row r="47" spans="1:21">
+      <c r="U46" s="5"/>
+      <c r="V46" s="11"/>
+    </row>
+    <row r="47" spans="1:22">
       <c r="A47" s="5"/>
       <c r="B47" s="5"/>
       <c r="C47" s="5"/>
@@ -2241,9 +2297,10 @@
       <c r="R47" s="5"/>
       <c r="S47" s="5"/>
       <c r="T47" s="5"/>
-      <c r="U47" s="11"/>
-    </row>
-    <row r="48" spans="1:21">
+      <c r="U47" s="5"/>
+      <c r="V47" s="11"/>
+    </row>
+    <row r="48" spans="1:22">
       <c r="A48" s="5"/>
       <c r="B48" s="5"/>
       <c r="C48" s="5"/>
@@ -2264,9 +2321,10 @@
       <c r="R48" s="5"/>
       <c r="S48" s="5"/>
       <c r="T48" s="5"/>
-      <c r="U48" s="11"/>
-    </row>
-    <row r="49" spans="1:21">
+      <c r="U48" s="5"/>
+      <c r="V48" s="11"/>
+    </row>
+    <row r="49" spans="1:22">
       <c r="A49" s="5"/>
       <c r="B49" s="5"/>
       <c r="C49" s="5"/>
@@ -2287,9 +2345,10 @@
       <c r="R49" s="5"/>
       <c r="S49" s="5"/>
       <c r="T49" s="5"/>
-      <c r="U49" s="11"/>
-    </row>
-    <row r="50" spans="1:21">
+      <c r="U49" s="5"/>
+      <c r="V49" s="11"/>
+    </row>
+    <row r="50" spans="1:22">
       <c r="A50" s="5"/>
       <c r="B50" s="5"/>
       <c r="C50" s="5"/>
@@ -2310,9 +2369,10 @@
       <c r="R50" s="5"/>
       <c r="S50" s="5"/>
       <c r="T50" s="5"/>
-      <c r="U50" s="11"/>
-    </row>
-    <row r="51" spans="1:21">
+      <c r="U50" s="5"/>
+      <c r="V50" s="11"/>
+    </row>
+    <row r="51" spans="1:22">
       <c r="A51" s="5"/>
       <c r="B51" s="5"/>
       <c r="C51" s="5"/>
@@ -2333,9 +2393,10 @@
       <c r="R51" s="5"/>
       <c r="S51" s="5"/>
       <c r="T51" s="5"/>
-      <c r="U51" s="11"/>
-    </row>
-    <row r="52" spans="1:21">
+      <c r="U51" s="5"/>
+      <c r="V51" s="11"/>
+    </row>
+    <row r="52" spans="1:22">
       <c r="A52" s="5"/>
       <c r="B52" s="5"/>
       <c r="C52" s="5"/>
@@ -2356,9 +2417,10 @@
       <c r="R52" s="5"/>
       <c r="S52" s="10"/>
       <c r="T52" s="5"/>
-      <c r="U52" s="11"/>
-    </row>
-    <row r="53" spans="1:21">
+      <c r="U52" s="5"/>
+      <c r="V52" s="11"/>
+    </row>
+    <row r="53" spans="1:22">
       <c r="A53" s="5"/>
       <c r="B53" s="5"/>
       <c r="C53" s="5"/>
@@ -2379,9 +2441,10 @@
       <c r="R53" s="5"/>
       <c r="S53" s="5"/>
       <c r="T53" s="5"/>
-      <c r="U53" s="11"/>
-    </row>
-    <row r="54" spans="1:21">
+      <c r="U53" s="5"/>
+      <c r="V53" s="11"/>
+    </row>
+    <row r="54" spans="1:22">
       <c r="A54" s="5"/>
       <c r="B54" s="5"/>
       <c r="C54" s="5"/>
@@ -2402,9 +2465,10 @@
       <c r="R54" s="5"/>
       <c r="S54" s="5"/>
       <c r="T54" s="5"/>
-      <c r="U54" s="11"/>
-    </row>
-    <row r="55" spans="1:21">
+      <c r="U54" s="5"/>
+      <c r="V54" s="11"/>
+    </row>
+    <row r="55" spans="1:22">
       <c r="A55" s="5"/>
       <c r="B55" s="5"/>
       <c r="C55" s="5"/>
@@ -2425,9 +2489,10 @@
       <c r="R55" s="5"/>
       <c r="S55" s="10"/>
       <c r="T55" s="5"/>
-      <c r="U55" s="11"/>
-    </row>
-    <row r="56" spans="1:21">
+      <c r="U55" s="5"/>
+      <c r="V55" s="11"/>
+    </row>
+    <row r="56" spans="1:22">
       <c r="A56" s="5"/>
       <c r="B56" s="5"/>
       <c r="C56" s="5"/>
@@ -2448,9 +2513,10 @@
       <c r="R56" s="5"/>
       <c r="S56" s="5"/>
       <c r="T56" s="5"/>
-      <c r="U56" s="11"/>
-    </row>
-    <row r="57" spans="1:21">
+      <c r="U56" s="5"/>
+      <c r="V56" s="11"/>
+    </row>
+    <row r="57" spans="1:22">
       <c r="A57" s="5"/>
       <c r="B57" s="5"/>
       <c r="C57" s="5"/>
@@ -2471,9 +2537,10 @@
       <c r="R57" s="5"/>
       <c r="S57" s="5"/>
       <c r="T57" s="5"/>
-      <c r="U57" s="11"/>
-    </row>
-    <row r="58" spans="1:21">
+      <c r="U57" s="5"/>
+      <c r="V57" s="11"/>
+    </row>
+    <row r="58" spans="1:22">
       <c r="A58" s="5"/>
       <c r="B58" s="5"/>
       <c r="C58" s="5"/>
@@ -2494,9 +2561,10 @@
       <c r="R58" s="5"/>
       <c r="S58" s="5"/>
       <c r="T58" s="5"/>
-      <c r="U58" s="11"/>
-    </row>
-    <row r="59" spans="1:21">
+      <c r="U58" s="5"/>
+      <c r="V58" s="11"/>
+    </row>
+    <row r="59" spans="1:22">
       <c r="A59" s="5"/>
       <c r="B59" s="5"/>
       <c r="C59" s="5"/>
@@ -2517,9 +2585,10 @@
       <c r="R59" s="5"/>
       <c r="S59" s="5"/>
       <c r="T59" s="5"/>
-      <c r="U59" s="11"/>
-    </row>
-    <row r="60" spans="1:21">
+      <c r="U59" s="5"/>
+      <c r="V59" s="11"/>
+    </row>
+    <row r="60" spans="1:22">
       <c r="A60" s="5"/>
       <c r="B60" s="5"/>
       <c r="C60" s="5"/>
@@ -2540,9 +2609,10 @@
       <c r="R60" s="5"/>
       <c r="S60" s="5"/>
       <c r="T60" s="5"/>
-      <c r="U60" s="11"/>
-    </row>
-    <row r="61" spans="1:21">
+      <c r="U60" s="5"/>
+      <c r="V60" s="11"/>
+    </row>
+    <row r="61" spans="1:22">
       <c r="A61" s="5"/>
       <c r="B61" s="5"/>
       <c r="C61" s="5"/>
@@ -2563,9 +2633,10 @@
       <c r="R61" s="5"/>
       <c r="S61" s="5"/>
       <c r="T61" s="5"/>
-      <c r="U61" s="11"/>
-    </row>
-    <row r="62" spans="1:21">
+      <c r="U61" s="5"/>
+      <c r="V61" s="11"/>
+    </row>
+    <row r="62" spans="1:22">
       <c r="A62" s="5"/>
       <c r="B62" s="5"/>
       <c r="C62" s="5"/>
@@ -2586,9 +2657,10 @@
       <c r="R62" s="5"/>
       <c r="S62" s="5"/>
       <c r="T62" s="5"/>
-      <c r="U62" s="11"/>
-    </row>
-    <row r="63" spans="1:21">
+      <c r="U62" s="5"/>
+      <c r="V62" s="11"/>
+    </row>
+    <row r="63" spans="1:22">
       <c r="A63" s="5"/>
       <c r="B63" s="5"/>
       <c r="C63" s="5"/>
@@ -2609,9 +2681,10 @@
       <c r="R63" s="5"/>
       <c r="S63" s="5"/>
       <c r="T63" s="5"/>
-      <c r="U63" s="11"/>
-    </row>
-    <row r="64" spans="1:21">
+      <c r="U63" s="5"/>
+      <c r="V63" s="11"/>
+    </row>
+    <row r="64" spans="1:22">
       <c r="A64" s="5"/>
       <c r="B64" s="5"/>
       <c r="C64" s="5"/>
@@ -2632,9 +2705,10 @@
       <c r="R64" s="5"/>
       <c r="S64" s="5"/>
       <c r="T64" s="5"/>
-      <c r="U64" s="11"/>
-    </row>
-    <row r="65" spans="1:21">
+      <c r="U64" s="5"/>
+      <c r="V64" s="11"/>
+    </row>
+    <row r="65" spans="1:22">
       <c r="A65" s="5"/>
       <c r="B65" s="5"/>
       <c r="C65" s="5"/>
@@ -2655,9 +2729,10 @@
       <c r="R65" s="5"/>
       <c r="S65" s="5"/>
       <c r="T65" s="5"/>
-      <c r="U65" s="11"/>
-    </row>
-    <row r="66" spans="1:21">
+      <c r="U65" s="5"/>
+      <c r="V65" s="11"/>
+    </row>
+    <row r="66" spans="1:22">
       <c r="A66" s="5"/>
       <c r="B66" s="5"/>
       <c r="C66" s="5"/>
@@ -2678,9 +2753,10 @@
       <c r="R66" s="5"/>
       <c r="S66" s="5"/>
       <c r="T66" s="5"/>
-      <c r="U66" s="11"/>
-    </row>
-    <row r="67" spans="1:21">
+      <c r="U66" s="5"/>
+      <c r="V66" s="11"/>
+    </row>
+    <row r="67" spans="1:22">
       <c r="A67" s="5"/>
       <c r="B67" s="5"/>
       <c r="C67" s="5"/>
@@ -2701,9 +2777,10 @@
       <c r="R67" s="5"/>
       <c r="S67" s="5"/>
       <c r="T67" s="5"/>
-      <c r="U67" s="11"/>
-    </row>
-    <row r="68" spans="1:21">
+      <c r="U67" s="5"/>
+      <c r="V67" s="11"/>
+    </row>
+    <row r="68" spans="1:22">
       <c r="A68" s="5"/>
       <c r="B68" s="5"/>
       <c r="C68" s="5"/>
@@ -2724,9 +2801,10 @@
       <c r="R68" s="5"/>
       <c r="S68" s="5"/>
       <c r="T68" s="5"/>
-      <c r="U68" s="11"/>
-    </row>
-    <row r="69" spans="1:21">
+      <c r="U68" s="5"/>
+      <c r="V68" s="11"/>
+    </row>
+    <row r="69" spans="1:22">
       <c r="A69" s="5"/>
       <c r="B69" s="5"/>
       <c r="C69" s="5"/>
@@ -2747,9 +2825,10 @@
       <c r="R69" s="5"/>
       <c r="S69" s="5"/>
       <c r="T69" s="5"/>
-      <c r="U69" s="11"/>
-    </row>
-    <row r="70" spans="1:21">
+      <c r="U69" s="5"/>
+      <c r="V69" s="11"/>
+    </row>
+    <row r="70" spans="1:22">
       <c r="A70" s="5"/>
       <c r="B70" s="5"/>
       <c r="C70" s="5"/>
@@ -2770,9 +2849,10 @@
       <c r="R70" s="5"/>
       <c r="S70" s="5"/>
       <c r="T70" s="5"/>
-      <c r="U70" s="11"/>
-    </row>
-    <row r="71" spans="1:21">
+      <c r="U70" s="5"/>
+      <c r="V70" s="11"/>
+    </row>
+    <row r="71" spans="1:22">
       <c r="A71" s="5"/>
       <c r="B71" s="5"/>
       <c r="C71" s="5"/>
@@ -2793,9 +2873,10 @@
       <c r="R71" s="5"/>
       <c r="S71" s="5"/>
       <c r="T71" s="5"/>
-      <c r="U71" s="11"/>
-    </row>
-    <row r="72" spans="1:21">
+      <c r="U71" s="5"/>
+      <c r="V71" s="11"/>
+    </row>
+    <row r="72" spans="1:22">
       <c r="A72" s="5"/>
       <c r="B72" s="5"/>
       <c r="C72" s="5"/>
@@ -2816,9 +2897,10 @@
       <c r="R72" s="5"/>
       <c r="S72" s="5"/>
       <c r="T72" s="5"/>
-      <c r="U72" s="11"/>
-    </row>
-    <row r="73" spans="1:21">
+      <c r="U72" s="5"/>
+      <c r="V72" s="11"/>
+    </row>
+    <row r="73" spans="1:22">
       <c r="A73" s="5"/>
       <c r="B73" s="5"/>
       <c r="C73" s="5"/>
@@ -2839,9 +2921,10 @@
       <c r="R73" s="5"/>
       <c r="S73" s="5"/>
       <c r="T73" s="5"/>
-      <c r="U73" s="11"/>
-    </row>
-    <row r="74" spans="1:21">
+      <c r="U73" s="5"/>
+      <c r="V73" s="11"/>
+    </row>
+    <row r="74" spans="1:22">
       <c r="A74" s="5"/>
       <c r="B74" s="5"/>
       <c r="C74" s="5"/>
@@ -2862,9 +2945,10 @@
       <c r="R74" s="5"/>
       <c r="S74" s="5"/>
       <c r="T74" s="5"/>
-      <c r="U74" s="11"/>
-    </row>
-    <row r="75" spans="1:21">
+      <c r="U74" s="5"/>
+      <c r="V74" s="11"/>
+    </row>
+    <row r="75" spans="1:22">
       <c r="A75" s="5"/>
       <c r="B75" s="5"/>
       <c r="C75" s="5"/>
@@ -2885,9 +2969,10 @@
       <c r="R75" s="5"/>
       <c r="S75" s="5"/>
       <c r="T75" s="5"/>
-      <c r="U75" s="11"/>
-    </row>
-    <row r="76" spans="1:21">
+      <c r="U75" s="5"/>
+      <c r="V75" s="11"/>
+    </row>
+    <row r="76" spans="1:22">
       <c r="A76" s="5"/>
       <c r="B76" s="5"/>
       <c r="C76" s="5"/>
@@ -2908,9 +2993,10 @@
       <c r="R76" s="5"/>
       <c r="S76" s="5"/>
       <c r="T76" s="5"/>
-      <c r="U76" s="11"/>
-    </row>
-    <row r="77" spans="1:21">
+      <c r="U76" s="5"/>
+      <c r="V76" s="11"/>
+    </row>
+    <row r="77" spans="1:22">
       <c r="A77" s="5"/>
       <c r="B77" s="5"/>
       <c r="C77" s="5"/>
@@ -2931,9 +3017,10 @@
       <c r="R77" s="5"/>
       <c r="S77" s="5"/>
       <c r="T77" s="5"/>
-      <c r="U77" s="11"/>
-    </row>
-    <row r="78" spans="1:21">
+      <c r="U77" s="5"/>
+      <c r="V77" s="11"/>
+    </row>
+    <row r="78" spans="1:22">
       <c r="A78" s="5"/>
       <c r="B78" s="5"/>
       <c r="C78" s="5"/>
@@ -2954,9 +3041,10 @@
       <c r="R78" s="5"/>
       <c r="S78" s="5"/>
       <c r="T78" s="5"/>
-      <c r="U78" s="11"/>
-    </row>
-    <row r="79" spans="1:21">
+      <c r="U78" s="5"/>
+      <c r="V78" s="11"/>
+    </row>
+    <row r="79" spans="1:22">
       <c r="A79" s="5"/>
       <c r="B79" s="5"/>
       <c r="C79" s="5"/>
@@ -2977,9 +3065,10 @@
       <c r="R79" s="5"/>
       <c r="S79" s="5"/>
       <c r="T79" s="5"/>
-      <c r="U79" s="11"/>
-    </row>
-    <row r="80" spans="1:21">
+      <c r="U79" s="5"/>
+      <c r="V79" s="11"/>
+    </row>
+    <row r="80" spans="1:22">
       <c r="A80" s="5"/>
       <c r="B80" s="5"/>
       <c r="C80" s="5"/>
@@ -3000,9 +3089,10 @@
       <c r="R80" s="5"/>
       <c r="S80" s="5"/>
       <c r="T80" s="5"/>
-      <c r="U80" s="11"/>
-    </row>
-    <row r="81" spans="1:21">
+      <c r="U80" s="5"/>
+      <c r="V80" s="11"/>
+    </row>
+    <row r="81" spans="1:22">
       <c r="A81" s="5"/>
       <c r="B81" s="5"/>
       <c r="C81" s="5"/>
@@ -3023,9 +3113,10 @@
       <c r="R81" s="5"/>
       <c r="S81" s="5"/>
       <c r="T81" s="5"/>
-      <c r="U81" s="11"/>
-    </row>
-    <row r="82" spans="1:21">
+      <c r="U81" s="5"/>
+      <c r="V81" s="11"/>
+    </row>
+    <row r="82" spans="1:22">
       <c r="A82" s="5"/>
       <c r="B82" s="5"/>
       <c r="C82" s="5"/>
@@ -3046,9 +3137,10 @@
       <c r="R82" s="5"/>
       <c r="S82" s="5"/>
       <c r="T82" s="5"/>
-      <c r="U82" s="11"/>
-    </row>
-    <row r="83" spans="1:21">
+      <c r="U82" s="5"/>
+      <c r="V82" s="11"/>
+    </row>
+    <row r="83" spans="1:22">
       <c r="A83" s="5"/>
       <c r="B83" s="5"/>
       <c r="C83" s="5"/>
@@ -3069,9 +3161,10 @@
       <c r="R83" s="5"/>
       <c r="S83" s="5"/>
       <c r="T83" s="5"/>
-      <c r="U83" s="11"/>
-    </row>
-    <row r="84" spans="1:21">
+      <c r="U83" s="5"/>
+      <c r="V83" s="11"/>
+    </row>
+    <row r="84" spans="1:22">
       <c r="A84" s="5"/>
       <c r="B84" s="5"/>
       <c r="C84" s="5"/>
@@ -3092,9 +3185,10 @@
       <c r="R84" s="5"/>
       <c r="S84" s="5"/>
       <c r="T84" s="5"/>
-      <c r="U84" s="11"/>
-    </row>
-    <row r="85" spans="1:21">
+      <c r="U84" s="5"/>
+      <c r="V84" s="11"/>
+    </row>
+    <row r="85" spans="1:22">
       <c r="A85" s="5"/>
       <c r="B85" s="5"/>
       <c r="C85" s="5"/>
@@ -3115,9 +3209,10 @@
       <c r="R85" s="5"/>
       <c r="S85" s="5"/>
       <c r="T85" s="5"/>
-      <c r="U85" s="11"/>
-    </row>
-    <row r="86" spans="1:21">
+      <c r="U85" s="5"/>
+      <c r="V85" s="11"/>
+    </row>
+    <row r="86" spans="1:22">
       <c r="A86" s="5"/>
       <c r="B86" s="5"/>
       <c r="C86" s="5"/>
@@ -3138,9 +3233,10 @@
       <c r="R86" s="5"/>
       <c r="S86" s="5"/>
       <c r="T86" s="5"/>
-      <c r="U86" s="11"/>
-    </row>
-    <row r="87" spans="1:21">
+      <c r="U86" s="5"/>
+      <c r="V86" s="11"/>
+    </row>
+    <row r="87" spans="1:22">
       <c r="A87" s="5"/>
       <c r="B87" s="5"/>
       <c r="C87" s="5"/>
@@ -3161,9 +3257,10 @@
       <c r="R87" s="5"/>
       <c r="S87" s="5"/>
       <c r="T87" s="5"/>
-      <c r="U87" s="11"/>
-    </row>
-    <row r="88" spans="1:21">
+      <c r="U87" s="5"/>
+      <c r="V87" s="11"/>
+    </row>
+    <row r="88" spans="1:22">
       <c r="A88" s="5"/>
       <c r="B88" s="5"/>
       <c r="C88" s="5"/>
@@ -3184,9 +3281,10 @@
       <c r="R88" s="5"/>
       <c r="S88" s="5"/>
       <c r="T88" s="5"/>
-      <c r="U88" s="11"/>
-    </row>
-    <row r="89" spans="1:21">
+      <c r="U88" s="5"/>
+      <c r="V88" s="11"/>
+    </row>
+    <row r="89" spans="1:22">
       <c r="A89" s="5"/>
       <c r="B89" s="5"/>
       <c r="C89" s="5"/>
@@ -3207,9 +3305,10 @@
       <c r="R89" s="5"/>
       <c r="S89" s="5"/>
       <c r="T89" s="5"/>
-      <c r="U89" s="11"/>
-    </row>
-    <row r="90" spans="1:21">
+      <c r="U89" s="5"/>
+      <c r="V89" s="11"/>
+    </row>
+    <row r="90" spans="1:22">
       <c r="A90" s="5"/>
       <c r="B90" s="5"/>
       <c r="C90" s="5"/>
@@ -3230,9 +3329,10 @@
       <c r="R90" s="5"/>
       <c r="S90" s="5"/>
       <c r="T90" s="5"/>
-      <c r="U90" s="11"/>
-    </row>
-    <row r="91" spans="1:21" ht="14.25">
+      <c r="U90" s="5"/>
+      <c r="V90" s="11"/>
+    </row>
+    <row r="91" spans="1:22" ht="14.25">
       <c r="A91" s="5"/>
       <c r="B91" s="5"/>
       <c r="C91" s="5"/>
@@ -3253,9 +3353,10 @@
       <c r="R91" s="5"/>
       <c r="S91" s="5"/>
       <c r="T91" s="5"/>
-      <c r="U91" s="11"/>
-    </row>
-    <row r="92" spans="1:21">
+      <c r="U91" s="5"/>
+      <c r="V91" s="11"/>
+    </row>
+    <row r="92" spans="1:22">
       <c r="A92" s="5"/>
       <c r="B92" s="5"/>
       <c r="C92" s="5"/>
@@ -3276,9 +3377,10 @@
       <c r="R92" s="5"/>
       <c r="S92" s="5"/>
       <c r="T92" s="5"/>
-      <c r="U92" s="11"/>
-    </row>
-    <row r="93" spans="1:21">
+      <c r="U92" s="5"/>
+      <c r="V92" s="11"/>
+    </row>
+    <row r="93" spans="1:22">
       <c r="A93" s="5"/>
       <c r="B93" s="5"/>
       <c r="C93" s="5"/>
@@ -3299,9 +3401,10 @@
       <c r="R93" s="5"/>
       <c r="S93" s="5"/>
       <c r="T93" s="5"/>
-      <c r="U93" s="11"/>
-    </row>
-    <row r="94" spans="1:21">
+      <c r="U93" s="5"/>
+      <c r="V93" s="11"/>
+    </row>
+    <row r="94" spans="1:22">
       <c r="A94" s="5"/>
       <c r="B94" s="5"/>
       <c r="C94" s="5"/>
@@ -3322,9 +3425,10 @@
       <c r="R94" s="5"/>
       <c r="S94" s="5"/>
       <c r="T94" s="5"/>
-      <c r="U94" s="11"/>
-    </row>
-    <row r="95" spans="1:21">
+      <c r="U94" s="5"/>
+      <c r="V94" s="11"/>
+    </row>
+    <row r="95" spans="1:22">
       <c r="A95" s="5"/>
       <c r="B95" s="5"/>
       <c r="C95" s="5"/>
@@ -3345,9 +3449,10 @@
       <c r="R95" s="5"/>
       <c r="S95" s="5"/>
       <c r="T95" s="5"/>
-      <c r="U95" s="11"/>
-    </row>
-    <row r="96" spans="1:21">
+      <c r="U95" s="5"/>
+      <c r="V95" s="11"/>
+    </row>
+    <row r="96" spans="1:22">
       <c r="A96" s="5"/>
       <c r="B96" s="5"/>
       <c r="C96" s="5"/>
@@ -3368,9 +3473,10 @@
       <c r="R96" s="5"/>
       <c r="S96" s="5"/>
       <c r="T96" s="5"/>
-      <c r="U96" s="11"/>
-    </row>
-    <row r="97" spans="1:21">
+      <c r="U96" s="5"/>
+      <c r="V96" s="11"/>
+    </row>
+    <row r="97" spans="1:22">
       <c r="A97" s="5"/>
       <c r="B97" s="5"/>
       <c r="C97" s="5"/>
@@ -3391,9 +3497,10 @@
       <c r="R97" s="5"/>
       <c r="S97" s="5"/>
       <c r="T97" s="5"/>
-      <c r="U97" s="11"/>
-    </row>
-    <row r="98" spans="1:21" ht="14.25">
+      <c r="U97" s="5"/>
+      <c r="V97" s="11"/>
+    </row>
+    <row r="98" spans="1:22" ht="14.25">
       <c r="A98" s="5"/>
       <c r="B98" s="5"/>
       <c r="C98" s="5"/>
@@ -3414,9 +3521,10 @@
       <c r="R98" s="5"/>
       <c r="S98" s="5"/>
       <c r="T98" s="5"/>
-      <c r="U98" s="11"/>
-    </row>
-    <row r="99" spans="1:21">
+      <c r="U98" s="5"/>
+      <c r="V98" s="11"/>
+    </row>
+    <row r="99" spans="1:22">
       <c r="A99" s="5"/>
       <c r="B99" s="5"/>
       <c r="C99" s="5"/>
@@ -3437,9 +3545,10 @@
       <c r="R99" s="5"/>
       <c r="S99" s="5"/>
       <c r="T99" s="5"/>
-      <c r="U99" s="11"/>
-    </row>
-    <row r="100" spans="1:21">
+      <c r="U99" s="5"/>
+      <c r="V99" s="11"/>
+    </row>
+    <row r="100" spans="1:22">
       <c r="A100" s="5"/>
       <c r="B100" s="5"/>
       <c r="C100" s="5"/>
@@ -3460,9 +3569,10 @@
       <c r="R100" s="5"/>
       <c r="S100" s="5"/>
       <c r="T100" s="5"/>
-      <c r="U100" s="11"/>
-    </row>
-    <row r="101" spans="1:21">
+      <c r="U100" s="5"/>
+      <c r="V100" s="11"/>
+    </row>
+    <row r="101" spans="1:22">
       <c r="A101" s="5"/>
       <c r="B101" s="5"/>
       <c r="C101" s="5"/>
@@ -3483,9 +3593,10 @@
       <c r="R101" s="5"/>
       <c r="S101" s="5"/>
       <c r="T101" s="5"/>
-      <c r="U101" s="11"/>
-    </row>
-    <row r="102" spans="1:21">
+      <c r="U101" s="5"/>
+      <c r="V101" s="11"/>
+    </row>
+    <row r="102" spans="1:22">
       <c r="A102" s="5"/>
       <c r="B102" s="5"/>
       <c r="C102" s="5"/>
@@ -3506,9 +3617,10 @@
       <c r="R102" s="5"/>
       <c r="S102" s="5"/>
       <c r="T102" s="5"/>
-      <c r="U102" s="11"/>
-    </row>
-    <row r="103" spans="1:21">
+      <c r="U102" s="5"/>
+      <c r="V102" s="11"/>
+    </row>
+    <row r="103" spans="1:22">
       <c r="A103" s="5"/>
       <c r="B103" s="5"/>
       <c r="C103" s="5"/>
@@ -3529,9 +3641,10 @@
       <c r="R103" s="5"/>
       <c r="S103" s="5"/>
       <c r="T103" s="5"/>
-      <c r="U103" s="11"/>
-    </row>
-    <row r="104" spans="1:21">
+      <c r="U103" s="5"/>
+      <c r="V103" s="11"/>
+    </row>
+    <row r="104" spans="1:22">
       <c r="A104" s="5"/>
       <c r="B104" s="5"/>
       <c r="C104" s="5"/>
@@ -3552,9 +3665,10 @@
       <c r="R104" s="5"/>
       <c r="S104" s="5"/>
       <c r="T104" s="5"/>
-      <c r="U104" s="11"/>
-    </row>
-    <row r="105" spans="1:21" ht="14.25">
+      <c r="U104" s="5"/>
+      <c r="V104" s="11"/>
+    </row>
+    <row r="105" spans="1:22" ht="14.25">
       <c r="A105" s="5"/>
       <c r="B105" s="5"/>
       <c r="C105" s="5"/>
@@ -3575,9 +3689,10 @@
       <c r="R105" s="5"/>
       <c r="S105" s="5"/>
       <c r="T105" s="5"/>
-      <c r="U105" s="11"/>
-    </row>
-    <row r="106" spans="1:21">
+      <c r="U105" s="5"/>
+      <c r="V105" s="11"/>
+    </row>
+    <row r="106" spans="1:22">
       <c r="A106" s="5"/>
       <c r="B106" s="5"/>
       <c r="C106" s="5"/>
@@ -3598,9 +3713,10 @@
       <c r="R106" s="5"/>
       <c r="S106" s="5"/>
       <c r="T106" s="5"/>
-      <c r="U106" s="11"/>
-    </row>
-    <row r="107" spans="1:21">
+      <c r="U106" s="5"/>
+      <c r="V106" s="11"/>
+    </row>
+    <row r="107" spans="1:22">
       <c r="A107" s="5"/>
       <c r="B107" s="5"/>
       <c r="C107" s="5"/>
@@ -3621,9 +3737,10 @@
       <c r="R107" s="5"/>
       <c r="S107" s="5"/>
       <c r="T107" s="5"/>
-      <c r="U107" s="11"/>
-    </row>
-    <row r="108" spans="1:21">
+      <c r="U107" s="5"/>
+      <c r="V107" s="11"/>
+    </row>
+    <row r="108" spans="1:22">
       <c r="A108" s="5"/>
       <c r="B108" s="5"/>
       <c r="C108" s="5"/>
@@ -3644,9 +3761,10 @@
       <c r="R108" s="5"/>
       <c r="S108" s="5"/>
       <c r="T108" s="5"/>
-      <c r="U108" s="11"/>
-    </row>
-    <row r="109" spans="1:21">
+      <c r="U108" s="5"/>
+      <c r="V108" s="11"/>
+    </row>
+    <row r="109" spans="1:22">
       <c r="A109" s="5"/>
       <c r="B109" s="5"/>
       <c r="C109" s="5"/>
@@ -3667,9 +3785,10 @@
       <c r="R109" s="5"/>
       <c r="S109" s="5"/>
       <c r="T109" s="5"/>
-      <c r="U109" s="11"/>
-    </row>
-    <row r="110" spans="1:21">
+      <c r="U109" s="5"/>
+      <c r="V109" s="11"/>
+    </row>
+    <row r="110" spans="1:22">
       <c r="A110" s="5"/>
       <c r="B110" s="5"/>
       <c r="C110" s="5"/>
@@ -3690,9 +3809,10 @@
       <c r="R110" s="5"/>
       <c r="S110" s="5"/>
       <c r="T110" s="5"/>
-      <c r="U110" s="11"/>
-    </row>
-    <row r="111" spans="1:21">
+      <c r="U110" s="5"/>
+      <c r="V110" s="11"/>
+    </row>
+    <row r="111" spans="1:22">
       <c r="A111" s="5"/>
       <c r="B111" s="5"/>
       <c r="C111" s="5"/>
@@ -3713,9 +3833,10 @@
       <c r="R111" s="5"/>
       <c r="S111" s="5"/>
       <c r="T111" s="5"/>
-      <c r="U111" s="11"/>
-    </row>
-    <row r="112" spans="1:21">
+      <c r="U111" s="5"/>
+      <c r="V111" s="11"/>
+    </row>
+    <row r="112" spans="1:22">
       <c r="A112" s="5"/>
       <c r="B112" s="5"/>
       <c r="C112" s="5"/>
@@ -3736,9 +3857,10 @@
       <c r="R112" s="5"/>
       <c r="S112" s="5"/>
       <c r="T112" s="5"/>
-      <c r="U112" s="11"/>
-    </row>
-    <row r="113" spans="1:21">
+      <c r="U112" s="5"/>
+      <c r="V112" s="11"/>
+    </row>
+    <row r="113" spans="1:22">
       <c r="A113" s="5"/>
       <c r="B113" s="5"/>
       <c r="C113" s="5"/>
@@ -3759,9 +3881,10 @@
       <c r="R113" s="5"/>
       <c r="S113" s="5"/>
       <c r="T113" s="5"/>
-      <c r="U113" s="11"/>
-    </row>
-    <row r="114" spans="1:21">
+      <c r="U113" s="5"/>
+      <c r="V113" s="11"/>
+    </row>
+    <row r="114" spans="1:22">
       <c r="A114" s="5"/>
       <c r="B114" s="5"/>
       <c r="C114" s="5"/>
@@ -3782,9 +3905,10 @@
       <c r="R114" s="5"/>
       <c r="S114" s="5"/>
       <c r="T114" s="5"/>
-      <c r="U114" s="11"/>
-    </row>
-    <row r="115" spans="1:21">
+      <c r="U114" s="5"/>
+      <c r="V114" s="11"/>
+    </row>
+    <row r="115" spans="1:22">
       <c r="A115" s="5"/>
       <c r="B115" s="5"/>
       <c r="C115" s="5"/>
@@ -3805,9 +3929,10 @@
       <c r="R115" s="5"/>
       <c r="S115" s="5"/>
       <c r="T115" s="5"/>
-      <c r="U115" s="11"/>
-    </row>
-    <row r="116" spans="1:21">
+      <c r="U115" s="5"/>
+      <c r="V115" s="11"/>
+    </row>
+    <row r="116" spans="1:22">
       <c r="A116" s="5"/>
       <c r="B116" s="5"/>
       <c r="C116" s="5"/>
@@ -3828,9 +3953,10 @@
       <c r="R116" s="5"/>
       <c r="S116" s="5"/>
       <c r="T116" s="5"/>
-      <c r="U116" s="11"/>
-    </row>
-    <row r="117" spans="1:21">
+      <c r="U116" s="5"/>
+      <c r="V116" s="11"/>
+    </row>
+    <row r="117" spans="1:22">
       <c r="A117" s="5"/>
       <c r="B117" s="5"/>
       <c r="C117" s="5"/>
@@ -3851,9 +3977,10 @@
       <c r="R117" s="5"/>
       <c r="S117" s="5"/>
       <c r="T117" s="5"/>
-      <c r="U117" s="11"/>
-    </row>
-    <row r="118" spans="1:21">
+      <c r="U117" s="5"/>
+      <c r="V117" s="11"/>
+    </row>
+    <row r="118" spans="1:22">
       <c r="A118" s="5"/>
       <c r="B118" s="5"/>
       <c r="C118" s="5"/>
@@ -3874,9 +4001,10 @@
       <c r="R118" s="5"/>
       <c r="S118" s="5"/>
       <c r="T118" s="5"/>
-      <c r="U118" s="11"/>
-    </row>
-    <row r="119" spans="1:21">
+      <c r="U118" s="5"/>
+      <c r="V118" s="11"/>
+    </row>
+    <row r="119" spans="1:22">
       <c r="A119" s="5"/>
       <c r="B119" s="5"/>
       <c r="C119" s="5"/>
@@ -3897,9 +4025,10 @@
       <c r="R119" s="5"/>
       <c r="S119" s="5"/>
       <c r="T119" s="5"/>
-      <c r="U119" s="11"/>
-    </row>
-    <row r="120" spans="1:21">
+      <c r="U119" s="5"/>
+      <c r="V119" s="11"/>
+    </row>
+    <row r="120" spans="1:22">
       <c r="A120" s="5"/>
       <c r="B120" s="5"/>
       <c r="C120" s="5"/>
@@ -3920,9 +4049,10 @@
       <c r="R120" s="5"/>
       <c r="S120" s="5"/>
       <c r="T120" s="5"/>
-      <c r="U120" s="11"/>
-    </row>
-    <row r="121" spans="1:21">
+      <c r="U120" s="5"/>
+      <c r="V120" s="11"/>
+    </row>
+    <row r="121" spans="1:22">
       <c r="A121" s="5"/>
       <c r="B121" s="5"/>
       <c r="C121" s="5"/>
@@ -3943,9 +4073,10 @@
       <c r="R121" s="5"/>
       <c r="S121" s="5"/>
       <c r="T121" s="5"/>
-      <c r="U121" s="11"/>
-    </row>
-    <row r="122" spans="1:21">
+      <c r="U121" s="5"/>
+      <c r="V121" s="11"/>
+    </row>
+    <row r="122" spans="1:22">
       <c r="A122" s="5"/>
       <c r="B122" s="5"/>
       <c r="C122" s="5"/>
@@ -3966,9 +4097,10 @@
       <c r="R122" s="5"/>
       <c r="S122" s="5"/>
       <c r="T122" s="5"/>
-      <c r="U122" s="11"/>
-    </row>
-    <row r="123" spans="1:21">
+      <c r="U122" s="5"/>
+      <c r="V122" s="11"/>
+    </row>
+    <row r="123" spans="1:22">
       <c r="A123" s="5"/>
       <c r="B123" s="5"/>
       <c r="C123" s="5"/>
@@ -3989,9 +4121,10 @@
       <c r="R123" s="5"/>
       <c r="S123" s="5"/>
       <c r="T123" s="5"/>
-      <c r="U123" s="11"/>
-    </row>
-    <row r="124" spans="1:21">
+      <c r="U123" s="5"/>
+      <c r="V123" s="11"/>
+    </row>
+    <row r="124" spans="1:22">
       <c r="A124" s="5"/>
       <c r="B124" s="5"/>
       <c r="C124" s="5"/>
@@ -4012,9 +4145,10 @@
       <c r="R124" s="5"/>
       <c r="S124" s="5"/>
       <c r="T124" s="5"/>
-      <c r="U124" s="11"/>
-    </row>
-    <row r="125" spans="1:21">
+      <c r="U124" s="5"/>
+      <c r="V124" s="11"/>
+    </row>
+    <row r="125" spans="1:22">
       <c r="A125" s="5"/>
       <c r="B125" s="5"/>
       <c r="C125" s="5"/>
@@ -4035,9 +4169,10 @@
       <c r="R125" s="5"/>
       <c r="S125" s="5"/>
       <c r="T125" s="5"/>
-      <c r="U125" s="11"/>
-    </row>
-    <row r="126" spans="1:21">
+      <c r="U125" s="5"/>
+      <c r="V125" s="11"/>
+    </row>
+    <row r="126" spans="1:22">
       <c r="A126" s="5"/>
       <c r="B126" s="5"/>
       <c r="C126" s="5"/>
@@ -4058,9 +4193,10 @@
       <c r="R126" s="5"/>
       <c r="S126" s="5"/>
       <c r="T126" s="5"/>
-      <c r="U126" s="11"/>
-    </row>
-    <row r="127" spans="1:21">
+      <c r="U126" s="5"/>
+      <c r="V126" s="11"/>
+    </row>
+    <row r="127" spans="1:22">
       <c r="A127" s="5"/>
       <c r="B127" s="5"/>
       <c r="C127" s="5"/>
@@ -4081,9 +4217,10 @@
       <c r="R127" s="5"/>
       <c r="S127" s="5"/>
       <c r="T127" s="5"/>
-      <c r="U127" s="11"/>
-    </row>
-    <row r="128" spans="1:21">
+      <c r="U127" s="5"/>
+      <c r="V127" s="11"/>
+    </row>
+    <row r="128" spans="1:22">
       <c r="A128" s="5"/>
       <c r="B128" s="5"/>
       <c r="C128" s="5"/>
@@ -4104,9 +4241,10 @@
       <c r="R128" s="5"/>
       <c r="S128" s="5"/>
       <c r="T128" s="5"/>
-      <c r="U128" s="11"/>
-    </row>
-    <row r="129" spans="1:21">
+      <c r="U128" s="5"/>
+      <c r="V128" s="11"/>
+    </row>
+    <row r="129" spans="1:22">
       <c r="A129" s="5"/>
       <c r="B129" s="5"/>
       <c r="C129" s="5"/>
@@ -4127,9 +4265,10 @@
       <c r="R129" s="5"/>
       <c r="S129" s="5"/>
       <c r="T129" s="5"/>
-      <c r="U129" s="11"/>
-    </row>
-    <row r="130" spans="1:21">
+      <c r="U129" s="5"/>
+      <c r="V129" s="11"/>
+    </row>
+    <row r="130" spans="1:22">
       <c r="A130" s="5"/>
       <c r="B130" s="5"/>
       <c r="C130" s="5"/>
@@ -4150,9 +4289,10 @@
       <c r="R130" s="5"/>
       <c r="S130" s="5"/>
       <c r="T130" s="5"/>
-      <c r="U130" s="11"/>
-    </row>
-    <row r="131" spans="1:21">
+      <c r="U130" s="5"/>
+      <c r="V130" s="11"/>
+    </row>
+    <row r="131" spans="1:22">
       <c r="A131" s="5"/>
       <c r="B131" s="5"/>
       <c r="C131" s="5"/>
@@ -4173,9 +4313,10 @@
       <c r="R131" s="5"/>
       <c r="S131" s="5"/>
       <c r="T131" s="5"/>
-      <c r="U131" s="11"/>
-    </row>
-    <row r="132" spans="1:21">
+      <c r="U131" s="5"/>
+      <c r="V131" s="11"/>
+    </row>
+    <row r="132" spans="1:22">
       <c r="A132" s="5"/>
       <c r="B132" s="5"/>
       <c r="C132" s="5"/>
@@ -4196,9 +4337,10 @@
       <c r="R132" s="5"/>
       <c r="S132" s="11"/>
       <c r="T132" s="5"/>
-      <c r="U132" s="11"/>
-    </row>
-    <row r="133" spans="1:21">
+      <c r="U132" s="5"/>
+      <c r="V132" s="11"/>
+    </row>
+    <row r="133" spans="1:22">
       <c r="A133" s="5"/>
       <c r="B133" s="5"/>
       <c r="C133" s="5"/>
@@ -4219,9 +4361,10 @@
       <c r="R133" s="5"/>
       <c r="S133" s="11"/>
       <c r="T133" s="5"/>
-      <c r="U133" s="11"/>
-    </row>
-    <row r="134" spans="1:21">
+      <c r="U133" s="5"/>
+      <c r="V133" s="11"/>
+    </row>
+    <row r="134" spans="1:22">
       <c r="A134" s="5"/>
       <c r="B134" s="5"/>
       <c r="C134" s="5"/>
@@ -4242,9 +4385,10 @@
       <c r="R134" s="5"/>
       <c r="S134" s="11"/>
       <c r="T134" s="5"/>
-      <c r="U134" s="11"/>
-    </row>
-    <row r="135" spans="1:21">
+      <c r="U134" s="5"/>
+      <c r="V134" s="11"/>
+    </row>
+    <row r="135" spans="1:22">
       <c r="A135" s="5"/>
       <c r="B135" s="5"/>
       <c r="C135" s="5"/>
@@ -4265,9 +4409,10 @@
       <c r="R135" s="5"/>
       <c r="S135" s="11"/>
       <c r="T135" s="5"/>
-      <c r="U135" s="11"/>
-    </row>
-    <row r="136" spans="1:21">
+      <c r="U135" s="5"/>
+      <c r="V135" s="11"/>
+    </row>
+    <row r="136" spans="1:22">
       <c r="A136" s="5"/>
       <c r="B136" s="5"/>
       <c r="C136" s="5"/>
@@ -4288,9 +4433,10 @@
       <c r="R136" s="5"/>
       <c r="S136" s="11"/>
       <c r="T136" s="5"/>
-      <c r="U136" s="11"/>
-    </row>
-    <row r="137" spans="1:21">
+      <c r="U136" s="5"/>
+      <c r="V136" s="11"/>
+    </row>
+    <row r="137" spans="1:22">
       <c r="A137" s="5"/>
       <c r="B137" s="5"/>
       <c r="C137" s="5"/>
@@ -4311,9 +4457,10 @@
       <c r="R137" s="5"/>
       <c r="S137" s="11"/>
       <c r="T137" s="5"/>
-      <c r="U137" s="11"/>
-    </row>
-    <row r="138" spans="1:21">
+      <c r="U137" s="5"/>
+      <c r="V137" s="11"/>
+    </row>
+    <row r="138" spans="1:22">
       <c r="A138" s="5"/>
       <c r="B138" s="5"/>
       <c r="C138" s="5"/>
@@ -4334,9 +4481,10 @@
       <c r="R138" s="5"/>
       <c r="S138" s="11"/>
       <c r="T138" s="5"/>
-      <c r="U138" s="11"/>
-    </row>
-    <row r="139" spans="1:21">
+      <c r="U138" s="5"/>
+      <c r="V138" s="11"/>
+    </row>
+    <row r="139" spans="1:22">
       <c r="A139" s="5"/>
       <c r="B139" s="5"/>
       <c r="C139" s="5"/>
@@ -4357,9 +4505,10 @@
       <c r="R139" s="5"/>
       <c r="S139" s="11"/>
       <c r="T139" s="5"/>
-      <c r="U139" s="11"/>
-    </row>
-    <row r="140" spans="1:21">
+      <c r="U139" s="5"/>
+      <c r="V139" s="11"/>
+    </row>
+    <row r="140" spans="1:22">
       <c r="A140" s="5"/>
       <c r="B140" s="5"/>
       <c r="C140" s="5"/>
@@ -4380,9 +4529,10 @@
       <c r="R140" s="5"/>
       <c r="S140" s="11"/>
       <c r="T140" s="5"/>
-      <c r="U140" s="11"/>
-    </row>
-    <row r="141" spans="1:21" s="16" customFormat="1">
+      <c r="U140" s="5"/>
+      <c r="V140" s="11"/>
+    </row>
+    <row r="141" spans="1:22" s="16" customFormat="1">
       <c r="A141" s="5"/>
       <c r="B141" s="5"/>
       <c r="C141" s="5"/>
@@ -4403,9 +4553,10 @@
       <c r="R141" s="5"/>
       <c r="S141" s="5"/>
       <c r="T141" s="5"/>
-      <c r="U141" s="11"/>
-    </row>
-    <row r="142" spans="1:21" s="17" customFormat="1">
+      <c r="U141" s="5"/>
+      <c r="V141" s="11"/>
+    </row>
+    <row r="142" spans="1:22" s="17" customFormat="1">
       <c r="A142" s="5"/>
       <c r="B142" s="5"/>
       <c r="C142" s="5"/>
@@ -4426,9 +4577,10 @@
       <c r="R142" s="5"/>
       <c r="S142" s="5"/>
       <c r="T142" s="5"/>
-      <c r="U142" s="11"/>
-    </row>
-    <row r="143" spans="1:21" s="17" customFormat="1">
+      <c r="U142" s="5"/>
+      <c r="V142" s="11"/>
+    </row>
+    <row r="143" spans="1:22" s="17" customFormat="1">
       <c r="A143" s="5"/>
       <c r="B143" s="5"/>
       <c r="C143" s="5"/>
@@ -4449,9 +4601,10 @@
       <c r="R143" s="5"/>
       <c r="S143" s="5"/>
       <c r="T143" s="5"/>
-      <c r="U143" s="11"/>
-    </row>
-    <row r="144" spans="1:21" s="17" customFormat="1">
+      <c r="U143" s="5"/>
+      <c r="V143" s="11"/>
+    </row>
+    <row r="144" spans="1:22" s="17" customFormat="1">
       <c r="A144" s="5"/>
       <c r="B144" s="5"/>
       <c r="C144" s="5"/>
@@ -4472,9 +4625,10 @@
       <c r="R144" s="5"/>
       <c r="S144" s="18"/>
       <c r="T144" s="5"/>
-      <c r="U144" s="11"/>
-    </row>
-    <row r="145" spans="1:21" s="17" customFormat="1">
+      <c r="U144" s="5"/>
+      <c r="V144" s="11"/>
+    </row>
+    <row r="145" spans="1:22" s="17" customFormat="1">
       <c r="A145" s="5"/>
       <c r="B145" s="5"/>
       <c r="C145" s="5"/>
@@ -4495,9 +4649,10 @@
       <c r="R145" s="5"/>
       <c r="S145" s="5"/>
       <c r="T145" s="5"/>
-      <c r="U145" s="11"/>
-    </row>
-    <row r="146" spans="1:21" s="17" customFormat="1">
+      <c r="U145" s="5"/>
+      <c r="V145" s="11"/>
+    </row>
+    <row r="146" spans="1:22" s="17" customFormat="1">
       <c r="A146" s="5"/>
       <c r="B146" s="5"/>
       <c r="C146" s="5"/>
@@ -4518,9 +4673,10 @@
       <c r="R146" s="5"/>
       <c r="S146" s="18"/>
       <c r="T146" s="5"/>
-      <c r="U146" s="11"/>
-    </row>
-    <row r="147" spans="1:21" s="17" customFormat="1">
+      <c r="U146" s="5"/>
+      <c r="V146" s="11"/>
+    </row>
+    <row r="147" spans="1:22" s="17" customFormat="1">
       <c r="A147" s="5"/>
       <c r="B147" s="5"/>
       <c r="C147" s="5"/>
@@ -4541,9 +4697,10 @@
       <c r="R147" s="5"/>
       <c r="S147" s="5"/>
       <c r="T147" s="5"/>
-      <c r="U147" s="11"/>
-    </row>
-    <row r="148" spans="1:21" s="17" customFormat="1">
+      <c r="U147" s="5"/>
+      <c r="V147" s="11"/>
+    </row>
+    <row r="148" spans="1:22" s="17" customFormat="1">
       <c r="A148" s="5"/>
       <c r="B148" s="5"/>
       <c r="C148" s="5"/>
@@ -4564,9 +4721,10 @@
       <c r="R148" s="5"/>
       <c r="S148" s="5"/>
       <c r="T148" s="5"/>
-      <c r="U148" s="11"/>
-    </row>
-    <row r="149" spans="1:21" s="17" customFormat="1">
+      <c r="U148" s="5"/>
+      <c r="V148" s="11"/>
+    </row>
+    <row r="149" spans="1:22" s="17" customFormat="1">
       <c r="A149" s="5"/>
       <c r="B149" s="5"/>
       <c r="C149" s="5"/>
@@ -4587,9 +4745,10 @@
       <c r="R149" s="5"/>
       <c r="S149" s="5"/>
       <c r="T149" s="5"/>
-      <c r="U149" s="11"/>
-    </row>
-    <row r="150" spans="1:21" s="17" customFormat="1">
+      <c r="U149" s="5"/>
+      <c r="V149" s="11"/>
+    </row>
+    <row r="150" spans="1:22" s="17" customFormat="1">
       <c r="A150" s="5"/>
       <c r="B150" s="5"/>
       <c r="C150" s="5"/>
@@ -4610,9 +4769,10 @@
       <c r="R150" s="5"/>
       <c r="S150" s="18"/>
       <c r="T150" s="5"/>
-      <c r="U150" s="11"/>
-    </row>
-    <row r="151" spans="1:21">
+      <c r="U150" s="5"/>
+      <c r="V150" s="11"/>
+    </row>
+    <row r="151" spans="1:22">
       <c r="A151" s="5"/>
       <c r="B151" s="5"/>
       <c r="C151" s="5"/>
@@ -4633,9 +4793,10 @@
       <c r="R151" s="5"/>
       <c r="S151" s="5"/>
       <c r="T151" s="5"/>
-      <c r="U151" s="11"/>
-    </row>
-    <row r="152" spans="1:21" s="17" customFormat="1">
+      <c r="U151" s="5"/>
+      <c r="V151" s="11"/>
+    </row>
+    <row r="152" spans="1:22" s="17" customFormat="1">
       <c r="A152" s="5"/>
       <c r="B152" s="5"/>
       <c r="C152" s="5"/>
@@ -4656,9 +4817,10 @@
       <c r="R152" s="5"/>
       <c r="S152" s="5"/>
       <c r="T152" s="5"/>
-      <c r="U152" s="11"/>
-    </row>
-    <row r="153" spans="1:21">
+      <c r="U152" s="5"/>
+      <c r="V152" s="11"/>
+    </row>
+    <row r="153" spans="1:22">
       <c r="A153" s="5"/>
       <c r="B153" s="5"/>
       <c r="C153" s="5"/>
@@ -4679,9 +4841,10 @@
       <c r="R153" s="5"/>
       <c r="S153" s="5"/>
       <c r="T153" s="5"/>
-      <c r="U153" s="11"/>
-    </row>
-    <row r="154" spans="1:21" s="17" customFormat="1">
+      <c r="U153" s="5"/>
+      <c r="V153" s="11"/>
+    </row>
+    <row r="154" spans="1:22" s="17" customFormat="1">
       <c r="A154" s="5"/>
       <c r="B154" s="5"/>
       <c r="C154" s="5"/>
@@ -4702,10 +4865,11 @@
       <c r="R154" s="5"/>
       <c r="S154" s="5"/>
       <c r="T154" s="5"/>
-      <c r="U154" s="11"/>
+      <c r="U154" s="5"/>
+      <c r="V154" s="11"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U1" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
+  <autoFilter ref="A1:V1" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
   <dataConsolidate/>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
updated document and add case
</commit_message>
<xml_diff>
--- a/projects/automation_exercise/api/case/testcase-automation_exercise.xlsx
+++ b/projects/automation_exercise/api/case/testcase-automation_exercise.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/606929f86db40629/Documents/Python/automation_framework/projects/automation_exercise/api/case/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="74" documentId="8_{B959E1B4-B71D-476A-B78C-D11EC8419DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A17B3769-6AE4-4BA4-A5D8-4554B1C7EB72}"/>
+  <xr:revisionPtr revIDLastSave="102" documentId="8_{B959E1B4-B71D-476A-B78C-D11EC8419DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{93DE387E-C4AE-4052-9297-4D0F728C7DC2}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AB49B25E-9B57-422D-B60E-7F12796728DD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{AB49B25E-9B57-422D-B60E-7F12796728DD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -23,17 +23,6 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -44,33 +33,7 @@
     <author>Olivia Dou</author>
   </authors>
   <commentList>
-    <comment ref="D11" authorId="0" shapeId="0" xr:uid="{B5BBE645-72D6-419C-BBAE-9E3E16CBD836}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="宋体"/>
-            <family val="3"/>
-            <charset val="134"/>
-          </rPr>
-          <t>Olivia Dou:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="宋体"/>
-            <family val="3"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
-会有脏数据，部分模型准确率为空值</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D51" authorId="0" shapeId="0" xr:uid="{2C9DE514-8D0A-4A37-825F-04CB76354E06}">
+    <comment ref="D52" authorId="0" shapeId="0" xr:uid="{2C9DE514-8D0A-4A37-825F-04CB76354E06}">
       <text>
         <r>
           <rPr>
@@ -96,7 +59,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O63" authorId="0" shapeId="0" xr:uid="{C962C448-2AF1-44F0-B1DD-E07C86A2D785}">
+    <comment ref="O64" authorId="0" shapeId="0" xr:uid="{C962C448-2AF1-44F0-B1DD-E07C86A2D785}">
       <text>
         <r>
           <rPr>
@@ -122,7 +85,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O64" authorId="0" shapeId="0" xr:uid="{A89CBD07-4F5C-4144-B5AD-5635780593A2}">
+    <comment ref="O65" authorId="0" shapeId="0" xr:uid="{A89CBD07-4F5C-4144-B5AD-5635780593A2}">
       <text>
         <r>
           <rPr>
@@ -148,7 +111,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O66" authorId="0" shapeId="0" xr:uid="{702345AA-186D-47A7-AD24-B0AE9F3EB042}">
+    <comment ref="O67" authorId="0" shapeId="0" xr:uid="{702345AA-186D-47A7-AD24-B0AE9F3EB042}">
       <text>
         <r>
           <rPr>
@@ -174,7 +137,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D91" authorId="0" shapeId="0" xr:uid="{70F2CE92-043A-4715-8389-EE7D40D6B005}">
+    <comment ref="D92" authorId="0" shapeId="0" xr:uid="{70F2CE92-043A-4715-8389-EE7D40D6B005}">
       <text>
         <r>
           <rPr>
@@ -201,7 +164,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D98" authorId="0" shapeId="0" xr:uid="{86C02B5B-9397-479A-8347-5ADEC6BFED9B}">
+    <comment ref="D99" authorId="0" shapeId="0" xr:uid="{86C02B5B-9397-479A-8347-5ADEC6BFED9B}">
       <text>
         <r>
           <rPr>
@@ -228,7 +191,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D105" authorId="0" shapeId="0" xr:uid="{DCDF529E-2EE7-4F64-80AC-224796653F95}">
+    <comment ref="D106" authorId="0" shapeId="0" xr:uid="{DCDF529E-2EE7-4F64-80AC-224796653F95}">
       <text>
         <r>
           <rPr>
@@ -255,7 +218,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O112" authorId="0" shapeId="0" xr:uid="{C812EAC0-7407-4E3D-A470-8E0B1C31EF80}">
+    <comment ref="O113" authorId="0" shapeId="0" xr:uid="{C812EAC0-7407-4E3D-A470-8E0B1C31EF80}">
       <text>
         <r>
           <rPr>
@@ -281,7 +244,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O114" authorId="0" shapeId="0" xr:uid="{185AA492-11BE-4576-97BD-74BE3797C4B3}">
+    <comment ref="O115" authorId="0" shapeId="0" xr:uid="{185AA492-11BE-4576-97BD-74BE3797C4B3}">
       <text>
         <r>
           <rPr>
@@ -307,7 +270,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O116" authorId="0" shapeId="0" xr:uid="{F90DFE34-1C1D-4DC5-A774-1BD7B775C997}">
+    <comment ref="O117" authorId="0" shapeId="0" xr:uid="{F90DFE34-1C1D-4DC5-A774-1BD7B775C997}">
       <text>
         <r>
           <rPr>
@@ -333,7 +296,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E124" authorId="0" shapeId="0" xr:uid="{1D66DA03-0E6E-4003-94E8-371E493401C7}">
+    <comment ref="E125" authorId="0" shapeId="0" xr:uid="{1D66DA03-0E6E-4003-94E8-371E493401C7}">
       <text>
         <r>
           <rPr>
@@ -364,7 +327,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="55">
   <si>
     <t>Case_Name</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -513,6 +476,74 @@
   </si>
   <si>
     <t>${projects.automation_exercise.libs.demo.py::function_used_by_teardown()}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>POST To Search Product</t>
+  </si>
+  <si>
+    <t>post_to_search_product</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{"search_product":"tshirt"}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/api/searchProduct</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>["=","$.responseCode",200];
+["=","$.products[*].category.category","Tshirts"]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>API1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>API2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>API5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>API6</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>["=","$.responseCode",400];
+["=","$.message","Bad request, search_product parameter is missing in POST request."]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>POST To Search Product without search_product parameter</t>
+  </si>
+  <si>
+    <t>post_to_search_product_without_parameter</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>API3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Get All Brands List</t>
+  </si>
+  <si>
+    <t>get_all_brand_list</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/api/brandsList</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>["=","$.responseCode",200];
+["=",["length","$.brands[*]","list relation"],34]</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -520,7 +551,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -720,13 +751,13 @@
     <xdr:from>
       <xdr:col>21</xdr:col>
       <xdr:colOff>1047750</xdr:colOff>
-      <xdr:row>1794</xdr:row>
+      <xdr:row>1788</xdr:row>
       <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
       <xdr:colOff>142875</xdr:colOff>
-      <xdr:row>1949</xdr:row>
+      <xdr:row>1943</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1055,8 +1086,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{571522A3-8A90-45FA-BDC2-DE8E1EFD9C0E}">
-  <dimension ref="A1:V154"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <dimension ref="A1:V155"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="18.125" style="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.5" style="12" customWidth="1"/>
@@ -1080,7 +1111,7 @@
     <col min="23" max="16384" width="9" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="8" customFormat="1" ht="27">
+    <row r="1" spans="1:22" s="8" customFormat="1" ht="27" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>23</v>
       </c>
@@ -1148,8 +1179,10 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:22" ht="67.5">
-      <c r="A2" s="5"/>
+    <row r="2" spans="1:22" ht="67.5" x14ac:dyDescent="0.15">
+      <c r="A2" s="5" t="s">
+        <v>43</v>
+      </c>
       <c r="B2" s="5" t="s">
         <v>13</v>
       </c>
@@ -1196,8 +1229,10 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:22" ht="81">
-      <c r="A3" s="5"/>
+    <row r="3" spans="1:22" ht="81" x14ac:dyDescent="0.15">
+      <c r="A3" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="B3" s="5" t="s">
         <v>19</v>
       </c>
@@ -1244,79 +1279,153 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:22">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
+    <row r="4" spans="1:22" ht="27" x14ac:dyDescent="0.15">
+      <c r="A4" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>9</v>
+      </c>
       <c r="G4" s="5"/>
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
       <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="5"/>
+      <c r="K4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L4" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>11</v>
+      </c>
       <c r="N4" s="5"/>
       <c r="O4" s="5"/>
-      <c r="P4" s="5"/>
+      <c r="P4" s="5">
+        <v>200</v>
+      </c>
       <c r="Q4" s="10"/>
       <c r="R4" s="5"/>
-      <c r="S4" s="5"/>
+      <c r="S4" s="5" t="s">
+        <v>54</v>
+      </c>
       <c r="T4" s="5"/>
       <c r="U4" s="5"/>
-      <c r="V4" s="11"/>
-    </row>
-    <row r="5" spans="1:22">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
+      <c r="V4" s="11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" ht="27" x14ac:dyDescent="0.15">
+      <c r="A5" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>9</v>
+      </c>
       <c r="G5" s="5"/>
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="9"/>
-      <c r="M5" s="5"/>
+      <c r="K5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>20</v>
+      </c>
       <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
-      <c r="P5" s="5"/>
+      <c r="O5" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="P5" s="5">
+        <v>200</v>
+      </c>
       <c r="Q5" s="10"/>
       <c r="R5" s="5"/>
-      <c r="S5" s="5"/>
+      <c r="S5" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="T5" s="5"/>
       <c r="U5" s="5"/>
-      <c r="V5" s="11"/>
-    </row>
-    <row r="6" spans="1:22">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
+      <c r="V5" s="11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" ht="67.5" x14ac:dyDescent="0.15">
+      <c r="A6" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>9</v>
+      </c>
       <c r="G6" s="5"/>
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="5"/>
+      <c r="K6" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L6" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>20</v>
+      </c>
       <c r="N6" s="5"/>
       <c r="O6" s="5"/>
-      <c r="P6" s="5"/>
+      <c r="P6" s="5">
+        <v>200</v>
+      </c>
       <c r="Q6" s="10"/>
       <c r="R6" s="5"/>
-      <c r="S6" s="5"/>
+      <c r="S6" s="5" t="s">
+        <v>47</v>
+      </c>
       <c r="T6" s="5"/>
       <c r="U6" s="5"/>
-      <c r="V6" s="11"/>
-    </row>
-    <row r="7" spans="1:22">
+      <c r="V6" s="11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
@@ -1340,7 +1449,7 @@
       <c r="U7" s="5"/>
       <c r="V7" s="11"/>
     </row>
-    <row r="8" spans="1:22">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -1364,7 +1473,7 @@
       <c r="U8" s="5"/>
       <c r="V8" s="11"/>
     </row>
-    <row r="9" spans="1:22">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
@@ -1388,7 +1497,7 @@
       <c r="U9" s="5"/>
       <c r="V9" s="11"/>
     </row>
-    <row r="10" spans="1:22">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -1412,7 +1521,7 @@
       <c r="U10" s="5"/>
       <c r="V10" s="11"/>
     </row>
-    <row r="11" spans="1:22">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -1436,7 +1545,7 @@
       <c r="U11" s="5"/>
       <c r="V11" s="11"/>
     </row>
-    <row r="12" spans="1:22">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -1460,7 +1569,7 @@
       <c r="U12" s="5"/>
       <c r="V12" s="11"/>
     </row>
-    <row r="13" spans="1:22">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -1484,7 +1593,7 @@
       <c r="U13" s="5"/>
       <c r="V13" s="11"/>
     </row>
-    <row r="14" spans="1:22">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -1508,7 +1617,7 @@
       <c r="U14" s="5"/>
       <c r="V14" s="11"/>
     </row>
-    <row r="15" spans="1:22">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -1532,7 +1641,7 @@
       <c r="U15" s="5"/>
       <c r="V15" s="11"/>
     </row>
-    <row r="16" spans="1:22">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -1556,7 +1665,7 @@
       <c r="U16" s="5"/>
       <c r="V16" s="11"/>
     </row>
-    <row r="17" spans="1:22">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -1580,7 +1689,7 @@
       <c r="U17" s="5"/>
       <c r="V17" s="11"/>
     </row>
-    <row r="18" spans="1:22">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -1604,7 +1713,7 @@
       <c r="U18" s="5"/>
       <c r="V18" s="11"/>
     </row>
-    <row r="19" spans="1:22">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A19" s="5"/>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -1628,7 +1737,7 @@
       <c r="U19" s="5"/>
       <c r="V19" s="11"/>
     </row>
-    <row r="20" spans="1:22">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -1652,7 +1761,7 @@
       <c r="U20" s="5"/>
       <c r="V20" s="11"/>
     </row>
-    <row r="21" spans="1:22">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A21" s="5"/>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -1676,7 +1785,7 @@
       <c r="U21" s="5"/>
       <c r="V21" s="11"/>
     </row>
-    <row r="22" spans="1:22">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A22" s="5"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -1700,7 +1809,7 @@
       <c r="U22" s="5"/>
       <c r="V22" s="11"/>
     </row>
-    <row r="23" spans="1:22">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A23" s="5"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -1724,7 +1833,7 @@
       <c r="U23" s="5"/>
       <c r="V23" s="11"/>
     </row>
-    <row r="24" spans="1:22">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A24" s="5"/>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
@@ -1748,7 +1857,7 @@
       <c r="U24" s="5"/>
       <c r="V24" s="11"/>
     </row>
-    <row r="25" spans="1:22">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A25" s="5"/>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -1772,7 +1881,7 @@
       <c r="U25" s="5"/>
       <c r="V25" s="11"/>
     </row>
-    <row r="26" spans="1:22">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A26" s="5"/>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
@@ -1796,7 +1905,7 @@
       <c r="U26" s="5"/>
       <c r="V26" s="11"/>
     </row>
-    <row r="27" spans="1:22">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A27" s="5"/>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -1820,7 +1929,7 @@
       <c r="U27" s="5"/>
       <c r="V27" s="11"/>
     </row>
-    <row r="28" spans="1:22">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A28" s="5"/>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -1844,7 +1953,7 @@
       <c r="U28" s="5"/>
       <c r="V28" s="11"/>
     </row>
-    <row r="29" spans="1:22">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A29" s="5"/>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -1868,7 +1977,7 @@
       <c r="U29" s="5"/>
       <c r="V29" s="11"/>
     </row>
-    <row r="30" spans="1:22">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A30" s="5"/>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
@@ -1892,7 +2001,7 @@
       <c r="U30" s="5"/>
       <c r="V30" s="11"/>
     </row>
-    <row r="31" spans="1:22">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A31" s="5"/>
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>
@@ -1916,7 +2025,7 @@
       <c r="U31" s="5"/>
       <c r="V31" s="11"/>
     </row>
-    <row r="32" spans="1:22">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A32" s="5"/>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -1940,7 +2049,7 @@
       <c r="U32" s="5"/>
       <c r="V32" s="11"/>
     </row>
-    <row r="33" spans="1:22">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A33" s="5"/>
       <c r="B33" s="5"/>
       <c r="C33" s="5"/>
@@ -1964,7 +2073,7 @@
       <c r="U33" s="5"/>
       <c r="V33" s="11"/>
     </row>
-    <row r="34" spans="1:22">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A34" s="5"/>
       <c r="B34" s="5"/>
       <c r="C34" s="5"/>
@@ -1988,7 +2097,7 @@
       <c r="U34" s="5"/>
       <c r="V34" s="11"/>
     </row>
-    <row r="35" spans="1:22">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A35" s="5"/>
       <c r="B35" s="5"/>
       <c r="C35" s="5"/>
@@ -2012,7 +2121,7 @@
       <c r="U35" s="5"/>
       <c r="V35" s="11"/>
     </row>
-    <row r="36" spans="1:22">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A36" s="5"/>
       <c r="B36" s="5"/>
       <c r="C36" s="5"/>
@@ -2036,7 +2145,7 @@
       <c r="U36" s="5"/>
       <c r="V36" s="11"/>
     </row>
-    <row r="37" spans="1:22">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A37" s="5"/>
       <c r="B37" s="5"/>
       <c r="C37" s="5"/>
@@ -2060,7 +2169,7 @@
       <c r="U37" s="5"/>
       <c r="V37" s="11"/>
     </row>
-    <row r="38" spans="1:22">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A38" s="5"/>
       <c r="B38" s="5"/>
       <c r="C38" s="5"/>
@@ -2084,7 +2193,7 @@
       <c r="U38" s="5"/>
       <c r="V38" s="11"/>
     </row>
-    <row r="39" spans="1:22">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A39" s="5"/>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
@@ -2108,7 +2217,7 @@
       <c r="U39" s="5"/>
       <c r="V39" s="11"/>
     </row>
-    <row r="40" spans="1:22">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A40" s="5"/>
       <c r="B40" s="5"/>
       <c r="C40" s="5"/>
@@ -2132,7 +2241,7 @@
       <c r="U40" s="5"/>
       <c r="V40" s="11"/>
     </row>
-    <row r="41" spans="1:22">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A41" s="5"/>
       <c r="B41" s="5"/>
       <c r="C41" s="5"/>
@@ -2156,7 +2265,7 @@
       <c r="U41" s="5"/>
       <c r="V41" s="11"/>
     </row>
-    <row r="42" spans="1:22">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A42" s="5"/>
       <c r="B42" s="5"/>
       <c r="C42" s="5"/>
@@ -2180,7 +2289,7 @@
       <c r="U42" s="5"/>
       <c r="V42" s="11"/>
     </row>
-    <row r="43" spans="1:22">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A43" s="5"/>
       <c r="B43" s="5"/>
       <c r="C43" s="5"/>
@@ -2204,7 +2313,7 @@
       <c r="U43" s="5"/>
       <c r="V43" s="11"/>
     </row>
-    <row r="44" spans="1:22">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A44" s="5"/>
       <c r="B44" s="5"/>
       <c r="C44" s="5"/>
@@ -2228,7 +2337,7 @@
       <c r="U44" s="5"/>
       <c r="V44" s="11"/>
     </row>
-    <row r="45" spans="1:22">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A45" s="5"/>
       <c r="B45" s="5"/>
       <c r="C45" s="5"/>
@@ -2252,7 +2361,7 @@
       <c r="U45" s="5"/>
       <c r="V45" s="11"/>
     </row>
-    <row r="46" spans="1:22">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A46" s="5"/>
       <c r="B46" s="5"/>
       <c r="C46" s="5"/>
@@ -2271,12 +2380,12 @@
       <c r="P46" s="5"/>
       <c r="Q46" s="10"/>
       <c r="R46" s="5"/>
-      <c r="S46" s="10"/>
+      <c r="S46" s="5"/>
       <c r="T46" s="5"/>
       <c r="U46" s="5"/>
       <c r="V46" s="11"/>
     </row>
-    <row r="47" spans="1:22">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A47" s="5"/>
       <c r="B47" s="5"/>
       <c r="C47" s="5"/>
@@ -2295,12 +2404,12 @@
       <c r="P47" s="5"/>
       <c r="Q47" s="10"/>
       <c r="R47" s="5"/>
-      <c r="S47" s="5"/>
+      <c r="S47" s="10"/>
       <c r="T47" s="5"/>
       <c r="U47" s="5"/>
       <c r="V47" s="11"/>
     </row>
-    <row r="48" spans="1:22">
+    <row r="48" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A48" s="5"/>
       <c r="B48" s="5"/>
       <c r="C48" s="5"/>
@@ -2324,7 +2433,7 @@
       <c r="U48" s="5"/>
       <c r="V48" s="11"/>
     </row>
-    <row r="49" spans="1:22">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A49" s="5"/>
       <c r="B49" s="5"/>
       <c r="C49" s="5"/>
@@ -2348,7 +2457,7 @@
       <c r="U49" s="5"/>
       <c r="V49" s="11"/>
     </row>
-    <row r="50" spans="1:22">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A50" s="5"/>
       <c r="B50" s="5"/>
       <c r="C50" s="5"/>
@@ -2372,7 +2481,7 @@
       <c r="U50" s="5"/>
       <c r="V50" s="11"/>
     </row>
-    <row r="51" spans="1:22">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A51" s="5"/>
       <c r="B51" s="5"/>
       <c r="C51" s="5"/>
@@ -2396,7 +2505,7 @@
       <c r="U51" s="5"/>
       <c r="V51" s="11"/>
     </row>
-    <row r="52" spans="1:22">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A52" s="5"/>
       <c r="B52" s="5"/>
       <c r="C52" s="5"/>
@@ -2415,12 +2524,12 @@
       <c r="P52" s="5"/>
       <c r="Q52" s="10"/>
       <c r="R52" s="5"/>
-      <c r="S52" s="10"/>
+      <c r="S52" s="5"/>
       <c r="T52" s="5"/>
       <c r="U52" s="5"/>
       <c r="V52" s="11"/>
     </row>
-    <row r="53" spans="1:22">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A53" s="5"/>
       <c r="B53" s="5"/>
       <c r="C53" s="5"/>
@@ -2439,12 +2548,12 @@
       <c r="P53" s="5"/>
       <c r="Q53" s="10"/>
       <c r="R53" s="5"/>
-      <c r="S53" s="5"/>
+      <c r="S53" s="10"/>
       <c r="T53" s="5"/>
       <c r="U53" s="5"/>
       <c r="V53" s="11"/>
     </row>
-    <row r="54" spans="1:22">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A54" s="5"/>
       <c r="B54" s="5"/>
       <c r="C54" s="5"/>
@@ -2468,7 +2577,7 @@
       <c r="U54" s="5"/>
       <c r="V54" s="11"/>
     </row>
-    <row r="55" spans="1:22">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A55" s="5"/>
       <c r="B55" s="5"/>
       <c r="C55" s="5"/>
@@ -2487,12 +2596,12 @@
       <c r="P55" s="5"/>
       <c r="Q55" s="10"/>
       <c r="R55" s="5"/>
-      <c r="S55" s="10"/>
+      <c r="S55" s="5"/>
       <c r="T55" s="5"/>
       <c r="U55" s="5"/>
       <c r="V55" s="11"/>
     </row>
-    <row r="56" spans="1:22">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A56" s="5"/>
       <c r="B56" s="5"/>
       <c r="C56" s="5"/>
@@ -2511,12 +2620,12 @@
       <c r="P56" s="5"/>
       <c r="Q56" s="10"/>
       <c r="R56" s="5"/>
-      <c r="S56" s="5"/>
+      <c r="S56" s="10"/>
       <c r="T56" s="5"/>
       <c r="U56" s="5"/>
       <c r="V56" s="11"/>
     </row>
-    <row r="57" spans="1:22">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A57" s="5"/>
       <c r="B57" s="5"/>
       <c r="C57" s="5"/>
@@ -2540,7 +2649,7 @@
       <c r="U57" s="5"/>
       <c r="V57" s="11"/>
     </row>
-    <row r="58" spans="1:22">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A58" s="5"/>
       <c r="B58" s="5"/>
       <c r="C58" s="5"/>
@@ -2557,14 +2666,14 @@
       <c r="N58" s="5"/>
       <c r="O58" s="5"/>
       <c r="P58" s="5"/>
-      <c r="Q58" s="5"/>
+      <c r="Q58" s="10"/>
       <c r="R58" s="5"/>
       <c r="S58" s="5"/>
       <c r="T58" s="5"/>
       <c r="U58" s="5"/>
       <c r="V58" s="11"/>
     </row>
-    <row r="59" spans="1:22">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A59" s="5"/>
       <c r="B59" s="5"/>
       <c r="C59" s="5"/>
@@ -2581,14 +2690,14 @@
       <c r="N59" s="5"/>
       <c r="O59" s="5"/>
       <c r="P59" s="5"/>
-      <c r="Q59" s="10"/>
+      <c r="Q59" s="5"/>
       <c r="R59" s="5"/>
       <c r="S59" s="5"/>
       <c r="T59" s="5"/>
       <c r="U59" s="5"/>
       <c r="V59" s="11"/>
     </row>
-    <row r="60" spans="1:22">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A60" s="5"/>
       <c r="B60" s="5"/>
       <c r="C60" s="5"/>
@@ -2605,14 +2714,14 @@
       <c r="N60" s="5"/>
       <c r="O60" s="5"/>
       <c r="P60" s="5"/>
-      <c r="Q60" s="5"/>
+      <c r="Q60" s="10"/>
       <c r="R60" s="5"/>
       <c r="S60" s="5"/>
       <c r="T60" s="5"/>
       <c r="U60" s="5"/>
       <c r="V60" s="11"/>
     </row>
-    <row r="61" spans="1:22">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A61" s="5"/>
       <c r="B61" s="5"/>
       <c r="C61" s="5"/>
@@ -2629,14 +2738,14 @@
       <c r="N61" s="5"/>
       <c r="O61" s="5"/>
       <c r="P61" s="5"/>
-      <c r="Q61" s="10"/>
+      <c r="Q61" s="5"/>
       <c r="R61" s="5"/>
       <c r="S61" s="5"/>
       <c r="T61" s="5"/>
       <c r="U61" s="5"/>
       <c r="V61" s="11"/>
     </row>
-    <row r="62" spans="1:22">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A62" s="5"/>
       <c r="B62" s="5"/>
       <c r="C62" s="5"/>
@@ -2653,14 +2762,14 @@
       <c r="N62" s="5"/>
       <c r="O62" s="5"/>
       <c r="P62" s="5"/>
-      <c r="Q62" s="5"/>
+      <c r="Q62" s="10"/>
       <c r="R62" s="5"/>
       <c r="S62" s="5"/>
       <c r="T62" s="5"/>
       <c r="U62" s="5"/>
       <c r="V62" s="11"/>
     </row>
-    <row r="63" spans="1:22">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A63" s="5"/>
       <c r="B63" s="5"/>
       <c r="C63" s="5"/>
@@ -2677,14 +2786,14 @@
       <c r="N63" s="5"/>
       <c r="O63" s="5"/>
       <c r="P63" s="5"/>
-      <c r="Q63" s="10"/>
+      <c r="Q63" s="5"/>
       <c r="R63" s="5"/>
       <c r="S63" s="5"/>
       <c r="T63" s="5"/>
       <c r="U63" s="5"/>
       <c r="V63" s="11"/>
     </row>
-    <row r="64" spans="1:22">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A64" s="5"/>
       <c r="B64" s="5"/>
       <c r="C64" s="5"/>
@@ -2708,7 +2817,7 @@
       <c r="U64" s="5"/>
       <c r="V64" s="11"/>
     </row>
-    <row r="65" spans="1:22">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A65" s="5"/>
       <c r="B65" s="5"/>
       <c r="C65" s="5"/>
@@ -2720,7 +2829,7 @@
       <c r="I65" s="5"/>
       <c r="J65" s="5"/>
       <c r="K65" s="5"/>
-      <c r="L65" s="13"/>
+      <c r="L65" s="9"/>
       <c r="M65" s="5"/>
       <c r="N65" s="5"/>
       <c r="O65" s="5"/>
@@ -2732,7 +2841,7 @@
       <c r="U65" s="5"/>
       <c r="V65" s="11"/>
     </row>
-    <row r="66" spans="1:22">
+    <row r="66" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A66" s="5"/>
       <c r="B66" s="5"/>
       <c r="C66" s="5"/>
@@ -2744,7 +2853,7 @@
       <c r="I66" s="5"/>
       <c r="J66" s="5"/>
       <c r="K66" s="5"/>
-      <c r="L66" s="9"/>
+      <c r="L66" s="13"/>
       <c r="M66" s="5"/>
       <c r="N66" s="5"/>
       <c r="O66" s="5"/>
@@ -2756,7 +2865,7 @@
       <c r="U66" s="5"/>
       <c r="V66" s="11"/>
     </row>
-    <row r="67" spans="1:22">
+    <row r="67" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A67" s="5"/>
       <c r="B67" s="5"/>
       <c r="C67" s="5"/>
@@ -2773,14 +2882,14 @@
       <c r="N67" s="5"/>
       <c r="O67" s="5"/>
       <c r="P67" s="5"/>
-      <c r="Q67" s="5"/>
+      <c r="Q67" s="10"/>
       <c r="R67" s="5"/>
       <c r="S67" s="5"/>
       <c r="T67" s="5"/>
       <c r="U67" s="5"/>
       <c r="V67" s="11"/>
     </row>
-    <row r="68" spans="1:22">
+    <row r="68" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A68" s="5"/>
       <c r="B68" s="5"/>
       <c r="C68" s="5"/>
@@ -2797,14 +2906,14 @@
       <c r="N68" s="5"/>
       <c r="O68" s="5"/>
       <c r="P68" s="5"/>
-      <c r="Q68" s="10"/>
+      <c r="Q68" s="5"/>
       <c r="R68" s="5"/>
       <c r="S68" s="5"/>
       <c r="T68" s="5"/>
       <c r="U68" s="5"/>
       <c r="V68" s="11"/>
     </row>
-    <row r="69" spans="1:22">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A69" s="5"/>
       <c r="B69" s="5"/>
       <c r="C69" s="5"/>
@@ -2828,7 +2937,7 @@
       <c r="U69" s="5"/>
       <c r="V69" s="11"/>
     </row>
-    <row r="70" spans="1:22">
+    <row r="70" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A70" s="5"/>
       <c r="B70" s="5"/>
       <c r="C70" s="5"/>
@@ -2845,14 +2954,14 @@
       <c r="N70" s="5"/>
       <c r="O70" s="5"/>
       <c r="P70" s="5"/>
-      <c r="Q70" s="5"/>
+      <c r="Q70" s="10"/>
       <c r="R70" s="5"/>
       <c r="S70" s="5"/>
       <c r="T70" s="5"/>
       <c r="U70" s="5"/>
       <c r="V70" s="11"/>
     </row>
-    <row r="71" spans="1:22">
+    <row r="71" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A71" s="5"/>
       <c r="B71" s="5"/>
       <c r="C71" s="5"/>
@@ -2876,7 +2985,7 @@
       <c r="U71" s="5"/>
       <c r="V71" s="11"/>
     </row>
-    <row r="72" spans="1:22">
+    <row r="72" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A72" s="5"/>
       <c r="B72" s="5"/>
       <c r="C72" s="5"/>
@@ -2893,14 +3002,14 @@
       <c r="N72" s="5"/>
       <c r="O72" s="5"/>
       <c r="P72" s="5"/>
-      <c r="Q72" s="10"/>
+      <c r="Q72" s="5"/>
       <c r="R72" s="5"/>
       <c r="S72" s="5"/>
       <c r="T72" s="5"/>
       <c r="U72" s="5"/>
       <c r="V72" s="11"/>
     </row>
-    <row r="73" spans="1:22">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A73" s="5"/>
       <c r="B73" s="5"/>
       <c r="C73" s="5"/>
@@ -2924,7 +3033,7 @@
       <c r="U73" s="5"/>
       <c r="V73" s="11"/>
     </row>
-    <row r="74" spans="1:22">
+    <row r="74" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A74" s="5"/>
       <c r="B74" s="5"/>
       <c r="C74" s="5"/>
@@ -2948,7 +3057,7 @@
       <c r="U74" s="5"/>
       <c r="V74" s="11"/>
     </row>
-    <row r="75" spans="1:22">
+    <row r="75" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A75" s="5"/>
       <c r="B75" s="5"/>
       <c r="C75" s="5"/>
@@ -2972,7 +3081,7 @@
       <c r="U75" s="5"/>
       <c r="V75" s="11"/>
     </row>
-    <row r="76" spans="1:22">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A76" s="5"/>
       <c r="B76" s="5"/>
       <c r="C76" s="5"/>
@@ -2996,7 +3105,7 @@
       <c r="U76" s="5"/>
       <c r="V76" s="11"/>
     </row>
-    <row r="77" spans="1:22">
+    <row r="77" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A77" s="5"/>
       <c r="B77" s="5"/>
       <c r="C77" s="5"/>
@@ -3020,7 +3129,7 @@
       <c r="U77" s="5"/>
       <c r="V77" s="11"/>
     </row>
-    <row r="78" spans="1:22">
+    <row r="78" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A78" s="5"/>
       <c r="B78" s="5"/>
       <c r="C78" s="5"/>
@@ -3044,7 +3153,7 @@
       <c r="U78" s="5"/>
       <c r="V78" s="11"/>
     </row>
-    <row r="79" spans="1:22">
+    <row r="79" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A79" s="5"/>
       <c r="B79" s="5"/>
       <c r="C79" s="5"/>
@@ -3068,7 +3177,7 @@
       <c r="U79" s="5"/>
       <c r="V79" s="11"/>
     </row>
-    <row r="80" spans="1:22">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A80" s="5"/>
       <c r="B80" s="5"/>
       <c r="C80" s="5"/>
@@ -3092,7 +3201,7 @@
       <c r="U80" s="5"/>
       <c r="V80" s="11"/>
     </row>
-    <row r="81" spans="1:22">
+    <row r="81" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A81" s="5"/>
       <c r="B81" s="5"/>
       <c r="C81" s="5"/>
@@ -3116,7 +3225,7 @@
       <c r="U81" s="5"/>
       <c r="V81" s="11"/>
     </row>
-    <row r="82" spans="1:22">
+    <row r="82" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A82" s="5"/>
       <c r="B82" s="5"/>
       <c r="C82" s="5"/>
@@ -3140,7 +3249,7 @@
       <c r="U82" s="5"/>
       <c r="V82" s="11"/>
     </row>
-    <row r="83" spans="1:22">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A83" s="5"/>
       <c r="B83" s="5"/>
       <c r="C83" s="5"/>
@@ -3164,7 +3273,7 @@
       <c r="U83" s="5"/>
       <c r="V83" s="11"/>
     </row>
-    <row r="84" spans="1:22">
+    <row r="84" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A84" s="5"/>
       <c r="B84" s="5"/>
       <c r="C84" s="5"/>
@@ -3188,7 +3297,7 @@
       <c r="U84" s="5"/>
       <c r="V84" s="11"/>
     </row>
-    <row r="85" spans="1:22">
+    <row r="85" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A85" s="5"/>
       <c r="B85" s="5"/>
       <c r="C85" s="5"/>
@@ -3212,7 +3321,7 @@
       <c r="U85" s="5"/>
       <c r="V85" s="11"/>
     </row>
-    <row r="86" spans="1:22">
+    <row r="86" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A86" s="5"/>
       <c r="B86" s="5"/>
       <c r="C86" s="5"/>
@@ -3236,7 +3345,7 @@
       <c r="U86" s="5"/>
       <c r="V86" s="11"/>
     </row>
-    <row r="87" spans="1:22">
+    <row r="87" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A87" s="5"/>
       <c r="B87" s="5"/>
       <c r="C87" s="5"/>
@@ -3260,7 +3369,7 @@
       <c r="U87" s="5"/>
       <c r="V87" s="11"/>
     </row>
-    <row r="88" spans="1:22">
+    <row r="88" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A88" s="5"/>
       <c r="B88" s="5"/>
       <c r="C88" s="5"/>
@@ -3284,7 +3393,7 @@
       <c r="U88" s="5"/>
       <c r="V88" s="11"/>
     </row>
-    <row r="89" spans="1:22">
+    <row r="89" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A89" s="5"/>
       <c r="B89" s="5"/>
       <c r="C89" s="5"/>
@@ -3308,7 +3417,7 @@
       <c r="U89" s="5"/>
       <c r="V89" s="11"/>
     </row>
-    <row r="90" spans="1:22">
+    <row r="90" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A90" s="5"/>
       <c r="B90" s="5"/>
       <c r="C90" s="5"/>
@@ -3332,7 +3441,7 @@
       <c r="U90" s="5"/>
       <c r="V90" s="11"/>
     </row>
-    <row r="91" spans="1:22" ht="14.25">
+    <row r="91" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A91" s="5"/>
       <c r="B91" s="5"/>
       <c r="C91" s="5"/>
@@ -3341,8 +3450,8 @@
       <c r="F91" s="5"/>
       <c r="G91" s="5"/>
       <c r="H91" s="5"/>
-      <c r="I91" s="14"/>
-      <c r="J91" s="15"/>
+      <c r="I91" s="5"/>
+      <c r="J91" s="5"/>
       <c r="K91" s="5"/>
       <c r="L91" s="9"/>
       <c r="M91" s="5"/>
@@ -3356,7 +3465,7 @@
       <c r="U91" s="5"/>
       <c r="V91" s="11"/>
     </row>
-    <row r="92" spans="1:22">
+    <row r="92" spans="1:22" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A92" s="5"/>
       <c r="B92" s="5"/>
       <c r="C92" s="5"/>
@@ -3365,8 +3474,8 @@
       <c r="F92" s="5"/>
       <c r="G92" s="5"/>
       <c r="H92" s="5"/>
-      <c r="I92" s="5"/>
-      <c r="J92" s="5"/>
+      <c r="I92" s="14"/>
+      <c r="J92" s="15"/>
       <c r="K92" s="5"/>
       <c r="L92" s="9"/>
       <c r="M92" s="5"/>
@@ -3380,7 +3489,7 @@
       <c r="U92" s="5"/>
       <c r="V92" s="11"/>
     </row>
-    <row r="93" spans="1:22">
+    <row r="93" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A93" s="5"/>
       <c r="B93" s="5"/>
       <c r="C93" s="5"/>
@@ -3404,7 +3513,7 @@
       <c r="U93" s="5"/>
       <c r="V93" s="11"/>
     </row>
-    <row r="94" spans="1:22">
+    <row r="94" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A94" s="5"/>
       <c r="B94" s="5"/>
       <c r="C94" s="5"/>
@@ -3428,7 +3537,7 @@
       <c r="U94" s="5"/>
       <c r="V94" s="11"/>
     </row>
-    <row r="95" spans="1:22">
+    <row r="95" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A95" s="5"/>
       <c r="B95" s="5"/>
       <c r="C95" s="5"/>
@@ -3452,7 +3561,7 @@
       <c r="U95" s="5"/>
       <c r="V95" s="11"/>
     </row>
-    <row r="96" spans="1:22">
+    <row r="96" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A96" s="5"/>
       <c r="B96" s="5"/>
       <c r="C96" s="5"/>
@@ -3476,7 +3585,7 @@
       <c r="U96" s="5"/>
       <c r="V96" s="11"/>
     </row>
-    <row r="97" spans="1:22">
+    <row r="97" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A97" s="5"/>
       <c r="B97" s="5"/>
       <c r="C97" s="5"/>
@@ -3500,7 +3609,7 @@
       <c r="U97" s="5"/>
       <c r="V97" s="11"/>
     </row>
-    <row r="98" spans="1:22" ht="14.25">
+    <row r="98" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A98" s="5"/>
       <c r="B98" s="5"/>
       <c r="C98" s="5"/>
@@ -3509,8 +3618,8 @@
       <c r="F98" s="5"/>
       <c r="G98" s="5"/>
       <c r="H98" s="5"/>
-      <c r="I98" s="14"/>
-      <c r="J98" s="15"/>
+      <c r="I98" s="5"/>
+      <c r="J98" s="5"/>
       <c r="K98" s="5"/>
       <c r="L98" s="9"/>
       <c r="M98" s="5"/>
@@ -3524,7 +3633,7 @@
       <c r="U98" s="5"/>
       <c r="V98" s="11"/>
     </row>
-    <row r="99" spans="1:22">
+    <row r="99" spans="1:22" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A99" s="5"/>
       <c r="B99" s="5"/>
       <c r="C99" s="5"/>
@@ -3533,8 +3642,8 @@
       <c r="F99" s="5"/>
       <c r="G99" s="5"/>
       <c r="H99" s="5"/>
-      <c r="I99" s="5"/>
-      <c r="J99" s="5"/>
+      <c r="I99" s="14"/>
+      <c r="J99" s="15"/>
       <c r="K99" s="5"/>
       <c r="L99" s="9"/>
       <c r="M99" s="5"/>
@@ -3548,7 +3657,7 @@
       <c r="U99" s="5"/>
       <c r="V99" s="11"/>
     </row>
-    <row r="100" spans="1:22">
+    <row r="100" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A100" s="5"/>
       <c r="B100" s="5"/>
       <c r="C100" s="5"/>
@@ -3572,7 +3681,7 @@
       <c r="U100" s="5"/>
       <c r="V100" s="11"/>
     </row>
-    <row r="101" spans="1:22">
+    <row r="101" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A101" s="5"/>
       <c r="B101" s="5"/>
       <c r="C101" s="5"/>
@@ -3596,7 +3705,7 @@
       <c r="U101" s="5"/>
       <c r="V101" s="11"/>
     </row>
-    <row r="102" spans="1:22">
+    <row r="102" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A102" s="5"/>
       <c r="B102" s="5"/>
       <c r="C102" s="5"/>
@@ -3620,7 +3729,7 @@
       <c r="U102" s="5"/>
       <c r="V102" s="11"/>
     </row>
-    <row r="103" spans="1:22">
+    <row r="103" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A103" s="5"/>
       <c r="B103" s="5"/>
       <c r="C103" s="5"/>
@@ -3644,7 +3753,7 @@
       <c r="U103" s="5"/>
       <c r="V103" s="11"/>
     </row>
-    <row r="104" spans="1:22">
+    <row r="104" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A104" s="5"/>
       <c r="B104" s="5"/>
       <c r="C104" s="5"/>
@@ -3668,7 +3777,7 @@
       <c r="U104" s="5"/>
       <c r="V104" s="11"/>
     </row>
-    <row r="105" spans="1:22" ht="14.25">
+    <row r="105" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A105" s="5"/>
       <c r="B105" s="5"/>
       <c r="C105" s="5"/>
@@ -3677,8 +3786,8 @@
       <c r="F105" s="5"/>
       <c r="G105" s="5"/>
       <c r="H105" s="5"/>
-      <c r="I105" s="14"/>
-      <c r="J105" s="15"/>
+      <c r="I105" s="5"/>
+      <c r="J105" s="5"/>
       <c r="K105" s="5"/>
       <c r="L105" s="9"/>
       <c r="M105" s="5"/>
@@ -3692,7 +3801,7 @@
       <c r="U105" s="5"/>
       <c r="V105" s="11"/>
     </row>
-    <row r="106" spans="1:22">
+    <row r="106" spans="1:22" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A106" s="5"/>
       <c r="B106" s="5"/>
       <c r="C106" s="5"/>
@@ -3701,8 +3810,8 @@
       <c r="F106" s="5"/>
       <c r="G106" s="5"/>
       <c r="H106" s="5"/>
-      <c r="I106" s="5"/>
-      <c r="J106" s="5"/>
+      <c r="I106" s="14"/>
+      <c r="J106" s="15"/>
       <c r="K106" s="5"/>
       <c r="L106" s="9"/>
       <c r="M106" s="5"/>
@@ -3716,7 +3825,7 @@
       <c r="U106" s="5"/>
       <c r="V106" s="11"/>
     </row>
-    <row r="107" spans="1:22">
+    <row r="107" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A107" s="5"/>
       <c r="B107" s="5"/>
       <c r="C107" s="5"/>
@@ -3740,7 +3849,7 @@
       <c r="U107" s="5"/>
       <c r="V107" s="11"/>
     </row>
-    <row r="108" spans="1:22">
+    <row r="108" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A108" s="5"/>
       <c r="B108" s="5"/>
       <c r="C108" s="5"/>
@@ -3764,7 +3873,7 @@
       <c r="U108" s="5"/>
       <c r="V108" s="11"/>
     </row>
-    <row r="109" spans="1:22">
+    <row r="109" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A109" s="5"/>
       <c r="B109" s="5"/>
       <c r="C109" s="5"/>
@@ -3788,7 +3897,7 @@
       <c r="U109" s="5"/>
       <c r="V109" s="11"/>
     </row>
-    <row r="110" spans="1:22">
+    <row r="110" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A110" s="5"/>
       <c r="B110" s="5"/>
       <c r="C110" s="5"/>
@@ -3812,7 +3921,7 @@
       <c r="U110" s="5"/>
       <c r="V110" s="11"/>
     </row>
-    <row r="111" spans="1:22">
+    <row r="111" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A111" s="5"/>
       <c r="B111" s="5"/>
       <c r="C111" s="5"/>
@@ -3836,7 +3945,7 @@
       <c r="U111" s="5"/>
       <c r="V111" s="11"/>
     </row>
-    <row r="112" spans="1:22">
+    <row r="112" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A112" s="5"/>
       <c r="B112" s="5"/>
       <c r="C112" s="5"/>
@@ -3860,7 +3969,7 @@
       <c r="U112" s="5"/>
       <c r="V112" s="11"/>
     </row>
-    <row r="113" spans="1:22">
+    <row r="113" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A113" s="5"/>
       <c r="B113" s="5"/>
       <c r="C113" s="5"/>
@@ -3884,7 +3993,7 @@
       <c r="U113" s="5"/>
       <c r="V113" s="11"/>
     </row>
-    <row r="114" spans="1:22">
+    <row r="114" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A114" s="5"/>
       <c r="B114" s="5"/>
       <c r="C114" s="5"/>
@@ -3908,7 +4017,7 @@
       <c r="U114" s="5"/>
       <c r="V114" s="11"/>
     </row>
-    <row r="115" spans="1:22">
+    <row r="115" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A115" s="5"/>
       <c r="B115" s="5"/>
       <c r="C115" s="5"/>
@@ -3932,7 +4041,7 @@
       <c r="U115" s="5"/>
       <c r="V115" s="11"/>
     </row>
-    <row r="116" spans="1:22">
+    <row r="116" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A116" s="5"/>
       <c r="B116" s="5"/>
       <c r="C116" s="5"/>
@@ -3956,7 +4065,7 @@
       <c r="U116" s="5"/>
       <c r="V116" s="11"/>
     </row>
-    <row r="117" spans="1:22">
+    <row r="117" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A117" s="5"/>
       <c r="B117" s="5"/>
       <c r="C117" s="5"/>
@@ -3980,7 +4089,7 @@
       <c r="U117" s="5"/>
       <c r="V117" s="11"/>
     </row>
-    <row r="118" spans="1:22">
+    <row r="118" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A118" s="5"/>
       <c r="B118" s="5"/>
       <c r="C118" s="5"/>
@@ -4004,7 +4113,7 @@
       <c r="U118" s="5"/>
       <c r="V118" s="11"/>
     </row>
-    <row r="119" spans="1:22">
+    <row r="119" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A119" s="5"/>
       <c r="B119" s="5"/>
       <c r="C119" s="5"/>
@@ -4028,7 +4137,7 @@
       <c r="U119" s="5"/>
       <c r="V119" s="11"/>
     </row>
-    <row r="120" spans="1:22">
+    <row r="120" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A120" s="5"/>
       <c r="B120" s="5"/>
       <c r="C120" s="5"/>
@@ -4052,7 +4161,7 @@
       <c r="U120" s="5"/>
       <c r="V120" s="11"/>
     </row>
-    <row r="121" spans="1:22">
+    <row r="121" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A121" s="5"/>
       <c r="B121" s="5"/>
       <c r="C121" s="5"/>
@@ -4076,7 +4185,7 @@
       <c r="U121" s="5"/>
       <c r="V121" s="11"/>
     </row>
-    <row r="122" spans="1:22">
+    <row r="122" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A122" s="5"/>
       <c r="B122" s="5"/>
       <c r="C122" s="5"/>
@@ -4100,7 +4209,7 @@
       <c r="U122" s="5"/>
       <c r="V122" s="11"/>
     </row>
-    <row r="123" spans="1:22">
+    <row r="123" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A123" s="5"/>
       <c r="B123" s="5"/>
       <c r="C123" s="5"/>
@@ -4124,7 +4233,7 @@
       <c r="U123" s="5"/>
       <c r="V123" s="11"/>
     </row>
-    <row r="124" spans="1:22">
+    <row r="124" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A124" s="5"/>
       <c r="B124" s="5"/>
       <c r="C124" s="5"/>
@@ -4148,7 +4257,7 @@
       <c r="U124" s="5"/>
       <c r="V124" s="11"/>
     </row>
-    <row r="125" spans="1:22">
+    <row r="125" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A125" s="5"/>
       <c r="B125" s="5"/>
       <c r="C125" s="5"/>
@@ -4172,7 +4281,7 @@
       <c r="U125" s="5"/>
       <c r="V125" s="11"/>
     </row>
-    <row r="126" spans="1:22">
+    <row r="126" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A126" s="5"/>
       <c r="B126" s="5"/>
       <c r="C126" s="5"/>
@@ -4196,7 +4305,7 @@
       <c r="U126" s="5"/>
       <c r="V126" s="11"/>
     </row>
-    <row r="127" spans="1:22">
+    <row r="127" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A127" s="5"/>
       <c r="B127" s="5"/>
       <c r="C127" s="5"/>
@@ -4220,7 +4329,7 @@
       <c r="U127" s="5"/>
       <c r="V127" s="11"/>
     </row>
-    <row r="128" spans="1:22">
+    <row r="128" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A128" s="5"/>
       <c r="B128" s="5"/>
       <c r="C128" s="5"/>
@@ -4244,7 +4353,7 @@
       <c r="U128" s="5"/>
       <c r="V128" s="11"/>
     </row>
-    <row r="129" spans="1:22">
+    <row r="129" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A129" s="5"/>
       <c r="B129" s="5"/>
       <c r="C129" s="5"/>
@@ -4268,7 +4377,7 @@
       <c r="U129" s="5"/>
       <c r="V129" s="11"/>
     </row>
-    <row r="130" spans="1:22">
+    <row r="130" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A130" s="5"/>
       <c r="B130" s="5"/>
       <c r="C130" s="5"/>
@@ -4292,7 +4401,7 @@
       <c r="U130" s="5"/>
       <c r="V130" s="11"/>
     </row>
-    <row r="131" spans="1:22">
+    <row r="131" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A131" s="5"/>
       <c r="B131" s="5"/>
       <c r="C131" s="5"/>
@@ -4316,7 +4425,7 @@
       <c r="U131" s="5"/>
       <c r="V131" s="11"/>
     </row>
-    <row r="132" spans="1:22">
+    <row r="132" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A132" s="5"/>
       <c r="B132" s="5"/>
       <c r="C132" s="5"/>
@@ -4335,12 +4444,12 @@
       <c r="P132" s="5"/>
       <c r="Q132" s="10"/>
       <c r="R132" s="5"/>
-      <c r="S132" s="11"/>
+      <c r="S132" s="5"/>
       <c r="T132" s="5"/>
       <c r="U132" s="5"/>
       <c r="V132" s="11"/>
     </row>
-    <row r="133" spans="1:22">
+    <row r="133" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A133" s="5"/>
       <c r="B133" s="5"/>
       <c r="C133" s="5"/>
@@ -4364,7 +4473,7 @@
       <c r="U133" s="5"/>
       <c r="V133" s="11"/>
     </row>
-    <row r="134" spans="1:22">
+    <row r="134" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A134" s="5"/>
       <c r="B134" s="5"/>
       <c r="C134" s="5"/>
@@ -4388,7 +4497,7 @@
       <c r="U134" s="5"/>
       <c r="V134" s="11"/>
     </row>
-    <row r="135" spans="1:22">
+    <row r="135" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A135" s="5"/>
       <c r="B135" s="5"/>
       <c r="C135" s="5"/>
@@ -4412,7 +4521,7 @@
       <c r="U135" s="5"/>
       <c r="V135" s="11"/>
     </row>
-    <row r="136" spans="1:22">
+    <row r="136" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A136" s="5"/>
       <c r="B136" s="5"/>
       <c r="C136" s="5"/>
@@ -4436,7 +4545,7 @@
       <c r="U136" s="5"/>
       <c r="V136" s="11"/>
     </row>
-    <row r="137" spans="1:22">
+    <row r="137" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A137" s="5"/>
       <c r="B137" s="5"/>
       <c r="C137" s="5"/>
@@ -4460,7 +4569,7 @@
       <c r="U137" s="5"/>
       <c r="V137" s="11"/>
     </row>
-    <row r="138" spans="1:22">
+    <row r="138" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A138" s="5"/>
       <c r="B138" s="5"/>
       <c r="C138" s="5"/>
@@ -4484,7 +4593,7 @@
       <c r="U138" s="5"/>
       <c r="V138" s="11"/>
     </row>
-    <row r="139" spans="1:22">
+    <row r="139" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A139" s="5"/>
       <c r="B139" s="5"/>
       <c r="C139" s="5"/>
@@ -4508,7 +4617,7 @@
       <c r="U139" s="5"/>
       <c r="V139" s="11"/>
     </row>
-    <row r="140" spans="1:22">
+    <row r="140" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A140" s="5"/>
       <c r="B140" s="5"/>
       <c r="C140" s="5"/>
@@ -4532,7 +4641,7 @@
       <c r="U140" s="5"/>
       <c r="V140" s="11"/>
     </row>
-    <row r="141" spans="1:22" s="16" customFormat="1">
+    <row r="141" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A141" s="5"/>
       <c r="B141" s="5"/>
       <c r="C141" s="5"/>
@@ -4551,12 +4660,12 @@
       <c r="P141" s="5"/>
       <c r="Q141" s="10"/>
       <c r="R141" s="5"/>
-      <c r="S141" s="5"/>
+      <c r="S141" s="11"/>
       <c r="T141" s="5"/>
       <c r="U141" s="5"/>
       <c r="V141" s="11"/>
     </row>
-    <row r="142" spans="1:22" s="17" customFormat="1">
+    <row r="142" spans="1:22" s="16" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A142" s="5"/>
       <c r="B142" s="5"/>
       <c r="C142" s="5"/>
@@ -4580,7 +4689,7 @@
       <c r="U142" s="5"/>
       <c r="V142" s="11"/>
     </row>
-    <row r="143" spans="1:22" s="17" customFormat="1">
+    <row r="143" spans="1:22" s="17" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A143" s="5"/>
       <c r="B143" s="5"/>
       <c r="C143" s="5"/>
@@ -4604,7 +4713,7 @@
       <c r="U143" s="5"/>
       <c r="V143" s="11"/>
     </row>
-    <row r="144" spans="1:22" s="17" customFormat="1">
+    <row r="144" spans="1:22" s="17" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A144" s="5"/>
       <c r="B144" s="5"/>
       <c r="C144" s="5"/>
@@ -4623,12 +4732,12 @@
       <c r="P144" s="5"/>
       <c r="Q144" s="10"/>
       <c r="R144" s="5"/>
-      <c r="S144" s="18"/>
+      <c r="S144" s="5"/>
       <c r="T144" s="5"/>
       <c r="U144" s="5"/>
       <c r="V144" s="11"/>
     </row>
-    <row r="145" spans="1:22" s="17" customFormat="1">
+    <row r="145" spans="1:22" s="17" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A145" s="5"/>
       <c r="B145" s="5"/>
       <c r="C145" s="5"/>
@@ -4647,12 +4756,12 @@
       <c r="P145" s="5"/>
       <c r="Q145" s="10"/>
       <c r="R145" s="5"/>
-      <c r="S145" s="5"/>
+      <c r="S145" s="18"/>
       <c r="T145" s="5"/>
       <c r="U145" s="5"/>
       <c r="V145" s="11"/>
     </row>
-    <row r="146" spans="1:22" s="17" customFormat="1">
+    <row r="146" spans="1:22" s="17" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A146" s="5"/>
       <c r="B146" s="5"/>
       <c r="C146" s="5"/>
@@ -4671,12 +4780,12 @@
       <c r="P146" s="5"/>
       <c r="Q146" s="10"/>
       <c r="R146" s="5"/>
-      <c r="S146" s="18"/>
+      <c r="S146" s="5"/>
       <c r="T146" s="5"/>
       <c r="U146" s="5"/>
       <c r="V146" s="11"/>
     </row>
-    <row r="147" spans="1:22" s="17" customFormat="1">
+    <row r="147" spans="1:22" s="17" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A147" s="5"/>
       <c r="B147" s="5"/>
       <c r="C147" s="5"/>
@@ -4695,12 +4804,12 @@
       <c r="P147" s="5"/>
       <c r="Q147" s="10"/>
       <c r="R147" s="5"/>
-      <c r="S147" s="5"/>
+      <c r="S147" s="18"/>
       <c r="T147" s="5"/>
       <c r="U147" s="5"/>
       <c r="V147" s="11"/>
     </row>
-    <row r="148" spans="1:22" s="17" customFormat="1">
+    <row r="148" spans="1:22" s="17" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A148" s="5"/>
       <c r="B148" s="5"/>
       <c r="C148" s="5"/>
@@ -4724,7 +4833,7 @@
       <c r="U148" s="5"/>
       <c r="V148" s="11"/>
     </row>
-    <row r="149" spans="1:22" s="17" customFormat="1">
+    <row r="149" spans="1:22" s="17" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A149" s="5"/>
       <c r="B149" s="5"/>
       <c r="C149" s="5"/>
@@ -4748,7 +4857,7 @@
       <c r="U149" s="5"/>
       <c r="V149" s="11"/>
     </row>
-    <row r="150" spans="1:22" s="17" customFormat="1">
+    <row r="150" spans="1:22" s="17" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A150" s="5"/>
       <c r="B150" s="5"/>
       <c r="C150" s="5"/>
@@ -4767,12 +4876,12 @@
       <c r="P150" s="5"/>
       <c r="Q150" s="10"/>
       <c r="R150" s="5"/>
-      <c r="S150" s="18"/>
+      <c r="S150" s="5"/>
       <c r="T150" s="5"/>
       <c r="U150" s="5"/>
       <c r="V150" s="11"/>
     </row>
-    <row r="151" spans="1:22">
+    <row r="151" spans="1:22" s="17" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A151" s="5"/>
       <c r="B151" s="5"/>
       <c r="C151" s="5"/>
@@ -4791,12 +4900,12 @@
       <c r="P151" s="5"/>
       <c r="Q151" s="10"/>
       <c r="R151" s="5"/>
-      <c r="S151" s="5"/>
+      <c r="S151" s="18"/>
       <c r="T151" s="5"/>
       <c r="U151" s="5"/>
       <c r="V151" s="11"/>
     </row>
-    <row r="152" spans="1:22" s="17" customFormat="1">
+    <row r="152" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A152" s="5"/>
       <c r="B152" s="5"/>
       <c r="C152" s="5"/>
@@ -4820,7 +4929,7 @@
       <c r="U152" s="5"/>
       <c r="V152" s="11"/>
     </row>
-    <row r="153" spans="1:22">
+    <row r="153" spans="1:22" s="17" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A153" s="5"/>
       <c r="B153" s="5"/>
       <c r="C153" s="5"/>
@@ -4844,7 +4953,7 @@
       <c r="U153" s="5"/>
       <c r="V153" s="11"/>
     </row>
-    <row r="154" spans="1:22" s="17" customFormat="1">
+    <row r="154" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A154" s="5"/>
       <c r="B154" s="5"/>
       <c r="C154" s="5"/>
@@ -4868,6 +4977,30 @@
       <c r="U154" s="5"/>
       <c r="V154" s="11"/>
     </row>
+    <row r="155" spans="1:22" s="17" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A155" s="5"/>
+      <c r="B155" s="5"/>
+      <c r="C155" s="5"/>
+      <c r="D155" s="5"/>
+      <c r="E155" s="5"/>
+      <c r="F155" s="5"/>
+      <c r="G155" s="5"/>
+      <c r="H155" s="5"/>
+      <c r="I155" s="5"/>
+      <c r="J155" s="5"/>
+      <c r="K155" s="5"/>
+      <c r="L155" s="9"/>
+      <c r="M155" s="5"/>
+      <c r="N155" s="5"/>
+      <c r="O155" s="5"/>
+      <c r="P155" s="5"/>
+      <c r="Q155" s="10"/>
+      <c r="R155" s="5"/>
+      <c r="S155" s="5"/>
+      <c r="T155" s="5"/>
+      <c r="U155" s="5"/>
+      <c r="V155" s="11"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
   <dataConsolidate/>
@@ -4880,10 +5013,13 @@
   <hyperlinks>
     <hyperlink ref="D3" r:id="rId1" location="collapse2" display="https://automationexercise.com/api_list - collapse2" xr:uid="{4CB74369-E6C3-4251-A75E-F43B9505B933}"/>
     <hyperlink ref="D2" r:id="rId2" location="collapse1" display="https://automationexercise.com/api_list - collapse1" xr:uid="{E10F699E-A2FA-4AA4-AD4F-F02AFFC6D94A}"/>
+    <hyperlink ref="D5" r:id="rId3" location="collapse5" display="https://automationexercise.com/api_list - collapse5" xr:uid="{1660F3A1-24DE-4B70-9BD4-1DD4413EF49F}"/>
+    <hyperlink ref="D6" r:id="rId4" location="collapse6" display="https://automationexercise.com/api_list - collapse6" xr:uid="{92F62890-D944-46D8-AB4D-388FB9993B8A}"/>
+    <hyperlink ref="D4" r:id="rId5" location="collapse3" display="https://automationexercise.com/api_list - collapse3" xr:uid="{AF74A331-B6FD-40A3-B6AF-15EC5DD54FC7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
-  <drawing r:id="rId4"/>
-  <legacyDrawing r:id="rId5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
+  <drawing r:id="rId7"/>
+  <legacyDrawing r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>